<commit_message>
docs: add Release Bundle P1-P2 and Release Steps P1-P2 sheets to the register
Every built file of the Parts 1-2 production bundle with path, checksum,
deploy order and sandbox test reference; deploy steps with commands.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -11,6 +11,8 @@
     <sheet name="Test Classes" sheetId="7" r:id="rId7"/>
     <sheet name="Backups" sheetId="8" r:id="rId8"/>
     <sheet name="Part 3 Plan" sheetId="9" r:id="rId9"/>
+    <sheet name="Release Bundle P1-P2" sheetId="10" r:id="rId10"/>
+    <sheet name="Release Steps P1-P2" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
@@ -22,6 +24,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle P1-P2'!$A$4:$K$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps P1-P2'!$A$4:$E$10</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -295,6 +299,2463 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="9" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="9" customWidth="1"/>
+    <col min="4" max="4" width="9" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="7" width="70" customWidth="1"/>
+    <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="30" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
+    <col min="11" max="11" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Production Release Bundle - Parts 1 and 2 (built components)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Every file in release/prod, converted from the sandbox-tested source. Checksums in release/prod/SHA256SUMS. Rebuild: bash scripts/release/build-prod-release.sh</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>Deploy order</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Bundle folder</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Part</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Metadata Type</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr" s="1">
+        <is>
+          <t>File path</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr" s="1">
+        <is>
+          <t>SHA-256 (first 12)</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr" s="1">
+        <is>
+          <t>For</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr" s="1">
+        <is>
+          <t>Tested in sandbox</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr" s="1">
+        <is>
+          <t>Prod Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialService.cls</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5b84b4f96887</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialServiceCTI</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialServiceCTI.cls</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9cc82f98c9fd</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialServiceCTI</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialServiceCTI.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingConfig</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskingConfig.cls</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">35b3fcb96581</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingConfig</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskingConfig.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
+        <v>1</v>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskUtil</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskUtil.cls</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ea923f1f15bc</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
+        <v>1</v>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskUtil</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskUtil.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
+        <v>1</v>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialServiceCTITest</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialServiceCTITest.cls</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">df752a8bbf08</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
+        <v>1</v>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialServiceCTITest</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialServiceCTITest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
+        <v>1</v>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialServiceTest.cls</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">0e94577583e0</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
+        <v>1</v>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/MaskedDialServiceTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
+        <v>1</v>
+      </c>
+      <c r="B17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingConfigTest</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskingConfigTest.cls</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">df947c8de87b</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <v>1</v>
+      </c>
+      <c r="B18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingConfigTest</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskingConfigTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2">
+        <v>1</v>
+      </c>
+      <c r="B19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskUtilTest</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskUtilTest.cls</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">c86517eb7fc7</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2">
+        <v>1</v>
+      </c>
+      <c r="B20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskUtilTest</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneMaskUtilTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2">
+        <v>1</v>
+      </c>
+      <c r="B21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneTestDataFactory</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneTestDataFactory.cls</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">838c454f7ee5</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2">
+        <v>1</v>
+      </c>
+      <c r="B22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneTestDataFactory</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/classes/PhoneTestDataFactory.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2">
+        <v>1</v>
+      </c>
+      <c r="B23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Metadata Record</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked_Phone_Field.Lead_Phone</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/customMetadata/Masked_Phone_Field.Lead_Phone.md</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">eb3602e65c12</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2">
+        <v>1</v>
+      </c>
+      <c r="B24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Metadata Record</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked_Phone_Field.Lead_Secondary_Phone</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/customMetadata/Masked_Phone_Field.Lead_Secondary_Phone.md</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">19daa00b73c7</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2">
+        <v>1</v>
+      </c>
+      <c r="B25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Metadata Record</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Masking_Setting.Default</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/customMetadata/Phone_Masking_Setting.Default.md</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">4f3042be143f</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2">
+        <v>1</v>
+      </c>
+      <c r="B26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked_Phone_Field__mdt</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/objects/Masked_Phone_Field__mdt.object</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">669f98730825</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2">
+        <v>1</v>
+      </c>
+      <c r="B27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/objects/Phone_Access_Audit__c.object</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1098c11ee9d4</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2">
+        <v>1</v>
+      </c>
+      <c r="B28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Masking_Setting__mdt</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/objects/Phone_Masking_Setting__mdt.object</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">e1943db5ee18</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2">
+        <v>1</v>
+      </c>
+      <c r="B29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Tab</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/tabs/Phone_Access_Audit__c.tab</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">fc02dd0727e9</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2">
+        <v>1</v>
+      </c>
+      <c r="B30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/package.xml</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9514afa794c8</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2">
+        <v>1</v>
+      </c>
+      <c r="B31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 1</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.1.0</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit_Viewer</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part1-foundations/permissionsets/Phone_Access_Audit_Viewer.permissionset</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">dea06e92ea46</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LO8zCAG</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2">
+        <v>2</v>
+      </c>
+      <c r="B32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedPhonePanelController</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/classes/MaskedPhonePanelController.cls</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1db09cd4a780</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2">
+        <v>2</v>
+      </c>
+      <c r="B33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedPhonePanelController</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/classes/MaskedPhonePanelController.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2">
+        <v>2</v>
+      </c>
+      <c r="B34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedPhonePanelControllerTest</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/classes/MaskedPhonePanelControllerTest.cls</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">8e22c948bff7</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2">
+        <v>2</v>
+      </c>
+      <c r="B35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedPhonePanelControllerTest</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/classes/MaskedPhonePanelControllerTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2">
+        <v>2</v>
+      </c>
+      <c r="B36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/lwc/maskedPhonePanel/maskedPhonePanel.css</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f1df701a3a2c</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2">
+        <v>2</v>
+      </c>
+      <c r="B37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/lwc/maskedPhonePanel/maskedPhonePanel.html</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">2cc369f04123</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2">
+        <v>2</v>
+      </c>
+      <c r="B38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/lwc/maskedPhonePanel/maskedPhonePanel.js</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">d44addcdfaf9</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="2">
+        <v>2</v>
+      </c>
+      <c r="B39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/lwc/maskedPhonePanel/maskedPhonePanel.js-meta.xml</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">0d33c6f7d7e6</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="2">
+        <v>2</v>
+      </c>
+      <c r="B40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-panel/package.xml</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">718673207c21</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2">
+        <v>3</v>
+      </c>
+      <c r="B41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">8ff8df2bf019</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2">
+        <v>3</v>
+      </c>
+      <c r="B42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2">
+        <v>3</v>
+      </c>
+      <c r="B43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Profile</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9c73dfa0992e</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:K43"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="110" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Production Deploy Steps - Parts 1 and 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Validate first, then quick deploy. Replace &lt;prod&gt; with the production org alias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Bundle</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>What</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Command / Where</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Prod Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part1-foundations</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part1-foundations --test-level RunSpecifiedTests --tests PhoneMaskingConfigTest --tests PhoneMaskUtilTest --tests MaskedDialServiceTest --tests MaskedDialServiceCTITest</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2">
+        <v>2</v>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-panel</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part2-panel --test-level RunSpecifiedTests --tests MaskedPhonePanelControllerTest</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2">
+        <v>3</v>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pilot only: clone Presales outbound -&gt; POC Masked Rep in Setup, then deploy</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">sf project deploy start --metadata-dir release/prod/part2-pilot --test-level NoTestRun</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2">
+        <v>4</v>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2">
+        <v>5</v>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2">
+        <v>6</v>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(check)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:E10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
feat: v1.3.0 masked click-to-dial for MCube and SlashRTC (built locally, not deployed)
Existing (approved, originals in backup/v1.3.0-pre-change):
- McubeSoftphoneAddOnController: + clickToCallMasked (additive only)
- mcubeSoftphoneCTIAddOn: masked-click branch; original call unchanged
- slashPhoneHelper.js: masked-click step before the unchanged flow
Our components: MaskedDialService (deferred audit, fieldKeyForMaskedNumber),
MaskedDialServiceCTI (resolveMaskedClick), tests, POC profile, POC page.
New: McubeMaskedClickToCallTest. Sandbox-only SlashRTC adapter URL.
Manifests, changelog, roadmap and Excel register updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -17,9 +17,9 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="D7" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="E7" s="2">
@@ -6472,9 +6472,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I56" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I56" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr" s="2">
@@ -6509,12 +6509,12 @@
       </c>
       <c r="D57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">MaskedDialService</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="2">
@@ -6524,17 +6524,17 @@
       </c>
       <c r="G57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add class access: MaskedDialServiceCTI (SlashRTC runApex)</t>
+          <t xml:space="preserve">Adds deferred audit (callout-safe) + field lookup from masked value</t>
         </is>
       </c>
       <c r="H57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I57" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr" s="2">
@@ -6544,12 +6544,12 @@
       </c>
       <c r="K57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Part 1 component updated</t>
         </is>
       </c>
     </row>
@@ -6569,12 +6569,12 @@
       </c>
       <c r="D58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page (update of new)</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">MaskedDialServiceCTI</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="2">
@@ -6584,17 +6584,17 @@
       </c>
       <c r="G58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Turn panel property Enable click-to-dial = true</t>
+          <t xml:space="preserve">Adds resolveMaskedClick (SlashRTC masked click)</t>
         </is>
       </c>
       <c r="H58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I58" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">MaskedDialServiceCTITest</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr" s="2">
@@ -6604,12 +6604,12 @@
       </c>
       <c r="K58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Part 1 component updated</t>
         </is>
       </c>
     </row>
@@ -6629,12 +6629,12 @@
       </c>
       <c r="D59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Message Channel</t>
+          <t xml:space="preserve">Apex Class (test, update)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MaskedDialRequest__c</t>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="2">
@@ -6644,7 +6644,7 @@
       </c>
       <c r="G59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fallback Option A only: panel sends {recordId, fieldKey} to adapters</t>
+          <t xml:space="preserve">+5 tests</t>
         </is>
       </c>
       <c r="H59" t="inlineStr" s="2">
@@ -6652,9 +6652,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I59" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+      <c r="I59" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr" s="2">
@@ -6664,12 +6664,12 @@
       </c>
       <c r="K59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows masked click-to-dial fails</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -6679,32 +6679,32 @@
       </c>
       <c r="B60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class (test, update)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Entry__c</t>
+          <t xml:space="preserve">MaskedDialServiceCTITest</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Entry field for primary number; copied to Phone__c and cleared</t>
+          <t xml:space="preserve">+3 tests</t>
         </is>
       </c>
       <c r="H60" t="inlineStr" s="2">
@@ -6712,9 +6712,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I60" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I60" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr" s="2">
@@ -6739,32 +6739,32 @@
       </c>
       <c r="B61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Entry__c</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Entry field for secondary number</t>
+          <t xml:space="preserve">Add class access: MaskedDialServiceCTI (SlashRTC runApex)</t>
         </is>
       </c>
       <c r="H61" t="inlineStr" s="2">
@@ -6772,9 +6772,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I61" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I61" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr" s="2">
@@ -6784,7 +6784,7 @@
       </c>
       <c r="K61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="L61" t="inlineStr" s="2">
@@ -6799,22 +6799,22 @@
       </c>
       <c r="B62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Page (update of new)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
         </is>
       </c>
       <c r="F62" t="inlineStr" s="2">
@@ -6824,17 +6824,17 @@
       </c>
       <c r="G62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Copies entry fields, locks primary after creation</t>
+          <t xml:space="preserve">Turn panel property Enable click-to-dial = true</t>
         </is>
       </c>
       <c r="H62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
-        </is>
-      </c>
-      <c r="I62" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr" s="2">
@@ -6844,7 +6844,7 @@
       </c>
       <c r="K62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="L62" t="inlineStr" s="2">
@@ -6859,22 +6859,22 @@
       </c>
       <c r="B63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Message Channel</t>
         </is>
       </c>
       <c r="E63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+          <t xml:space="preserve">MaskedDialRequest__c</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="2">
@@ -6884,7 +6884,7 @@
       </c>
       <c r="G63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Tests incl. 200-record bulk</t>
+          <t xml:space="preserve">Fallback Option A only: panel sends {recordId, fieldKey} to adapters</t>
         </is>
       </c>
       <c r="H63" t="inlineStr" s="2">
@@ -6892,9 +6892,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I63" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I63" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="J63" t="inlineStr" s="2">
@@ -6904,12 +6904,12 @@
       </c>
       <c r="K63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="L63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows masked click-to-dial fails</t>
         </is>
       </c>
     </row>
@@ -6919,12 +6919,12 @@
       </c>
       <c r="B64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D64" t="inlineStr" s="2">
@@ -6934,7 +6934,7 @@
       </c>
       <c r="E64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Masked__c</t>
+          <t xml:space="preserve">Phone_Entry__c</t>
         </is>
       </c>
       <c r="F64" t="inlineStr" s="2">
@@ -6944,7 +6944,7 @@
       </c>
       <c r="G64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked primary for layouts / list views / reports</t>
+          <t xml:space="preserve">Entry field for primary number; copied to Phone__c and cleared</t>
         </is>
       </c>
       <c r="H64" t="inlineStr" s="2">
@@ -6979,12 +6979,12 @@
       </c>
       <c r="B65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D65" t="inlineStr" s="2">
@@ -6994,7 +6994,7 @@
       </c>
       <c r="E65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
+          <t xml:space="preserve">Secondary_Phone_Entry__c</t>
         </is>
       </c>
       <c r="F65" t="inlineStr" s="2">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="G65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked secondary</t>
+          <t xml:space="preserve">Entry field for secondary number</t>
         </is>
       </c>
       <c r="H65" t="inlineStr" s="2">
@@ -7039,37 +7039,37 @@
       </c>
       <c r="B66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_To_Masked__c</t>
+          <t xml:space="preserve">LeadPhoneEntryHandler</t>
         </is>
       </c>
       <c r="F66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_Detail__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked call number</t>
+          <t xml:space="preserve">Copies entry fields, locks primary after creation</t>
         </is>
       </c>
       <c r="H66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
       <c r="I66" t="inlineStr" s="6">
@@ -7099,22 +7099,22 @@
       </c>
       <c r="B67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
       <c r="F67" t="inlineStr" s="2">
@@ -7124,12 +7124,12 @@
       </c>
       <c r="G67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal for TL / Head / Admin: reason, 30 s, audit</t>
+          <t xml:space="preserve">Tests incl. 200-record bulk</t>
         </is>
       </c>
       <c r="H67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I67" t="inlineStr" s="6">
@@ -7159,32 +7159,32 @@
       </c>
       <c r="B68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">Phone_Masked__c</t>
         </is>
       </c>
       <c r="F68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Formula: masked primary for layouts / list views / reports</t>
         </is>
       </c>
       <c r="H68" t="inlineStr" s="2">
@@ -7219,12 +7219,12 @@
       </c>
       <c r="B69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D69" t="inlineStr" s="2">
@@ -7234,17 +7234,17 @@
       </c>
       <c r="E69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
+          <t xml:space="preserve">Formula: masked secondary</t>
         </is>
       </c>
       <c r="H69" t="inlineStr" s="2">
@@ -7279,32 +7279,32 @@
       </c>
       <c r="B70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">Call_To_Masked__c</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call_Detail__c</t>
         </is>
       </c>
       <c r="G70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Who may reveal</t>
+          <t xml:space="preserve">Formula: masked call number</t>
         </is>
       </c>
       <c r="H70" t="inlineStr" s="2">
@@ -7349,12 +7349,12 @@
       </c>
       <c r="D71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="2">
@@ -7364,12 +7364,12 @@
       </c>
       <c r="G71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grants Reveal_Phone_Number to TL / Head / Admin</t>
+          <t xml:space="preserve">Reveal for TL / Head / Admin: reason, 30 s, audit</t>
         </is>
       </c>
       <c r="H71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="I71" t="inlineStr" s="6">
@@ -7409,12 +7409,12 @@
       </c>
       <c r="D72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
@@ -7424,12 +7424,12 @@
       </c>
       <c r="G72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nightly delete of audit rows older than 1 year (batch + schedulable)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I72" t="inlineStr" s="6">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="L72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7469,22 +7469,22 @@
       </c>
       <c r="D73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
         </is>
       </c>
       <c r="H73" t="inlineStr" s="2">
@@ -7529,12 +7529,12 @@
       </c>
       <c r="D74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
@@ -7544,7 +7544,7 @@
       </c>
       <c r="G74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add Reveal button + reason picker</t>
+          <t xml:space="preserve">Who may reveal</t>
         </is>
       </c>
       <c r="H74" t="inlineStr" s="2">
@@ -7579,22 +7579,22 @@
       </c>
       <c r="B75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="2">
@@ -7604,12 +7604,12 @@
       </c>
       <c r="G75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masks numbers typed in free text on save</t>
+          <t xml:space="preserve">Grants Reveal_Phone_Number to TL / Head / Admin</t>
         </is>
       </c>
       <c r="H75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I75" t="inlineStr" s="6">
@@ -7629,7 +7629,7 @@
       </c>
       <c r="L75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7639,22 +7639,22 @@
       </c>
       <c r="B76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
@@ -7664,12 +7664,12 @@
       </c>
       <c r="G76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Nightly delete of audit rows older than 1 year (batch + schedulable)</t>
         </is>
       </c>
       <c r="H76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="I76" t="inlineStr" s="6">
@@ -7689,7 +7689,7 @@
       </c>
       <c r="L76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -7699,37 +7699,37 @@
       </c>
       <c r="B77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masks numbers in Chatter posts</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I77" t="inlineStr" s="6">
@@ -7759,22 +7759,22 @@
       </c>
       <c r="B78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
@@ -7784,17 +7784,17 @@
       </c>
       <c r="G78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Search a number, masked result, audited</t>
+          <t xml:space="preserve">Add Reveal button + reason picker</t>
         </is>
       </c>
       <c r="H78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
-        </is>
-      </c>
-      <c r="I78" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J78" t="inlineStr" s="2">
@@ -7804,12 +7804,12 @@
       </c>
       <c r="K78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7819,12 +7819,12 @@
       </c>
       <c r="B79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D79" t="inlineStr" s="2">
@@ -7834,7 +7834,7 @@
       </c>
       <c r="E79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
@@ -7844,17 +7844,17 @@
       </c>
       <c r="G79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server side of findByNumber</t>
+          <t xml:space="preserve">Masks numbers typed in free text on save</t>
         </is>
       </c>
       <c r="H79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J79" t="inlineStr" s="2">
@@ -7864,12 +7864,12 @@
       </c>
       <c r="K79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -7879,12 +7879,12 @@
       </c>
       <c r="B80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D80" t="inlineStr" s="2">
@@ -7894,7 +7894,7 @@
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -7912,9 +7912,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I80" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+      <c r="I80" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J80" t="inlineStr" s="2">
@@ -7924,7 +7924,7 @@
       </c>
       <c r="K80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L80" t="inlineStr" s="2">
@@ -7939,37 +7939,37 @@
       </c>
       <c r="B81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Full phone-field access for integration users</t>
+          <t xml:space="preserve">Masks numbers in Chatter posts</t>
         </is>
       </c>
       <c r="H81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="I81" t="inlineStr" s="6">
@@ -7989,7 +7989,7 @@
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -7999,62 +7999,302 @@
       </c>
       <c r="B82" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 8</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.8.0</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">findByNumber</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Search a number, masked result, audited</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Jest</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="L82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2">
+        <v>79</v>
+      </c>
+      <c r="B83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 8</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.8.0</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberController</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Server side of findByNumber</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="L83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2">
+        <v>80</v>
+      </c>
+      <c r="B84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 8</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.8.0</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2">
+        <v>81</v>
+      </c>
+      <c r="B85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v2.0.0</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Full phone-field access for integration users</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign to integration users</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2">
+        <v>82</v>
+      </c>
+      <c r="B86" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Security fix</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr" s="2">
+      <c r="C86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">optional</t>
         </is>
       </c>
-      <c r="D82" t="inlineStr" s="2">
+      <c r="D86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr" s="2">
+      <c r="E86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
-      <c r="F82" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr" s="2">
+      <c r="F86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">MCube endpoint + key over HTTPS instead of hard-coded token / http</t>
         </is>
       </c>
-      <c r="H82" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr" s="6">
+      <c r="H86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Planned</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K82" t="inlineStr" s="2">
+      <c r="J86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr" s="2">
+      <c r="L86" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L82"/>
+  <autoFilter ref="A4:L86"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -8254,7 +8494,7 @@
       </c>
       <c r="H6" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I6" t="inlineStr" s="2">
@@ -8262,9 +8502,9 @@
           <t xml:space="preserve">backup/v1.3.0-pre-change</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J6" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="K6" t="inlineStr" s="2">
@@ -8314,7 +8554,7 @@
       </c>
       <c r="H7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I7" t="inlineStr" s="2">
@@ -8322,9 +8562,9 @@
           <t xml:space="preserve">backup/v1.3.0-pre-change</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J7" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="K7" t="inlineStr" s="2">
@@ -8374,7 +8614,7 @@
       </c>
       <c r="H8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I8" t="inlineStr" s="2">
@@ -8382,9 +8622,9 @@
           <t xml:space="preserve">backup/v1.3.0-pre-change</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J8" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="K8" t="inlineStr" s="2">
@@ -8434,7 +8674,7 @@
       </c>
       <c r="H9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I9" t="inlineStr" s="2">
@@ -14639,12 +14879,12 @@
       </c>
       <c r="D56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">MaskedDialService</t>
         </is>
       </c>
       <c r="F56" t="inlineStr" s="2">
@@ -14654,7 +14894,7 @@
       </c>
       <c r="G56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H56" t="inlineStr" s="2">
@@ -14664,7 +14904,7 @@
       </c>
       <c r="I56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
         </is>
       </c>
       <c r="J56" t="inlineStr" s="2">
@@ -14679,7 +14919,7 @@
       </c>
       <c r="L56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add new @RemoteAction clickToCallMasked(recordId, fieldKey): resolves via MaskedDialService, then reuses clickToCallRemote</t>
+          <t xml:space="preserve">Part 1 component updated</t>
         </is>
       </c>
     </row>
@@ -14699,12 +14939,12 @@
       </c>
       <c r="D57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeMaskedClickToCallTest</t>
+          <t xml:space="preserve">MaskedDialServiceCTI</t>
         </is>
       </c>
       <c r="F57" t="inlineStr" s="2">
@@ -14724,7 +14964,7 @@
       </c>
       <c r="I57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MaskedDialServiceCTITest</t>
         </is>
       </c>
       <c r="J57" t="inlineStr" s="2">
@@ -14739,7 +14979,7 @@
       </c>
       <c r="L57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New class so the existing test class stays untouched</t>
+          <t xml:space="preserve">Part 1 component updated</t>
         </is>
       </c>
     </row>
@@ -14759,12 +14999,12 @@
       </c>
       <c r="D58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mcubeSoftphoneCTIAddOn</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F58" t="inlineStr" s="2">
@@ -14799,7 +15039,7 @@
       </c>
       <c r="L58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">In onClickToDial: if the click comes from the masked panel, call the new server method with recordId + fieldKey</t>
+          <t xml:space="preserve">Add new @RemoteAction clickToCallMasked(recordId, fieldKey): resolves via MaskedDialService, then reuses clickToCallRemote</t>
         </is>
       </c>
     </row>
@@ -14819,12 +15059,12 @@
       </c>
       <c r="D59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test, update)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">slashPhone (slashPhoneHelper.js)</t>
+          <t xml:space="preserve">MaskedDialServiceCTITest</t>
         </is>
       </c>
       <c r="F59" t="inlineStr" s="2">
@@ -14834,7 +15074,7 @@
       </c>
       <c r="G59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H59" t="inlineStr" s="2">
@@ -14859,7 +15099,7 @@
       </c>
       <c r="L59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">In onClickToDial listener: if masked click, runApex MaskedDialServiceCTI.resolveForDial, then continue existing flow</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -14879,12 +15119,12 @@
       </c>
       <c r="D60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page (update of new)</t>
+          <t xml:space="preserve">Apex Class (test, update)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
         </is>
       </c>
       <c r="F60" t="inlineStr" s="2">
@@ -14909,7 +15149,7 @@
       </c>
       <c r="J60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K60" t="inlineStr" s="6">
@@ -14939,12 +15179,12 @@
       </c>
       <c r="D61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">McubeMaskedClickToCallTest</t>
         </is>
       </c>
       <c r="F61" t="inlineStr" s="2">
@@ -14969,7 +15209,7 @@
       </c>
       <c r="J61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K61" t="inlineStr" s="6">
@@ -14979,7 +15219,7 @@
       </c>
       <c r="L61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">New class so the existing test class stays untouched</t>
         </is>
       </c>
     </row>
@@ -14989,32 +15229,32 @@
       </c>
       <c r="B62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Entry__c</t>
+          <t xml:space="preserve">mcubeSoftphoneCTIAddOn</t>
         </is>
       </c>
       <c r="F62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H62" t="inlineStr" s="2">
@@ -15039,7 +15279,7 @@
       </c>
       <c r="L62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">In onClickToDial: if the click comes from the masked panel, call the new server method with recordId + fieldKey</t>
         </is>
       </c>
     </row>
@@ -15049,32 +15289,32 @@
       </c>
       <c r="B63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Entry__c</t>
+          <t xml:space="preserve">slashPhone (slashPhoneHelper.js)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H63" t="inlineStr" s="2">
@@ -15099,7 +15339,7 @@
       </c>
       <c r="L63" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">In onClickToDial listener: if masked click, runApex MaskedDialServiceCTI.resolveForDial, then continue existing flow</t>
         </is>
       </c>
     </row>
@@ -15109,22 +15349,22 @@
       </c>
       <c r="B64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Page (update of new)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
         </is>
       </c>
       <c r="F64" t="inlineStr" s="2">
@@ -15144,12 +15384,12 @@
       </c>
       <c r="I64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K64" t="inlineStr" s="6">
@@ -15169,22 +15409,22 @@
       </c>
       <c r="B65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="C65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="D65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadTriggerHandler</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F65" t="inlineStr" s="2">
@@ -15194,7 +15434,7 @@
       </c>
       <c r="G65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H65" t="inlineStr" s="2">
@@ -15209,7 +15449,7 @@
       </c>
       <c r="J65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K65" t="inlineStr" s="6">
@@ -15219,7 +15459,7 @@
       </c>
       <c r="L65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hook for entry-field copy (if routed through handler)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -15239,17 +15479,17 @@
       </c>
       <c r="D66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+          <t xml:space="preserve">Phone_Entry__c</t>
         </is>
       </c>
       <c r="F66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G66" t="inlineStr" s="2">
@@ -15299,22 +15539,22 @@
       </c>
       <c r="D67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadTrigger</t>
+          <t xml:space="preserve">Secondary_Phone_Entry__c</t>
         </is>
       </c>
       <c r="F67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H67" t="inlineStr" s="2">
@@ -15339,7 +15579,7 @@
       </c>
       <c r="L67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call LeadPhoneEntryHandler before insert / update</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -15359,12 +15599,12 @@
       </c>
       <c r="D68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NewLeadCmp</t>
+          <t xml:space="preserve">LeadPhoneEntryHandler</t>
         </is>
       </c>
       <c r="F68" t="inlineStr" s="2">
@@ -15374,7 +15614,7 @@
       </c>
       <c r="G68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H68" t="inlineStr" s="2">
@@ -15384,7 +15624,7 @@
       </c>
       <c r="I68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
       <c r="J68" t="inlineStr" s="2">
@@ -15399,7 +15639,7 @@
       </c>
       <c r="L68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone inputs use entry fields</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -15419,12 +15659,12 @@
       </c>
       <c r="D69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NewRefLeadCmp</t>
+          <t xml:space="preserve">LeadTriggerHandler</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="2">
@@ -15459,7 +15699,7 @@
       </c>
       <c r="L69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone inputs use entry fields</t>
+          <t xml:space="preserve">Hook for entry-field copy (if routed through handler)</t>
         </is>
       </c>
     </row>
@@ -15479,12 +15719,12 @@
       </c>
       <c r="D70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="2">
@@ -15494,7 +15734,7 @@
       </c>
       <c r="G70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H70" t="inlineStr" s="2">
@@ -15519,7 +15759,7 @@
       </c>
       <c r="L70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -15539,12 +15779,12 @@
       </c>
       <c r="D71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">LeadTrigger</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="2">
@@ -15579,7 +15819,7 @@
       </c>
       <c r="L71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Call LeadPhoneEntryHandler before insert / update</t>
         </is>
       </c>
     </row>
@@ -15589,32 +15829,32 @@
       </c>
       <c r="B72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_To_Masked__c</t>
+          <t xml:space="preserve">NewLeadCmp</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_Detail__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H72" t="inlineStr" s="2">
@@ -15639,7 +15879,7 @@
       </c>
       <c r="L72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone inputs use entry fields</t>
         </is>
       </c>
     </row>
@@ -15649,32 +15889,32 @@
       </c>
       <c r="B73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Masked__c</t>
+          <t xml:space="preserve">NewRefLeadCmp</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H73" t="inlineStr" s="2">
@@ -15699,7 +15939,7 @@
       </c>
       <c r="L73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone inputs use entry fields</t>
         </is>
       </c>
     </row>
@@ -15709,32 +15949,32 @@
       </c>
       <c r="B74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H74" t="inlineStr" s="2">
@@ -15759,7 +15999,7 @@
       </c>
       <c r="L74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -15769,22 +16009,22 @@
       </c>
       <c r="B75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadBulkPushController</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="2">
@@ -15819,7 +16059,7 @@
       </c>
       <c r="L75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -15839,22 +16079,22 @@
       </c>
       <c r="D76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadHistoryandActivityController</t>
+          <t xml:space="preserve">Call_To_Masked__c</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call_Detail__c</t>
         </is>
       </c>
       <c r="G76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H76" t="inlineStr" s="2">
@@ -15879,7 +16119,7 @@
       </c>
       <c r="L76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return Call_To__c masked</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -15899,22 +16139,22 @@
       </c>
       <c r="D77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeController</t>
+          <t xml:space="preserve">Phone_Masked__c</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H77" t="inlineStr" s="2">
@@ -15939,7 +16179,7 @@
       </c>
       <c r="L77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -15959,22 +16199,22 @@
       </c>
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMsgConversationController</t>
+          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H78" t="inlineStr" s="2">
@@ -15999,7 +16239,7 @@
       </c>
       <c r="L78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Resolve number server-side for send</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -16024,7 +16264,7 @@
       </c>
       <c r="E79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadYotelBulkPushController</t>
+          <t xml:space="preserve">LeadBulkPushController</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
@@ -16084,7 +16324,7 @@
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MakeCallController</t>
+          <t xml:space="preserve">LeadHistoryandActivityController</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -16119,7 +16359,7 @@
       </c>
       <c r="L80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values; number resolved server-side</t>
+          <t xml:space="preserve">Return Call_To__c masked</t>
         </is>
       </c>
     </row>
@@ -16144,7 +16384,7 @@
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">LeadMergeController</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
@@ -16179,7 +16419,7 @@
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask numbers before writing log__c</t>
+          <t xml:space="preserve">Return masked values</t>
         </is>
       </c>
     </row>
@@ -16204,7 +16444,7 @@
       </c>
       <c r="E82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OfflineCallAppAPI</t>
+          <t xml:space="preserve">LeadMsgConversationController</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
@@ -16239,7 +16479,7 @@
       </c>
       <c r="L82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server-side number lookup</t>
+          <t xml:space="preserve">Resolve number server-side for send</t>
         </is>
       </c>
     </row>
@@ -16264,7 +16504,7 @@
       </c>
       <c r="E83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updateContactDetails</t>
+          <t xml:space="preserve">LeadYotelBulkPushController</t>
         </is>
       </c>
       <c r="F83" t="inlineStr" s="2">
@@ -16299,7 +16539,7 @@
       </c>
       <c r="L83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Same</t>
+          <t xml:space="preserve">Return masked values</t>
         </is>
       </c>
     </row>
@@ -16319,12 +16559,12 @@
       </c>
       <c r="D84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">MakeCallController</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
@@ -16359,7 +16599,7 @@
       </c>
       <c r="L84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve">Return masked values; number resolved server-side</t>
         </is>
       </c>
     </row>
@@ -16379,12 +16619,12 @@
       </c>
       <c r="D85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
@@ -16419,7 +16659,7 @@
       </c>
       <c r="L85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve">Mask numbers before writing log__c</t>
         </is>
       </c>
     </row>
@@ -16439,12 +16679,12 @@
       </c>
       <c r="D86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeCmp</t>
+          <t xml:space="preserve">OfflineCallAppAPI</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
@@ -16479,7 +16719,7 @@
       </c>
       <c r="L86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve">Server-side number lookup</t>
         </is>
       </c>
     </row>
@@ -16499,12 +16739,12 @@
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MakeCall</t>
+          <t xml:space="preserve">updateContactDetails</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
@@ -16539,7 +16779,7 @@
       </c>
       <c r="L87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers on screen</t>
+          <t xml:space="preserve">Same</t>
         </is>
       </c>
     </row>
@@ -16564,7 +16804,7 @@
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeLightningPage</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
@@ -16599,7 +16839,7 @@
       </c>
       <c r="L88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show Call_To__c masked</t>
+          <t xml:space="preserve">Show masked field</t>
         </is>
       </c>
     </row>
@@ -16624,7 +16864,7 @@
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
@@ -16659,7 +16899,7 @@
       </c>
       <c r="L89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Show masked field</t>
         </is>
       </c>
     </row>
@@ -16679,12 +16919,12 @@
       </c>
       <c r="D90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">LeadMergeCmp</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
@@ -16719,7 +16959,7 @@
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Masked numbers</t>
         </is>
       </c>
     </row>
@@ -16739,12 +16979,12 @@
       </c>
       <c r="D91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">MakeCall</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -16779,7 +17019,7 @@
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Masked numbers on screen</t>
         </is>
       </c>
     </row>
@@ -16799,12 +17039,12 @@
       </c>
       <c r="D92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">mCubeLightningPage</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
@@ -16839,7 +17079,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Show Call_To__c masked</t>
         </is>
       </c>
     </row>
@@ -16859,12 +17099,12 @@
       </c>
       <c r="D93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">offlineCallQuickActionCmp</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F93" t="inlineStr" s="2">
@@ -16899,7 +17139,7 @@
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -16924,7 +17164,7 @@
       </c>
       <c r="E94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">utilityCallComponent</t>
+          <t xml:space="preserve">leadBulkPush</t>
         </is>
       </c>
       <c r="F94" t="inlineStr" s="2">
@@ -16959,7 +17199,7 @@
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -16969,32 +17209,32 @@
       </c>
       <c r="B95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H95" t="inlineStr" s="2">
@@ -17019,7 +17259,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -17029,22 +17269,22 @@
       </c>
       <c r="B96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">leadYotelPush</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -17054,7 +17294,7 @@
       </c>
       <c r="G96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H96" t="inlineStr" s="2">
@@ -17079,7 +17319,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -17089,22 +17329,22 @@
       </c>
       <c r="B97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">offlineCallQuickActionCmp</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -17114,7 +17354,7 @@
       </c>
       <c r="G97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H97" t="inlineStr" s="2">
@@ -17124,7 +17364,7 @@
       </c>
       <c r="I97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J97" t="inlineStr" s="2">
@@ -17139,7 +17379,7 @@
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve">G-Talk: send recordId only</t>
         </is>
       </c>
     </row>
@@ -17149,22 +17389,22 @@
       </c>
       <c r="B98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">utilityCallComponent</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -17174,7 +17414,7 @@
       </c>
       <c r="G98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H98" t="inlineStr" s="2">
@@ -17184,7 +17424,7 @@
       </c>
       <c r="I98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J98" t="inlineStr" s="2">
@@ -17199,7 +17439,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">G-Talk: send recordId only</t>
         </is>
       </c>
     </row>
@@ -17219,17 +17459,17 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G99" t="inlineStr" s="2">
@@ -17279,12 +17519,12 @@
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
@@ -17339,12 +17579,12 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
@@ -17364,7 +17604,7 @@
       </c>
       <c r="I101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J101" t="inlineStr" s="2">
@@ -17379,7 +17619,7 @@
       </c>
       <c r="L101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -17399,12 +17639,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -17424,7 +17664,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -17449,22 +17689,22 @@
       </c>
       <c r="B103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -17484,7 +17724,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -17499,7 +17739,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -17509,12 +17749,12 @@
       </c>
       <c r="B104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D104" t="inlineStr" s="2">
@@ -17524,7 +17764,7 @@
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -17569,22 +17809,22 @@
       </c>
       <c r="B105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -17594,7 +17834,7 @@
       </c>
       <c r="G105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H105" t="inlineStr" s="2">
@@ -17619,7 +17859,7 @@
       </c>
       <c r="L105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -17629,27 +17869,27 @@
       </c>
       <c r="B106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G106" t="inlineStr" s="2">
@@ -17664,7 +17904,7 @@
       </c>
       <c r="I106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J106" t="inlineStr" s="2">
@@ -17699,12 +17939,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -17714,7 +17954,7 @@
       </c>
       <c r="G107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H107" t="inlineStr" s="2">
@@ -17724,7 +17964,7 @@
       </c>
       <c r="I107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J107" t="inlineStr" s="2">
@@ -17739,7 +17979,7 @@
       </c>
       <c r="L107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -17759,12 +17999,12 @@
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -17774,7 +18014,7 @@
       </c>
       <c r="G108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H108" t="inlineStr" s="2">
@@ -17799,7 +18039,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -17809,22 +18049,22 @@
       </c>
       <c r="B109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
@@ -17834,7 +18074,7 @@
       </c>
       <c r="G109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H109" t="inlineStr" s="2">
@@ -17844,12 +18084,12 @@
       </c>
       <c r="I109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K109" t="inlineStr" s="6">
@@ -17859,7 +18099,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -17869,27 +18109,27 @@
       </c>
       <c r="B110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G110" t="inlineStr" s="2">
@@ -17904,12 +18144,12 @@
       </c>
       <c r="I110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K110" t="inlineStr" s="6">
@@ -17929,22 +18169,22 @@
       </c>
       <c r="B111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
@@ -17954,7 +18194,7 @@
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -17964,12 +18204,12 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K111" t="inlineStr" s="6">
@@ -17979,7 +18219,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -17989,22 +18229,22 @@
       </c>
       <c r="B112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
@@ -18029,7 +18269,7 @@
       </c>
       <c r="J112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K112" t="inlineStr" s="6">
@@ -18039,7 +18279,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -18049,22 +18289,22 @@
       </c>
       <c r="B113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -18074,7 +18314,7 @@
       </c>
       <c r="G113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H113" t="inlineStr" s="2">
@@ -18084,7 +18324,7 @@
       </c>
       <c r="I113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J113" t="inlineStr" s="2">
@@ -18099,7 +18339,7 @@
       </c>
       <c r="L113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18109,22 +18349,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -18134,7 +18374,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -18159,7 +18399,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18169,22 +18409,22 @@
       </c>
       <c r="B115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -18194,7 +18434,7 @@
       </c>
       <c r="G115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H115" t="inlineStr" s="2">
@@ -18204,7 +18444,7 @@
       </c>
       <c r="I115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -18219,7 +18459,7 @@
       </c>
       <c r="L115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -18229,12 +18469,12 @@
       </c>
       <c r="B116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D116" t="inlineStr" s="2">
@@ -18244,7 +18484,7 @@
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -18279,7 +18519,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -18299,12 +18539,12 @@
       </c>
       <c r="D117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -18339,7 +18579,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -18359,12 +18599,12 @@
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -18419,12 +18659,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -18484,7 +18724,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -18519,7 +18759,7 @@
       </c>
       <c r="L120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -18539,12 +18779,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -18579,7 +18819,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -18589,22 +18829,22 @@
       </c>
       <c r="B122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -18629,7 +18869,7 @@
       </c>
       <c r="J122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K122" t="inlineStr" s="6">
@@ -18639,7 +18879,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -18649,22 +18889,22 @@
       </c>
       <c r="B123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -18689,7 +18929,7 @@
       </c>
       <c r="J123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K123" t="inlineStr" s="6">
@@ -18699,7 +18939,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -18709,22 +18949,22 @@
       </c>
       <c r="B124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -18749,7 +18989,7 @@
       </c>
       <c r="J124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K124" t="inlineStr" s="6">
@@ -18759,7 +18999,7 @@
       </c>
       <c r="L124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -18769,22 +19009,22 @@
       </c>
       <c r="B125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -18809,7 +19049,7 @@
       </c>
       <c r="J125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K125" t="inlineStr" s="6">
@@ -18819,7 +19059,7 @@
       </c>
       <c r="L125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -18844,7 +19084,7 @@
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -18899,12 +19139,12 @@
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -18914,7 +19154,7 @@
       </c>
       <c r="G127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H127" t="inlineStr" s="2">
@@ -18939,7 +19179,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -18959,12 +19199,12 @@
       </c>
       <c r="D128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -18979,7 +19219,7 @@
       </c>
       <c r="H128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I128" t="inlineStr" s="2">
@@ -18999,7 +19239,7 @@
       </c>
       <c r="L128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -19019,12 +19259,12 @@
       </c>
       <c r="D129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -19039,7 +19279,7 @@
       </c>
       <c r="H129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I129" t="inlineStr" s="2">
@@ -19049,7 +19289,7 @@
       </c>
       <c r="J129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K129" t="inlineStr" s="6">
@@ -19059,7 +19299,7 @@
       </c>
       <c r="L129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -19069,22 +19309,22 @@
       </c>
       <c r="B130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F130" t="inlineStr" s="2">
@@ -19094,7 +19334,7 @@
       </c>
       <c r="G130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H130" t="inlineStr" s="2">
@@ -19109,7 +19349,7 @@
       </c>
       <c r="J130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K130" t="inlineStr" s="6">
@@ -19119,7 +19359,7 @@
       </c>
       <c r="L130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -19129,22 +19369,22 @@
       </c>
       <c r="B131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -19154,7 +19394,7 @@
       </c>
       <c r="G131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H131" t="inlineStr" s="2">
@@ -19169,7 +19409,7 @@
       </c>
       <c r="J131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K131" t="inlineStr" s="6">
@@ -19179,7 +19419,7 @@
       </c>
       <c r="L131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -19189,22 +19429,22 @@
       </c>
       <c r="B132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F132" t="inlineStr" s="2">
@@ -19219,7 +19459,7 @@
       </c>
       <c r="H132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I132" t="inlineStr" s="2">
@@ -19229,7 +19469,7 @@
       </c>
       <c r="J132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K132" t="inlineStr" s="6">
@@ -19239,7 +19479,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -19249,22 +19489,22 @@
       </c>
       <c r="B133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -19279,7 +19519,7 @@
       </c>
       <c r="H133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I133" t="inlineStr" s="2">
@@ -19289,7 +19529,7 @@
       </c>
       <c r="J133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K133" t="inlineStr" s="6">
@@ -19299,7 +19539,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -19309,22 +19549,22 @@
       </c>
       <c r="B134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -19334,12 +19574,12 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I134" t="inlineStr" s="2">
@@ -19349,7 +19589,7 @@
       </c>
       <c r="J134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K134" t="inlineStr" s="6">
@@ -19359,7 +19599,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -19369,22 +19609,22 @@
       </c>
       <c r="B135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -19394,12 +19634,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -19409,7 +19649,7 @@
       </c>
       <c r="J135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K135" t="inlineStr" s="6">
@@ -19419,7 +19659,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -19429,22 +19669,22 @@
       </c>
       <c r="B136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -19454,12 +19694,12 @@
       </c>
       <c r="G136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I136" t="inlineStr" s="2">
@@ -19469,7 +19709,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -19479,7 +19719,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -19489,22 +19729,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -19514,12 +19754,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -19529,7 +19769,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -19539,7 +19779,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -19549,7 +19789,7 @@
       </c>
       <c r="B138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C138" t="inlineStr" s="2">
@@ -19564,7 +19804,7 @@
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -19599,7 +19839,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -19609,7 +19849,7 @@
       </c>
       <c r="B139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C139" t="inlineStr" s="2">
@@ -19624,7 +19864,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -19649,7 +19889,7 @@
       </c>
       <c r="J139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K139" t="inlineStr" s="6">
@@ -19659,7 +19899,7 @@
       </c>
       <c r="L139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -19669,7 +19909,7 @@
       </c>
       <c r="B140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C140" t="inlineStr" s="2">
@@ -19684,7 +19924,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -19709,7 +19949,7 @@
       </c>
       <c r="J140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K140" t="inlineStr" s="6">
@@ -19719,7 +19959,7 @@
       </c>
       <c r="L140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -19729,62 +19969,302 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M9</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K141" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2">
+        <v>138</v>
+      </c>
+      <c r="B142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M10</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K142" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2">
+        <v>139</v>
+      </c>
+      <c r="B143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K143" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2">
+        <v>140</v>
+      </c>
+      <c r="B144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K144" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2">
+        <v>141</v>
+      </c>
+      <c r="B145" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C141" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr" s="2">
+      <c r="C145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E141" t="inlineStr" s="2">
+      <c r="E145" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F141" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G141" t="inlineStr" s="2">
+      <c r="F145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H141" t="inlineStr" s="2">
+      <c r="H145" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I141" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J141" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-      <c r="K141" t="inlineStr" s="6">
+      <c r="I145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L141" t="inlineStr" s="2">
+      <c r="L145" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L141"/>
+  <autoFilter ref="A4:L145"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
deploy: v1.3.0 to sandbox; release bundle Part 3; register updated
- Code 0Afft000000LY6jCAG: 8/8, 60 tests passed (incl. existing
  McubeSoftphoneAddOnControllerTest); coverage 87.9-100%
- Pilot 0Afft000000LYBZCA4: POC page click-to-dial ON, POC profile access
- Added missing McubeMaskedClickToCallTest.cls-meta.xml
- SlashRTC CTI Adapter URL: manual step by the project owner (not deployed)
- release/prod/part3-dialers + rebuilt part1-foundations, README, SHA256SUMS
- Excel register: Part 3 deployed, Release Bundle / Release Steps sheets

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -11,8 +11,8 @@
     <sheet name="Test Classes" sheetId="7" r:id="rId7"/>
     <sheet name="Backups" sheetId="8" r:id="rId8"/>
     <sheet name="Part 3 Plan" sheetId="9" r:id="rId9"/>
-    <sheet name="Release Bundle P1-P2" sheetId="10" r:id="rId10"/>
-    <sheet name="Release Steps P1-P2" sheetId="11" r:id="rId11"/>
+    <sheet name="Release Bundle" sheetId="10" r:id="rId10"/>
+    <sheet name="Release Steps" sheetId="11" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
@@ -21,11 +21,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$59</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$145</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle P1-P2'!$A$4:$K$43</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps P1-P2'!$A$4:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$11</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -319,7 +319,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - Parts 1 and 2 (built components)</t>
+          <t>Production Release Bundle - built components (Parts 1-3)</t>
         </is>
       </c>
     </row>
@@ -423,7 +423,7 @@
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5b84b4f96887</t>
+          <t xml:space="preserve">fa00d87d27a2</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="2">
@@ -533,7 +533,7 @@
       </c>
       <c r="H7" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9cc82f98c9fd</t>
+          <t xml:space="preserve">c5bedd971363</t>
         </is>
       </c>
       <c r="I7" t="inlineStr" s="2">
@@ -863,7 +863,7 @@
       </c>
       <c r="H13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">df752a8bbf08</t>
+          <t xml:space="preserve">2de826792691</t>
         </is>
       </c>
       <c r="I13" t="inlineStr" s="2">
@@ -973,7 +973,7 @@
       </c>
       <c r="H15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">0e94577583e0</t>
+          <t xml:space="preserve">be47f9305354</t>
         </is>
       </c>
       <c r="I15" t="inlineStr" s="2">
@@ -2373,47 +2373,47 @@
       </c>
       <c r="B41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part3-dialers</t>
         </is>
       </c>
       <c r="C41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="E41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="G41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part3-dialers/classes/McubeSoftphoneAddOnController.cls</t>
         </is>
       </c>
       <c r="H41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">8ff8df2bf019</t>
+          <t xml:space="preserve">da6120f267a8</t>
         </is>
       </c>
       <c r="I41" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+          <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
       <c r="J41" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K41" t="inlineStr" s="6">
@@ -2428,47 +2428,47 @@
       </c>
       <c r="B42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part3-dialers</t>
         </is>
       </c>
       <c r="C42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 3</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.3.0</t>
         </is>
       </c>
       <c r="E42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="G42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part3-dialers/classes/McubeSoftphoneAddOnController.cls-meta.xml</t>
         </is>
       </c>
       <c r="H42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">a242f6e22b47</t>
         </is>
       </c>
       <c r="I42" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+          <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
       <c r="J42" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K42" t="inlineStr" s="6">
@@ -2483,57 +2483,717 @@
       </c>
       <c r="B43" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">McubeMaskedClickToCallTest</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/classes/McubeMaskedClickToCallTest.cls</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f6269ed82086</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2">
+        <v>3</v>
+      </c>
+      <c r="B44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">McubeMaskedClickToCallTest</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/classes/McubeMaskedClickToCallTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2">
+        <v>3</v>
+      </c>
+      <c r="B45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">slashPhone</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/aura/slashPhone/slashPhone.cmp</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">47376363b806</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2">
+        <v>3</v>
+      </c>
+      <c r="B46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">slashPhone</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/aura/slashPhone/slashPhone.cmp-meta.xml</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">785614510f32</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2">
+        <v>3</v>
+      </c>
+      <c r="B47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">slashPhone</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/aura/slashPhone/slashPhone.css</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">d0da498d01a2</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2">
+        <v>3</v>
+      </c>
+      <c r="B48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">slashPhone</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/aura/slashPhone/slashPhoneController.js</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">270ad3190442</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2">
+        <v>3</v>
+      </c>
+      <c r="B49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">slashPhone</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/aura/slashPhone/slashPhoneHelper.js</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">0dd6fb07c512</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2">
+        <v>3</v>
+      </c>
+      <c r="B50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/package.xml</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">6888e0c79e3e</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2">
+        <v>3</v>
+      </c>
+      <c r="B51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Visualforce Page</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mcubeSoftphoneCTIAddOn</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/pages/mcubeSoftphoneCTIAddOn.page</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">04cf84ceaff4</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2">
+        <v>3</v>
+      </c>
+      <c r="B52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part3-dialers</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.3.0</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Visualforce Page</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mcubeSoftphoneCTIAddOn</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part3-dialers/pages/mcubeSoftphoneCTIAddOn.page-meta.xml</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b4c9950e6bc4</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2">
+        <v>4</v>
+      </c>
+      <c r="B53" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr" s="2">
+      <c r="C53" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr" s="2">
+      <c r="D53" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr" s="2">
+      <c r="E53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">04cdfd7cd66e</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2">
+        <v>4</v>
+      </c>
+      <c r="B54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2">
+        <v>4</v>
+      </c>
+      <c r="B55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr" s="2">
+      <c r="F55" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr" s="2">
+      <c r="G55" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H43" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">9c73dfa0992e</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr" s="2">
+      <c r="H55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">e9c9172813ab</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr" s="4">
+      <c r="J55" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr" s="6">
+      <c r="K55" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K43"/>
+  <autoFilter ref="A4:K55"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -2557,7 +3217,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps - Parts 1 and 2</t>
+          <t>Production Deploy Steps (Parts 1-3)</t>
         </is>
       </c>
     </row>
@@ -2671,47 +3331,49 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2">
-        <v>4</v>
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3b</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part3-dialers</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part3-dialers --test-level RunSpecifiedTests --tests McubeMaskedClickToCallTest --tests McubeSoftphoneAddOnControllerTest</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="6">
@@ -2722,31 +3384,56 @@
     </row>
     <row r="10">
       <c r="A10" s="2">
+        <v>5</v>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2">
         <v>6</v>
       </c>
-      <c r="B10" t="inlineStr" s="2">
+      <c r="B11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr" s="2">
+      <c r="C11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="2">
+      <c r="D11" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr" s="6">
+      <c r="E11" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E10"/>
+  <autoFilter ref="A4:E11"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -2910,9 +3597,9 @@
           <t xml:space="preserve">Dialer adapters MCube + SlashRTC (POC)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="D7" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="E7" s="2">
@@ -6472,14 +7159,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I56" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I56" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J56" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K56" t="inlineStr" s="2">
@@ -6532,14 +7219,14 @@
           <t xml:space="preserve">MaskedDialServiceTest</t>
         </is>
       </c>
-      <c r="I57" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I57" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J57" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K57" t="inlineStr" s="2">
@@ -6592,14 +7279,14 @@
           <t xml:space="preserve">MaskedDialServiceCTITest</t>
         </is>
       </c>
-      <c r="I58" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I58" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J58" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K58" t="inlineStr" s="2">
@@ -6652,14 +7339,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I59" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I59" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J59" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K59" t="inlineStr" s="2">
@@ -6712,14 +7399,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I60" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I60" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J60" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K60" t="inlineStr" s="2">
@@ -6772,14 +7459,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I61" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I61" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J61" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LYBZCA4</t>
         </is>
       </c>
       <c r="K61" t="inlineStr" s="2">
@@ -6832,14 +7519,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I62" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I62" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J62" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LYBZCA4</t>
         </is>
       </c>
       <c r="K62" t="inlineStr" s="2">
@@ -8502,9 +9189,9 @@
           <t xml:space="preserve">backup/v1.3.0-pre-change</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="J6" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K6" t="inlineStr" s="2">
@@ -8562,9 +9249,9 @@
           <t xml:space="preserve">backup/v1.3.0-pre-change</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="J7" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K7" t="inlineStr" s="2">
@@ -8622,9 +9309,9 @@
           <t xml:space="preserve">backup/v1.3.0-pre-change</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="J8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LY6jCAG</t>
         </is>
       </c>
       <c r="K8" t="inlineStr" s="2">
@@ -8674,7 +9361,7 @@
       </c>
       <c r="H9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved 2026-10-06</t>
+          <t xml:space="preserve">Manual by you (Setup)</t>
         </is>
       </c>
       <c r="I9" t="inlineStr" s="2">
@@ -8684,7 +9371,7 @@
       </c>
       <c r="J9" t="inlineStr" s="8">
         <is>
-          <t xml:space="preserve">Sandbox only</t>
+          <t xml:space="preserve">Sandbox only - manual</t>
         </is>
       </c>
       <c r="K9" t="inlineStr" s="2">
@@ -20569,17 +21256,17 @@
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">SlashRTC call center adapter URL -&gt; sandbox index page</t>
+          <t xml:space="preserve">SlashRTC call center CTI Adapter URL -&gt; /apex/index (sandbox only, done manually by you)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Call Centers</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Not done</t>
+          <t xml:space="preserve">Setup &gt; Call Centers &gt; SlashRTC Call Center Adapter &gt; Edit</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="8">
+        <is>
+          <t xml:space="preserve">Manual - pending</t>
         </is>
       </c>
       <c r="F12" t="inlineStr" s="2">
@@ -21002,12 +21689,12 @@
     <row r="11">
       <c r="A11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeMaskedClickToCallTest</t>
+          <t xml:space="preserve">McubeMaskedClickToCallTest + McubeSoftphoneAddOnControllerTest</t>
         </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController.clickToCallMasked</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
@@ -21017,98 +21704,94 @@
       </c>
       <c r="D11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">target &gt; 85%</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">87.9%</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+          <t xml:space="preserve">MaskedDialServiceTest (v1.3.0, +5)</t>
         </is>
       </c>
       <c r="B12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+          <t xml:space="preserve">MaskedDialService</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D12" s="2">
+        <v>23</v>
       </c>
       <c r="E12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">target &gt; 85%</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">100%</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(existing test classes of Part 5 components)</t>
+          <t xml:space="preserve">MaskedDialServiceCTITest (v1.3.0, +3)</t>
         </is>
       </c>
       <c r="B13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5 changed classes</t>
+          <t xml:space="preserve">MaskedDialServiceCTI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+          <t xml:space="preserve">Part 3</t>
+        </is>
+      </c>
+      <c r="D13" s="2">
+        <v>9</v>
       </c>
       <c r="E13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">keep &gt;= current</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">94.4%</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">LeadPhoneEntryHandler</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="2">
@@ -21130,17 +21813,17 @@
     <row r="15">
       <c r="A15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">(existing test classes of Part 5 components)</t>
         </is>
       </c>
       <c r="B15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Part 5 changed classes</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="2">
@@ -21150,7 +21833,7 @@
       </c>
       <c r="E15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">target &gt; 85%</t>
+          <t xml:space="preserve">keep &gt;= current</t>
         </is>
       </c>
       <c r="F15" t="inlineStr" s="6">
@@ -21162,17 +21845,17 @@
     <row r="16">
       <c r="A16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="B16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService, FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="2">
@@ -21194,37 +21877,101 @@
     <row r="17">
       <c r="A17" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">target &gt; 85%</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FreeTextMaskService, FeedItemPhoneMaskTrigger</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 7</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">target &gt; 85%</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr" s="2">
+      <c r="B19" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr" s="2">
+      <c r="C19" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 8</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr" s="2">
+      <c r="D19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">target &gt; 85%</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr" s="7">
+      <c r="F19" t="inlineStr" s="7">
         <is>
           <t xml:space="preserve">Conditional</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F17"/>
+  <autoFilter ref="A4:F19"/>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>

</xml_diff>

<commit_message>
docs: Part 4 plan in the register (components, impact, backup)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -13,19 +13,21 @@
     <sheet name="Part 3 Plan" sheetId="9" r:id="rId9"/>
     <sheet name="Release Bundle" sheetId="10" r:id="rId10"/>
     <sheet name="Release Steps" sheetId="11" r:id="rId11"/>
+    <sheet name="Part 4 Plan" sheetId="12" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$88</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$145</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$146</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -3443,6 +3445,459 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="70" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 4 (v1.4.0) - Lead creation with hidden numbers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; originals backed up in backup/v1.4.0-pre-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Field (Phone)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lead.Phone_Entry__c</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Label "Phone". Reps type the primary number here when creating a Lead. Always empty after save.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked reps can create Leads</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Field (Phone)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lead.Secondary_Phone_Entry__c</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Label "Secondary Phone". Add / change the secondary number. Always empty after save.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked reps can add or change the secondary number</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Before insert / update: copies entry -&gt; Phone__c / Secondary_Phone__c and clears the entry fields. Primary is locked once set (error if an entry value tries to change it). Bulk-safe, no SOQL / DML.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Numbers are saved in the real (hidden) fields exactly as today</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Insert, update, lock, secondary change, blank, 200-record bulk, runAs masked user; &gt; 85%, no SeeAllData</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Trigger</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadTrigger</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Add ONE call at the very top (after the bypass check): LeadPhoneEntryHandler.beforeSave(...) for before insert / update. Everything else unchanged.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Formatting, duplicate check, round robin and validation rules all see the copied number as today</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Medium: LeadTrigger runs for every Lead save; covered by existing LeadTrigger tests + new tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp (Lead New button, desktop + mobile)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">In the existing onload step: if the form did not receive Phone__c (user cannot see it), show the entry inputs (required Phone + Secondary Phone) instead.</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Users who can see Phone__c: no change. Masked users: same form, entry inputs.</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewRefLeadCmp (New Referral Lead quick action)</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Same as NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Same</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New (update)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Profile</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Edit access to the 2 entry fields</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">POC users can type numbers</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New (update)</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Add "Secondary Phone" entry field to the details so POC users can add / change the secondary number</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">POC users only</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">RelatedSourceHandler, LeadTriggerHandler</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing formatting + duplicate check keep working on Phone__c</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Deferred to Part 11</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New_Lead_Page, New_Lead_Page1_sales</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone fields swapped for panel + entry field at go-live</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change now</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Unaffected</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Integrations</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Website / portals / MCube / LeadCreationAPI</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Still write Phone__c directly; entry fields not used</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F16"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
@@ -3631,9 +4086,9 @@
           <t xml:space="preserve">Lead creation with hidden numbers</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="D8" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="E8" s="2">
@@ -7639,9 +8094,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I64" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I64" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J64" t="inlineStr" s="2">
@@ -7699,9 +8154,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I65" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I65" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J65" t="inlineStr" s="2">
@@ -7759,9 +8214,9 @@
           <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I66" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J66" t="inlineStr" s="2">
@@ -7819,9 +8274,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I67" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I67" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J67" t="inlineStr" s="2">
@@ -7846,32 +8301,32 @@
       </c>
       <c r="B68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Masked__c</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked primary for layouts / list views / reports</t>
+          <t xml:space="preserve">Edit access to Phone_Entry__c, Secondary_Phone_Entry__c</t>
         </is>
       </c>
       <c r="H68" t="inlineStr" s="2">
@@ -7879,9 +8334,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I68" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I68" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J68" t="inlineStr" s="2">
@@ -7891,12 +8346,12 @@
       </c>
       <c r="K68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="L68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Reps get it at go-live (Part 11)</t>
         </is>
       </c>
     </row>
@@ -7906,32 +8361,32 @@
       </c>
       <c r="B69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="C69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="D69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Lightning Page (update of new)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked secondary</t>
+          <t xml:space="preserve">Add Secondary_Phone_Entry__c (New secondary number) to the details</t>
         </is>
       </c>
       <c r="H69" t="inlineStr" s="2">
@@ -7939,9 +8394,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I69" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I69" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J69" t="inlineStr" s="2">
@@ -7951,7 +8406,7 @@
       </c>
       <c r="K69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="L69" t="inlineStr" s="2">
@@ -7981,17 +8436,17 @@
       </c>
       <c r="E70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_To_Masked__c</t>
+          <t xml:space="preserve">Phone_Masked__c</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_Detail__c</t>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked call number</t>
+          <t xml:space="preserve">Formula: masked primary for layouts / list views / reports</t>
         </is>
       </c>
       <c r="H70" t="inlineStr" s="2">
@@ -8026,37 +8481,37 @@
       </c>
       <c r="B71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal for TL / Head / Admin: reason, 30 s, audit</t>
+          <t xml:space="preserve">Formula: masked secondary</t>
         </is>
       </c>
       <c r="H71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I71" t="inlineStr" s="6">
@@ -8086,32 +8541,32 @@
       </c>
       <c r="B72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">Call_To_Masked__c</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call_Detail__c</t>
         </is>
       </c>
       <c r="G72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Formula: masked call number</t>
         </is>
       </c>
       <c r="H72" t="inlineStr" s="2">
@@ -8156,27 +8611,27 @@
       </c>
       <c r="D73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
+          <t xml:space="preserve">Reveal for TL / Head / Admin: reason, 30 s, audit</t>
         </is>
       </c>
       <c r="H73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="I73" t="inlineStr" s="6">
@@ -8216,12 +8671,12 @@
       </c>
       <c r="D74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
@@ -8231,7 +8686,7 @@
       </c>
       <c r="G74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Who may reveal</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H74" t="inlineStr" s="2">
@@ -8276,22 +8731,22 @@
       </c>
       <c r="D75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grants Reveal_Phone_Number to TL / Head / Admin</t>
+          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
         </is>
       </c>
       <c r="H75" t="inlineStr" s="2">
@@ -8336,12 +8791,12 @@
       </c>
       <c r="D76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
@@ -8351,12 +8806,12 @@
       </c>
       <c r="G76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nightly delete of audit rows older than 1 year (batch + schedulable)</t>
+          <t xml:space="preserve">Who may reveal</t>
         </is>
       </c>
       <c r="H76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I76" t="inlineStr" s="6">
@@ -8376,7 +8831,7 @@
       </c>
       <c r="L76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8396,12 +8851,12 @@
       </c>
       <c r="D77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
@@ -8411,7 +8866,7 @@
       </c>
       <c r="G77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Grants Reveal_Phone_Number to TL / Head / Admin</t>
         </is>
       </c>
       <c r="H77" t="inlineStr" s="2">
@@ -8456,12 +8911,12 @@
       </c>
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
@@ -8471,12 +8926,12 @@
       </c>
       <c r="G78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add Reveal button + reason picker</t>
+          <t xml:space="preserve">Nightly delete of audit rows older than 1 year (batch + schedulable)</t>
         </is>
       </c>
       <c r="H78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="I78" t="inlineStr" s="6">
@@ -8496,7 +8951,7 @@
       </c>
       <c r="L78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -8506,22 +8961,22 @@
       </c>
       <c r="B79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
@@ -8531,12 +8986,12 @@
       </c>
       <c r="G79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masks numbers typed in free text on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I79" t="inlineStr" s="6">
@@ -8556,7 +9011,7 @@
       </c>
       <c r="L79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8566,22 +9021,22 @@
       </c>
       <c r="B80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -8591,7 +9046,7 @@
       </c>
       <c r="G80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Add Reveal button + reason picker</t>
         </is>
       </c>
       <c r="H80" t="inlineStr" s="2">
@@ -8636,22 +9091,22 @@
       </c>
       <c r="D81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masks numbers in Chatter posts</t>
+          <t xml:space="preserve">Masks numbers typed in free text on save</t>
         </is>
       </c>
       <c r="H81" t="inlineStr" s="2">
@@ -8676,7 +9131,7 @@
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -8686,22 +9141,22 @@
       </c>
       <c r="B82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
@@ -8711,17 +9166,17 @@
       </c>
       <c r="G82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Search a number, masked result, audited</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
-        </is>
-      </c>
-      <c r="I82" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J82" t="inlineStr" s="2">
@@ -8731,12 +9186,12 @@
       </c>
       <c r="K82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8746,42 +9201,42 @@
       </c>
       <c r="B83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server side of findByNumber</t>
+          <t xml:space="preserve">Masks numbers in Chatter posts</t>
         </is>
       </c>
       <c r="H83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
-        </is>
-      </c>
-      <c r="I83" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J83" t="inlineStr" s="2">
@@ -8791,7 +9246,7 @@
       </c>
       <c r="K83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L83" t="inlineStr" s="2">
@@ -8816,12 +9271,12 @@
       </c>
       <c r="D84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
@@ -8831,12 +9286,12 @@
       </c>
       <c r="G84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Search a number, masked result, audited</t>
         </is>
       </c>
       <c r="H84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="I84" t="inlineStr" s="7">
@@ -8856,7 +9311,7 @@
       </c>
       <c r="L84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -8866,22 +9321,22 @@
       </c>
       <c r="B85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
@@ -8891,17 +9346,17 @@
       </c>
       <c r="G85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Full phone-field access for integration users</t>
+          <t xml:space="preserve">Server side of findByNumber</t>
         </is>
       </c>
       <c r="H85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="J85" t="inlineStr" s="2">
@@ -8911,12 +9366,12 @@
       </c>
       <c r="K85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="L85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -8926,62 +9381,182 @@
       </c>
       <c r="B86" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 8</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.8.0</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="L86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2">
+        <v>83</v>
+      </c>
+      <c r="B87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v2.0.0</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Full phone-field access for integration users</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign to integration users</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2">
+        <v>84</v>
+      </c>
+      <c r="B88" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Security fix</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr" s="2">
+      <c r="C88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">optional</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr" s="2">
+      <c r="D88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
-      <c r="E86" t="inlineStr" s="2">
+      <c r="E88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
-      <c r="F86" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr" s="2">
+      <c r="F88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">MCube endpoint + key over HTTPS instead of hard-coded token / http</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr" s="6">
+      <c r="H88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Planned</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K86" t="inlineStr" s="2">
+      <c r="J88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr" s="2">
+      <c r="L88" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L86"/>
+  <autoFilter ref="A4:L88"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -9471,22 +10046,22 @@
       </c>
       <c r="F11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone inputs use entry fields</t>
+          <t xml:space="preserve">On form load: if the user cannot see Phone__c, show Phone (entry) + Secondary Phone (entry) inputs instead</t>
         </is>
       </c>
       <c r="G11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone__c input disappears for masked users</t>
+          <t xml:space="preserve">Phone__c input disappears for masked users, so they could not create Leads</t>
         </is>
       </c>
       <c r="H11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
       <c r="J11" t="inlineStr" s="6">
@@ -9501,7 +10076,7 @@
       </c>
       <c r="L11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">No change for users who can see Phone__c</t>
         </is>
       </c>
     </row>
@@ -9531,7 +10106,7 @@
       </c>
       <c r="F12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone inputs use entry fields</t>
+          <t xml:space="preserve">Same as NewLeadCmp (New Referral Lead quick action)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr" s="2">
@@ -9541,12 +10116,12 @@
       </c>
       <c r="H12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
       <c r="J12" t="inlineStr" s="6">
@@ -9591,22 +10166,22 @@
       </c>
       <c r="F13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call LeadPhoneEntryHandler before insert / update</t>
+          <t xml:space="preserve">One call at the very top (before insert / update): LeadPhoneEntryHandler copies entry fields before the existing formatting and duplicate check</t>
         </is>
       </c>
       <c r="G13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Copy entry fields</t>
+          <t xml:space="preserve">Copy must run before RelatedSourceHandler.checkMobileNumber / duplicateCheck</t>
         </is>
       </c>
       <c r="H13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
       <c r="J13" t="inlineStr" s="6">
@@ -9621,7 +10196,7 @@
       </c>
       <c r="L13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Existing logic untouched</t>
         </is>
       </c>
     </row>
@@ -9646,37 +10221,37 @@
       </c>
       <c r="E14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadTriggerHandler</t>
+          <t xml:space="preserve">LeadTriggerHandler / RelatedSourceHandler</t>
         </is>
       </c>
       <c r="F14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hook for entry-field copy (if routed through handler)</t>
+          <t xml:space="preserve">No change (existing tests re-run)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep trigger thin</t>
+          <t xml:space="preserve">Dependency</t>
         </is>
       </c>
       <c r="H14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
         </is>
       </c>
       <c r="K14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L14" t="inlineStr" s="2">
@@ -9691,12 +10266,12 @@
       </c>
       <c r="B15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="2">
@@ -9726,7 +10301,7 @@
       </c>
       <c r="I15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
       <c r="J15" t="inlineStr" s="6">
@@ -9751,12 +10326,12 @@
       </c>
       <c r="B16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="2">
@@ -9786,7 +10361,7 @@
       </c>
       <c r="I16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
       <c r="J16" t="inlineStr" s="6">
@@ -16346,12 +16921,12 @@
       </c>
       <c r="D69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadTriggerHandler</t>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
       <c r="F69" t="inlineStr" s="2">
@@ -16361,7 +16936,7 @@
       </c>
       <c r="G69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H69" t="inlineStr" s="2">
@@ -16386,7 +16961,7 @@
       </c>
       <c r="L69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Hook for entry-field copy (if routed through handler)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -16406,12 +16981,12 @@
       </c>
       <c r="D70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+          <t xml:space="preserve">LeadTrigger</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="2">
@@ -16421,7 +16996,7 @@
       </c>
       <c r="G70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H70" t="inlineStr" s="2">
@@ -16446,7 +17021,7 @@
       </c>
       <c r="L70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">One call at the very top (before insert / update): LeadPhoneEntryHandler copies entry fields before the existing formatting and duplicate check</t>
         </is>
       </c>
     </row>
@@ -16466,12 +17041,12 @@
       </c>
       <c r="D71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadTrigger</t>
+          <t xml:space="preserve">NewLeadCmp</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="2">
@@ -16506,7 +17081,7 @@
       </c>
       <c r="L71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call LeadPhoneEntryHandler before insert / update</t>
+          <t xml:space="preserve">On form load: if the user cannot see Phone__c, show Phone (entry) + Secondary Phone (entry) inputs instead</t>
         </is>
       </c>
     </row>
@@ -16531,7 +17106,7 @@
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NewLeadCmp</t>
+          <t xml:space="preserve">NewRefLeadCmp</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
@@ -16566,7 +17141,7 @@
       </c>
       <c r="L72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone inputs use entry fields</t>
+          <t xml:space="preserve">Same as NewLeadCmp (New Referral Lead quick action)</t>
         </is>
       </c>
     </row>
@@ -16586,12 +17161,12 @@
       </c>
       <c r="D73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Page (update of new)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">NewRefLeadCmp</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
@@ -16601,7 +17176,7 @@
       </c>
       <c r="G73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H73" t="inlineStr" s="2">
@@ -16616,7 +17191,7 @@
       </c>
       <c r="J73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K73" t="inlineStr" s="6">
@@ -16626,7 +17201,7 @@
       </c>
       <c r="L73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone inputs use entry fields</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -16646,12 +17221,12 @@
       </c>
       <c r="D74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
@@ -16661,7 +17236,7 @@
       </c>
       <c r="G74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H74" t="inlineStr" s="2">
@@ -16676,7 +17251,7 @@
       </c>
       <c r="J74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K74" t="inlineStr" s="6">
@@ -16686,7 +17261,7 @@
       </c>
       <c r="L74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Reps get it at go-live (Part 11)</t>
         </is>
       </c>
     </row>
@@ -16696,32 +17271,32 @@
       </c>
       <c r="B75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 4</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.4.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Call_To_Masked__c</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call_Detail__c</t>
         </is>
       </c>
       <c r="G75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H75" t="inlineStr" s="2">
@@ -16746,7 +17321,7 @@
       </c>
       <c r="L75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -16771,12 +17346,12 @@
       </c>
       <c r="E76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_To_Masked__c</t>
+          <t xml:space="preserve">Phone_Masked__c</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_Detail__c</t>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G76" t="inlineStr" s="2">
@@ -16831,7 +17406,7 @@
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Masked__c</t>
+          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
@@ -16886,22 +17461,22 @@
       </c>
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
+          <t xml:space="preserve">LeadBulkPushController</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H78" t="inlineStr" s="2">
@@ -16926,7 +17501,7 @@
       </c>
       <c r="L78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Return masked values</t>
         </is>
       </c>
     </row>
@@ -16951,7 +17526,7 @@
       </c>
       <c r="E79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadBulkPushController</t>
+          <t xml:space="preserve">LeadHistoryandActivityController</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
@@ -16986,7 +17561,7 @@
       </c>
       <c r="L79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values</t>
+          <t xml:space="preserve">Return Call_To__c masked</t>
         </is>
       </c>
     </row>
@@ -17011,7 +17586,7 @@
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadHistoryandActivityController</t>
+          <t xml:space="preserve">LeadMergeController</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -17046,7 +17621,7 @@
       </c>
       <c r="L80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return Call_To__c masked</t>
+          <t xml:space="preserve">Return masked values</t>
         </is>
       </c>
     </row>
@@ -17071,7 +17646,7 @@
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeController</t>
+          <t xml:space="preserve">LeadMsgConversationController</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
@@ -17106,7 +17681,7 @@
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values</t>
+          <t xml:space="preserve">Resolve number server-side for send</t>
         </is>
       </c>
     </row>
@@ -17131,7 +17706,7 @@
       </c>
       <c r="E82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMsgConversationController</t>
+          <t xml:space="preserve">LeadYotelBulkPushController</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
@@ -17166,7 +17741,7 @@
       </c>
       <c r="L82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Resolve number server-side for send</t>
+          <t xml:space="preserve">Return masked values</t>
         </is>
       </c>
     </row>
@@ -17191,7 +17766,7 @@
       </c>
       <c r="E83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadYotelBulkPushController</t>
+          <t xml:space="preserve">MakeCallController</t>
         </is>
       </c>
       <c r="F83" t="inlineStr" s="2">
@@ -17226,7 +17801,7 @@
       </c>
       <c r="L83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values</t>
+          <t xml:space="preserve">Return masked values; number resolved server-side</t>
         </is>
       </c>
     </row>
@@ -17251,7 +17826,7 @@
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MakeCallController</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
@@ -17286,7 +17861,7 @@
       </c>
       <c r="L84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values; number resolved server-side</t>
+          <t xml:space="preserve">Mask numbers before writing log__c</t>
         </is>
       </c>
     </row>
@@ -17311,7 +17886,7 @@
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">OfflineCallAppAPI</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
@@ -17346,7 +17921,7 @@
       </c>
       <c r="L85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask numbers before writing log__c</t>
+          <t xml:space="preserve">Server-side number lookup</t>
         </is>
       </c>
     </row>
@@ -17371,7 +17946,7 @@
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OfflineCallAppAPI</t>
+          <t xml:space="preserve">updateContactDetails</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
@@ -17406,7 +17981,7 @@
       </c>
       <c r="L86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server-side number lookup</t>
+          <t xml:space="preserve">Same</t>
         </is>
       </c>
     </row>
@@ -17426,12 +18001,12 @@
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updateContactDetails</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
@@ -17466,7 +18041,7 @@
       </c>
       <c r="L87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Same</t>
+          <t xml:space="preserve">Show masked field</t>
         </is>
       </c>
     </row>
@@ -17491,7 +18066,7 @@
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
@@ -17551,7 +18126,7 @@
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">LeadMergeCmp</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
@@ -17586,7 +18161,7 @@
       </c>
       <c r="L89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve">Masked numbers</t>
         </is>
       </c>
     </row>
@@ -17611,7 +18186,7 @@
       </c>
       <c r="E90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeCmp</t>
+          <t xml:space="preserve">MakeCall</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
@@ -17646,7 +18221,7 @@
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve">Masked numbers on screen</t>
         </is>
       </c>
     </row>
@@ -17671,7 +18246,7 @@
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MakeCall</t>
+          <t xml:space="preserve">mCubeLightningPage</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -17706,7 +18281,7 @@
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers on screen</t>
+          <t xml:space="preserve">Show Call_To__c masked</t>
         </is>
       </c>
     </row>
@@ -17731,7 +18306,7 @@
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeLightningPage</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
@@ -17766,7 +18341,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show Call_To__c masked</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -17786,12 +18361,12 @@
       </c>
       <c r="D93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">leadBulkPush</t>
         </is>
       </c>
       <c r="F93" t="inlineStr" s="2">
@@ -17826,7 +18401,7 @@
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -17851,7 +18426,7 @@
       </c>
       <c r="E94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F94" t="inlineStr" s="2">
@@ -17886,7 +18461,7 @@
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -17911,7 +18486,7 @@
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">leadYotelPush</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
@@ -17946,7 +18521,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -17971,7 +18546,7 @@
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">offlineCallQuickActionCmp</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -18006,7 +18581,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">G-Talk: send recordId only</t>
         </is>
       </c>
     </row>
@@ -18031,7 +18606,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">offlineCallQuickActionCmp</t>
+          <t xml:space="preserve">utilityCallComponent</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -18076,32 +18651,32 @@
       </c>
       <c r="B98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">utilityCallComponent</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H98" t="inlineStr" s="2">
@@ -18126,7 +18701,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18146,17 +18721,17 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G99" t="inlineStr" s="2">
@@ -18206,12 +18781,12 @@
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
@@ -18231,7 +18806,7 @@
       </c>
       <c r="I100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J100" t="inlineStr" s="2">
@@ -18246,7 +18821,7 @@
       </c>
       <c r="L100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -18271,7 +18846,7 @@
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
@@ -18291,7 +18866,7 @@
       </c>
       <c r="I101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J101" t="inlineStr" s="2">
@@ -18306,7 +18881,7 @@
       </c>
       <c r="L101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18326,12 +18901,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -18351,7 +18926,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -18391,7 +18966,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -18446,12 +19021,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -18506,12 +19081,12 @@
       </c>
       <c r="D105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -18556,22 +19131,22 @@
       </c>
       <c r="B106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -18591,7 +19166,7 @@
       </c>
       <c r="I106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J106" t="inlineStr" s="2">
@@ -18606,7 +19181,7 @@
       </c>
       <c r="L106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -18626,12 +19201,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -18651,7 +19226,7 @@
       </c>
       <c r="I107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J107" t="inlineStr" s="2">
@@ -18666,7 +19241,7 @@
       </c>
       <c r="L107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18686,12 +19261,12 @@
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -18701,7 +19276,7 @@
       </c>
       <c r="G108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H108" t="inlineStr" s="2">
@@ -18726,7 +19301,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -18751,17 +19326,17 @@
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H109" t="inlineStr" s="2">
@@ -18771,7 +19346,7 @@
       </c>
       <c r="I109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J109" t="inlineStr" s="2">
@@ -18786,7 +19361,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18806,22 +19381,22 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -18831,7 +19406,7 @@
       </c>
       <c r="I110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J110" t="inlineStr" s="2">
@@ -18846,7 +19421,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -18866,12 +19441,12 @@
       </c>
       <c r="D111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
@@ -18916,22 +19491,22 @@
       </c>
       <c r="B112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
@@ -18941,7 +19516,7 @@
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -18951,12 +19526,12 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K112" t="inlineStr" s="6">
@@ -18966,7 +19541,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -18986,12 +19561,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -19011,7 +19586,7 @@
       </c>
       <c r="I113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J113" t="inlineStr" s="2">
@@ -19046,12 +19621,12 @@
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -19071,7 +19646,7 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
@@ -19086,7 +19661,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -19111,7 +19686,7 @@
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -19121,7 +19696,7 @@
       </c>
       <c r="G115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H115" t="inlineStr" s="2">
@@ -19131,7 +19706,7 @@
       </c>
       <c r="I115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -19146,7 +19721,7 @@
       </c>
       <c r="L115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -19156,22 +19731,22 @@
       </c>
       <c r="B116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -19206,7 +19781,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -19226,12 +19801,12 @@
       </c>
       <c r="D117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -19266,7 +19841,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -19291,7 +19866,7 @@
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -19346,12 +19921,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -19386,7 +19961,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -19411,7 +19986,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -19446,7 +20021,7 @@
       </c>
       <c r="L120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -19471,7 +20046,7 @@
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -19506,7 +20081,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -19531,7 +20106,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -19591,7 +20166,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -19646,12 +20221,12 @@
       </c>
       <c r="D124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -19686,7 +20261,7 @@
       </c>
       <c r="L124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -19696,22 +20271,22 @@
       </c>
       <c r="B125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -19736,7 +20311,7 @@
       </c>
       <c r="J125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K125" t="inlineStr" s="6">
@@ -19746,7 +20321,7 @@
       </c>
       <c r="L125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -19771,7 +20346,7 @@
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -19831,7 +20406,7 @@
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -19866,7 +20441,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -20011,7 +20586,7 @@
       </c>
       <c r="E130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F130" t="inlineStr" s="2">
@@ -20046,7 +20621,7 @@
       </c>
       <c r="L130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -20066,12 +20641,12 @@
       </c>
       <c r="D131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -20081,7 +20656,7 @@
       </c>
       <c r="G131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H131" t="inlineStr" s="2">
@@ -20106,7 +20681,7 @@
       </c>
       <c r="L131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -20126,12 +20701,12 @@
       </c>
       <c r="D132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F132" t="inlineStr" s="2">
@@ -20141,12 +20716,12 @@
       </c>
       <c r="G132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I132" t="inlineStr" s="2">
@@ -20166,7 +20741,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -20186,12 +20761,12 @@
       </c>
       <c r="D133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -20216,7 +20791,7 @@
       </c>
       <c r="J133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K133" t="inlineStr" s="6">
@@ -20226,7 +20801,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -20236,22 +20811,22 @@
       </c>
       <c r="B134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -20261,12 +20836,12 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I134" t="inlineStr" s="2">
@@ -20276,7 +20851,7 @@
       </c>
       <c r="J134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K134" t="inlineStr" s="6">
@@ -20286,7 +20861,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -20306,12 +20881,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -20321,7 +20896,7 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
@@ -20346,7 +20921,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -20371,7 +20946,7 @@
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -20431,7 +21006,7 @@
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -20476,22 +21051,22 @@
       </c>
       <c r="B138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -20501,12 +21076,12 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I138" t="inlineStr" s="2">
@@ -20516,7 +21091,7 @@
       </c>
       <c r="J138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K138" t="inlineStr" s="6">
@@ -20526,7 +21101,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -20536,7 +21111,7 @@
       </c>
       <c r="B139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C139" t="inlineStr" s="2">
@@ -20551,7 +21126,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -20576,7 +21151,7 @@
       </c>
       <c r="J139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K139" t="inlineStr" s="6">
@@ -20586,7 +21161,7 @@
       </c>
       <c r="L139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -20611,7 +21186,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -20636,7 +21211,7 @@
       </c>
       <c r="J140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K140" t="inlineStr" s="6">
@@ -20646,7 +21221,7 @@
       </c>
       <c r="L140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -20656,7 +21231,7 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
@@ -20671,7 +21246,7 @@
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -20696,7 +21271,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -20706,7 +21281,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -20731,7 +21306,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -20766,7 +21341,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -20776,7 +21351,7 @@
       </c>
       <c r="B143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C143" t="inlineStr" s="2">
@@ -20791,7 +21366,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -20826,7 +21401,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -20851,7 +21426,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -20886,7 +21461,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -20896,62 +21471,122 @@
       </c>
       <c r="B145" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K145" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2">
+        <v>142</v>
+      </c>
+      <c r="B146" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C145" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr" s="2">
+      <c r="C146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E145" t="inlineStr" s="2">
+      <c r="E146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F145" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G145" t="inlineStr" s="2">
+      <c r="F146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H145" t="inlineStr" s="2">
+      <c r="H146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I145" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J145" t="inlineStr" s="2">
+      <c r="I146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="K145" t="inlineStr" s="6">
+      <c r="K146" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L145" t="inlineStr" s="2">
+      <c r="L146" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L145"/>
+  <autoFilter ref="A4:L146"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -22138,32 +22773,32 @@
     <row r="8">
       <c r="A8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before Part 4</t>
+          <t xml:space="preserve">Part 4 pre-change backup</t>
         </is>
       </c>
       <c r="B8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Re-retrieve Part 4 components and compare with baseline</t>
+          <t xml:space="preserve">LeadTrigger, NewLeadCmp, NewRefLeadCmp, RelatedSourceHandler, LeadTriggerHandler (+tests), New_Lead_Page, New_Lead_Page1_sales (changed since baseline: +8 lines tab display), Lead.New_Referral_Lead</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">backup/v1.4.0-pre-change</t>
+          <t xml:space="preserve">backup/v1.4.0-pre-change (with SHA256SUMS)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-10-06</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">9b32c8c</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Backed up</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v1.4.0 Lead creation with hidden numbers (built locally, not deployed)
New: Lead.Phone_Entry__c, Lead.Secondary_Phone_Entry__c, LeadPhoneEntryHandler
(+ test, 11 tests incl. 200-record bulk and real saves through LeadTrigger).
Existing (approved, originals in backup/v1.4.0-pre-change), additions only:
- LeadTrigger: one call at the top (before insert/update)
- NewLeadCmp, NewRefLeadCmp: entry inputs for users who cannot see Phone__c
Our components: POC profile (entry fields), POC page (Secondary Phone entry).
Manifests, release bundle part4-lead-entry, changelog, roadmap, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -25,8 +25,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$55</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -321,7 +321,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-3)</t>
+          <t>Production Release Bundle - built components (Parts 1-4)</t>
         </is>
       </c>
     </row>
@@ -3035,47 +3035,47 @@
       </c>
       <c r="B53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part4-lead-entry</t>
         </is>
       </c>
       <c r="C53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="E53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">LeadTrigger.trigger</t>
         </is>
       </c>
       <c r="G53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part4-lead-entry/triggers/LeadTrigger.trigger</t>
         </is>
       </c>
       <c r="H53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">04cdfd7cd66e</t>
+          <t xml:space="preserve">d76c4f8924ec</t>
         </is>
       </c>
       <c r="I53" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J53" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K53" t="inlineStr" s="6">
@@ -3090,47 +3090,47 @@
       </c>
       <c r="B54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part4-lead-entry</t>
         </is>
       </c>
       <c r="C54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 4</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.4.0</t>
         </is>
       </c>
       <c r="E54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">LeadTrigger.trigger</t>
         </is>
       </c>
       <c r="G54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part4-lead-entry/triggers/LeadTrigger.trigger-meta.xml</t>
         </is>
       </c>
       <c r="H54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">7a7f3d2d53ba</t>
         </is>
       </c>
       <c r="I54" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J54" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K54" t="inlineStr" s="6">
@@ -3145,57 +3145,1157 @@
       </c>
       <c r="B55" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/classes/LeadPhoneEntryHandler.cls</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">44394fa359a3</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2">
+        <v>4</v>
+      </c>
+      <c r="B56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/classes/LeadPhoneEntryHandler.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2">
+        <v>4</v>
+      </c>
+      <c r="B57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/classes/LeadPhoneEntryHandlerTest.cls</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ff4bcdf806b0</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2">
+        <v>4</v>
+      </c>
+      <c r="B58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/classes/LeadPhoneEntryHandlerTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2">
+        <v>4</v>
+      </c>
+      <c r="B59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmp.auradoc</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">60705e943572</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2">
+        <v>4</v>
+      </c>
+      <c r="B60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmp.cmp</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">a883464b3486</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2">
+        <v>4</v>
+      </c>
+      <c r="B61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmp.cmp-meta.xml</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">26bafa2e57d5</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2">
+        <v>4</v>
+      </c>
+      <c r="B62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmp.css</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">e0afee0398c4</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2">
+        <v>4</v>
+      </c>
+      <c r="B63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmp.design</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5ff4b67b38f3</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2">
+        <v>4</v>
+      </c>
+      <c r="B64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmpController.js</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">441aea094a35</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2">
+        <v>4</v>
+      </c>
+      <c r="B65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmpHelper.js</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f78896d8f5bd</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2">
+        <v>4</v>
+      </c>
+      <c r="B66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewLeadCmp</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewLeadCmp/NewLeadCmpRenderer.js</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">38731048a539</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2">
+        <v>4</v>
+      </c>
+      <c r="B67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewRefLeadCmp</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewRefLeadCmp/NewRefLeadCmp.cmp</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">8dc9a335294b</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2">
+        <v>4</v>
+      </c>
+      <c r="B68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewRefLeadCmp</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewRefLeadCmp/NewRefLeadCmp.cmp-meta.xml</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3757f400d527</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2">
+        <v>4</v>
+      </c>
+      <c r="B69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewRefLeadCmp</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewRefLeadCmp/NewRefLeadCmpController.js</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">1645bb0df45f</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2">
+        <v>4</v>
+      </c>
+      <c r="B70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">NewRefLeadCmp</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/aura/NewRefLeadCmp/NewRefLeadCmpHelper.js</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f78896d8f5bd</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2">
+        <v>4</v>
+      </c>
+      <c r="B71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lead</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/objects/Lead.object</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">aafbb3299259</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2">
+        <v>4</v>
+      </c>
+      <c r="B72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part4-lead-entry</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 4</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.4.0</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part4-lead-entry/package.xml</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9451f1667341</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2">
+        <v>5</v>
+      </c>
+      <c r="B73" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr" s="2">
+      <c r="C73" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D55" t="inlineStr" s="2">
+      <c r="D73" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr" s="2">
+      <c r="E73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2">
+        <v>5</v>
+      </c>
+      <c r="B74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2">
+        <v>5</v>
+      </c>
+      <c r="B75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F55" t="inlineStr" s="2">
+      <c r="F75" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G55" t="inlineStr" s="2">
+      <c r="G75" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H55" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">e9c9172813ab</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr" s="2">
+      <c r="H75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">86d290d2bafe</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr" s="4">
+      <c r="J75" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K55" t="inlineStr" s="6">
+      <c r="K75" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K55"/>
+  <autoFilter ref="A4:K75"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -3219,7 +4319,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-3)</t>
+          <t>Production Deploy Steps (Parts 1-4)</t>
         </is>
       </c>
     </row>
@@ -3360,47 +4460,49 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2">
-        <v>4</v>
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3c</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part4-lead-entry</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part4-lead-entry --test-level RunSpecifiedTests --tests LeadPhoneEntryHandlerTest --tests LeadTriggerTest --tests LeadTriggerHandlerTest</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E10" t="inlineStr" s="6">
@@ -3411,31 +4513,56 @@
     </row>
     <row r="11">
       <c r="A11" s="2">
+        <v>5</v>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2">
         <v>6</v>
       </c>
-      <c r="B11" t="inlineStr" s="2">
+      <c r="B12" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr" s="2">
+      <c r="C12" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr" s="2">
+      <c r="D12" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr" s="6">
+      <c r="E12" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E11"/>
+  <autoFilter ref="A4:E12"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -4088,7 +5215,7 @@
       </c>
       <c r="D8" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="E8" s="2">
@@ -8096,7 +9223,7 @@
       </c>
       <c r="I64" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J64" t="inlineStr" s="2">
@@ -8156,7 +9283,7 @@
       </c>
       <c r="I65" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J65" t="inlineStr" s="2">
@@ -8216,7 +9343,7 @@
       </c>
       <c r="I66" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J66" t="inlineStr" s="2">
@@ -8276,7 +9403,7 @@
       </c>
       <c r="I67" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J67" t="inlineStr" s="2">
@@ -8336,7 +9463,7 @@
       </c>
       <c r="I68" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J68" t="inlineStr" s="2">
@@ -8396,7 +9523,7 @@
       </c>
       <c r="I69" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr" s="2">
@@ -10056,7 +11183,7 @@
       </c>
       <c r="H11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I11" t="inlineStr" s="2">
@@ -10064,9 +11191,9 @@
           <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J11" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="K11" t="inlineStr" s="2">
@@ -10116,7 +11243,7 @@
       </c>
       <c r="H12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I12" t="inlineStr" s="2">
@@ -10124,9 +11251,9 @@
           <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J12" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="K12" t="inlineStr" s="2">
@@ -10176,7 +11303,7 @@
       </c>
       <c r="H13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I13" t="inlineStr" s="2">
@@ -10184,9 +11311,9 @@
           <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J13" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="K13" t="inlineStr" s="2">
@@ -22416,12 +23543,12 @@
     <row r="14">
       <c r="A14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
+          <t xml:space="preserve">LeadPhoneEntryHandlerTest (+ LeadTriggerTest, LeadTriggerHandlerTest)</t>
         </is>
       </c>
       <c r="B14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadPhoneEntryHandler</t>
+          <t xml:space="preserve">LeadPhoneEntryHandler, LeadTrigger</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="2">
@@ -22429,19 +23556,17 @@
           <t xml:space="preserve">Part 4</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
+      <c r="D14" s="2">
+        <v>11</v>
       </c>
       <c r="E14" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">target &gt; 85%</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="F14" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
deploy: v1.4.0 to sandbox; tracking files updated
- Code 0Afft000000Lc77CAC: 7/7, 20 tests passed (incl. existing
  LeadTriggerTest, LeadTriggerHandlerTest); LeadPhoneEntryHandler 100%
- Pilot 0Afft000000LcALCA0: POC profile entry fields, POC page entry field
- Observed: Salesforce gave read-only on the new entry fields to 22 existing
  profiles (harmless, left as is; reviewed at Part 11)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -3073,9 +3073,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J53" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J53" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K53" t="inlineStr" s="6">
@@ -3128,9 +3128,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J54" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J54" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K54" t="inlineStr" s="6">
@@ -3183,9 +3183,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J55" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J55" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K55" t="inlineStr" s="6">
@@ -3238,9 +3238,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J56" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J56" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K56" t="inlineStr" s="6">
@@ -3293,9 +3293,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J57" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J57" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K57" t="inlineStr" s="6">
@@ -3348,9 +3348,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J58" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J58" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K58" t="inlineStr" s="6">
@@ -3403,9 +3403,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J59" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J59" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K59" t="inlineStr" s="6">
@@ -3458,9 +3458,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J60" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J60" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K60" t="inlineStr" s="6">
@@ -3513,9 +3513,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J61" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J61" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K61" t="inlineStr" s="6">
@@ -3568,9 +3568,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J62" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J62" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K62" t="inlineStr" s="6">
@@ -3623,9 +3623,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J63" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J63" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K63" t="inlineStr" s="6">
@@ -3678,9 +3678,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J64" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J64" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K64" t="inlineStr" s="6">
@@ -3733,9 +3733,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J65" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J65" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K65" t="inlineStr" s="6">
@@ -3788,9 +3788,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J66" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J66" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K66" t="inlineStr" s="6">
@@ -3843,9 +3843,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J67" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J67" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K67" t="inlineStr" s="6">
@@ -3898,9 +3898,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J68" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J68" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K68" t="inlineStr" s="6">
@@ -3953,9 +3953,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J69" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J69" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K69" t="inlineStr" s="6">
@@ -4008,9 +4008,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J70" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J70" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K70" t="inlineStr" s="6">
@@ -4063,9 +4063,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J71" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J71" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K71" t="inlineStr" s="6">
@@ -4118,9 +4118,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J72" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J72" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K72" t="inlineStr" s="6">
@@ -5213,9 +5213,9 @@
           <t xml:space="preserve">Lead creation with hidden numbers</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="D8" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="E8" s="2">
@@ -9221,14 +9221,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I64" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I64" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J64" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K64" t="inlineStr" s="2">
@@ -9281,14 +9281,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I65" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I65" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J65" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K65" t="inlineStr" s="2">
@@ -9341,14 +9341,14 @@
           <t xml:space="preserve">LeadPhoneEntryHandlerTest</t>
         </is>
       </c>
-      <c r="I66" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I66" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J66" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K66" t="inlineStr" s="2">
@@ -9401,14 +9401,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I67" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I67" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J67" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K67" t="inlineStr" s="2">
@@ -9461,14 +9461,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I68" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I68" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J68" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LcALCA0</t>
         </is>
       </c>
       <c r="K68" t="inlineStr" s="2">
@@ -9521,14 +9521,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I69" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I69" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J69" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LcALCA0</t>
         </is>
       </c>
       <c r="K69" t="inlineStr" s="2">
@@ -11191,9 +11191,9 @@
           <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="J11" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K11" t="inlineStr" s="2">
@@ -11251,9 +11251,9 @@
           <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="J12" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K12" t="inlineStr" s="2">
@@ -11311,9 +11311,9 @@
           <t xml:space="preserve">backup/v1.4.0-pre-change</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="J13" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lc77CAC</t>
         </is>
       </c>
       <c r="K13" t="inlineStr" s="2">
@@ -23557,16 +23557,16 @@
         </is>
       </c>
       <c r="D14" s="2">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="E14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">target &gt; 85%</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+          <t xml:space="preserve">Handler 100% Â· LeadTrigger 80.1%</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Part 5a plan in the register (calling screens)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -14,13 +14,14 @@
     <sheet name="Release Bundle" sheetId="10" r:id="rId10"/>
     <sheet name="Release Steps" sheetId="11" r:id="rId11"/>
     <sheet name="Part 4 Plan" sheetId="12" r:id="rId12"/>
+    <sheet name="Part 5a Plan" sheetId="13" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$146</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
@@ -28,6 +29,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -5025,6 +5027,331 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="40" customWidth="1"/>
+    <col min="4" max="4" width="80" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 5a (v1.5.0) - Calling screens</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; originals in backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService (+ PhoneDisplayServiceTest)</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">isMaskedUser(): true when the user cannot read Lead.Phone__c. maskForDisplay(): "+91 9876543221" -&gt; "+91 98XXXXXX21". resolve(recordId, maskedValue, candidates): finds the real number on the server (with sharing) and writes an audit row.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Same masking rule on every screen</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Field (formula)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lead.Phone_Masked__c</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LEFT 2 + X + RIGHT 2 of Phone__c</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked number on the call panels</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Updated (ours)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">+ logAccess(): one audit row per MakeCall / G-Talk dial (deferred when a callout follows)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Every masked call is audited</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MakeCallController</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">readContacts: masked list for masked users (Lead + Related Source numbers). callCustomer: if the number contains X, find the real one on the server, then call MCube exactly as today.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Current users: no change. Masked users: masked list, call still placed.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low-medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">OfflineCallAppAPI</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">getLeadPhone / getOppPhone: masked for masked users. triggerCall: if the number contains X, find the real one on the server before the G-Talk callout.</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Same</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low-medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel, CallPanel_Outbound</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Show Phone_Masked__c instead of the blank Phone__c for masked users (detected on load).</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked users see 98XXXXXX21 instead of an empty line</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura / LWC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MakeCall, utilityCallComponent, offlineCallQuickActionCmp</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">They display what Apex returns and send it back; Apex now handles masked values.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Note</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LWC</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">offlineCallQuickActionCmp</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing issue found (not changed): treats the getLeadPhone result (a map) as a text number and shows a debug alert.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Report to the owner of this component</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F12"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
@@ -9558,32 +9885,32 @@
       </c>
       <c r="D70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Masked__c</t>
+          <t xml:space="preserve">PhoneDisplayService</t>
         </is>
       </c>
       <c r="F70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked primary for layouts / list views / reports</t>
+          <t xml:space="preserve">5a: one rule for all screens - is this user masked? masks numbers for display; resolves a masked number back to the real one (with sharing, audited)</t>
         </is>
       </c>
       <c r="H70" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I70" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J70" t="inlineStr" s="2">
@@ -9618,22 +9945,22 @@
       </c>
       <c r="D71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="F71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G71" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked secondary</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H71" t="inlineStr" s="2">
@@ -9641,9 +9968,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I71" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I71" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J71" t="inlineStr" s="2">
@@ -9678,32 +10005,32 @@
       </c>
       <c r="D72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_To_Masked__c</t>
+          <t xml:space="preserve">MaskedDialService</t>
         </is>
       </c>
       <c r="F72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call_Detail__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked call number</t>
+          <t xml:space="preserve">5a: + logAccess (audit rows for MakeCall / G-Talk, deferred when a callout follows)</t>
         </is>
       </c>
       <c r="H72" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I72" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J72" t="inlineStr" s="2">
@@ -9728,42 +10055,42 @@
       </c>
       <c r="B73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">Phone_Masked__c</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal for TL / Head / Admin: reason, 30 s, audit</t>
+          <t xml:space="preserve">5a: Formula: masked primary (call panels; later list views / reports)</t>
         </is>
       </c>
       <c r="H73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
-        </is>
-      </c>
-      <c r="I73" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J73" t="inlineStr" s="2">
@@ -9788,32 +10115,32 @@
       </c>
       <c r="B74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">Secondary_Phone_Masked__c</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Formula: masked secondary</t>
         </is>
       </c>
       <c r="H74" t="inlineStr" s="2">
@@ -9848,12 +10175,12 @@
       </c>
       <c r="B75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="2">
@@ -9863,17 +10190,17 @@
       </c>
       <c r="E75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Call_To_Masked__c</t>
         </is>
       </c>
       <c r="F75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve">Call_Detail__c</t>
         </is>
       </c>
       <c r="G75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
+          <t xml:space="preserve">Formula: masked call number</t>
         </is>
       </c>
       <c r="H75" t="inlineStr" s="2">
@@ -9918,12 +10245,12 @@
       </c>
       <c r="D76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F76" t="inlineStr" s="2">
@@ -9933,12 +10260,12 @@
       </c>
       <c r="G76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Who may reveal</t>
+          <t xml:space="preserve">Reveal for TL / Head / Admin: reason, 30 s, audit</t>
         </is>
       </c>
       <c r="H76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="I76" t="inlineStr" s="6">
@@ -9978,12 +10305,12 @@
       </c>
       <c r="D77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F77" t="inlineStr" s="2">
@@ -9993,7 +10320,7 @@
       </c>
       <c r="G77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Grants Reveal_Phone_Number to TL / Head / Admin</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H77" t="inlineStr" s="2">
@@ -10038,27 +10365,27 @@
       </c>
       <c r="D78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Nightly delete of audit rows older than 1 year (batch + schedulable)</t>
+          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
         </is>
       </c>
       <c r="H78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I78" t="inlineStr" s="6">
@@ -10078,7 +10405,7 @@
       </c>
       <c r="L78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -10098,12 +10425,12 @@
       </c>
       <c r="D79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F79" t="inlineStr" s="2">
@@ -10113,7 +10440,7 @@
       </c>
       <c r="G79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Who may reveal</t>
         </is>
       </c>
       <c r="H79" t="inlineStr" s="2">
@@ -10158,12 +10485,12 @@
       </c>
       <c r="D80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -10173,7 +10500,7 @@
       </c>
       <c r="G80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add Reveal button + reason picker</t>
+          <t xml:space="preserve">Grants Reveal_Phone_Number to TL / Head / Admin</t>
         </is>
       </c>
       <c r="H80" t="inlineStr" s="2">
@@ -10208,12 +10535,12 @@
       </c>
       <c r="B81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D81" t="inlineStr" s="2">
@@ -10223,7 +10550,7 @@
       </c>
       <c r="E81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F81" t="inlineStr" s="2">
@@ -10233,12 +10560,12 @@
       </c>
       <c r="G81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masks numbers typed in free text on save</t>
+          <t xml:space="preserve">Nightly delete of audit rows older than 1 year (batch + schedulable)</t>
         </is>
       </c>
       <c r="H81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="I81" t="inlineStr" s="6">
@@ -10258,7 +10585,7 @@
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -10268,12 +10595,12 @@
       </c>
       <c r="B82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D82" t="inlineStr" s="2">
@@ -10283,7 +10610,7 @@
       </c>
       <c r="E82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F82" t="inlineStr" s="2">
@@ -10328,37 +10655,37 @@
       </c>
       <c r="B83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masks numbers in Chatter posts</t>
+          <t xml:space="preserve">Add Reveal button + reason picker</t>
         </is>
       </c>
       <c r="H83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="I83" t="inlineStr" s="6">
@@ -10388,22 +10715,22 @@
       </c>
       <c r="B84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
@@ -10413,17 +10740,17 @@
       </c>
       <c r="G84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Search a number, masked result, audited</t>
+          <t xml:space="preserve">Masks numbers typed in free text on save</t>
         </is>
       </c>
       <c r="H84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
-        </is>
-      </c>
-      <c r="I84" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J84" t="inlineStr" s="2">
@@ -10433,12 +10760,12 @@
       </c>
       <c r="K84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -10448,22 +10775,22 @@
       </c>
       <c r="B85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
@@ -10473,17 +10800,17 @@
       </c>
       <c r="G85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server side of findByNumber</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="H85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
-        </is>
-      </c>
-      <c r="I85" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J85" t="inlineStr" s="2">
@@ -10493,7 +10820,7 @@
       </c>
       <c r="K85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L85" t="inlineStr" s="2">
@@ -10508,42 +10835,42 @@
       </c>
       <c r="B86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masks numbers in Chatter posts</t>
         </is>
       </c>
       <c r="H86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I86" t="inlineStr" s="7">
-        <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
         </is>
       </c>
       <c r="J86" t="inlineStr" s="2">
@@ -10553,7 +10880,7 @@
       </c>
       <c r="K86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="L86" t="inlineStr" s="2">
@@ -10568,22 +10895,22 @@
       </c>
       <c r="B87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
@@ -10593,17 +10920,17 @@
       </c>
       <c r="G87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Full phone-field access for integration users</t>
+          <t xml:space="preserve">Search a number, masked result, audited</t>
         </is>
       </c>
       <c r="H87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I87" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">Jest</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="J87" t="inlineStr" s="2">
@@ -10613,12 +10940,12 @@
       </c>
       <c r="K87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="L87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -10628,62 +10955,242 @@
       </c>
       <c r="B88" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 8</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.8.0</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberController</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Server side of findByNumber</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2">
+        <v>85</v>
+      </c>
+      <c r="B89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 8</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.8.0</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr" s="7">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conditional</t>
+        </is>
+      </c>
+      <c r="L89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2">
+        <v>86</v>
+      </c>
+      <c r="B90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v2.0.0</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Full phone-field access for integration users</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Planned</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign to integration users</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2">
+        <v>87</v>
+      </c>
+      <c r="B91" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Security fix</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr" s="2">
+      <c r="C91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">optional</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr" s="2">
+      <c r="D91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr" s="2">
+      <c r="E91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
-      <c r="F88" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr" s="2">
+      <c r="F91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">MCube endpoint + key over HTTPS instead of hard-coded token / http</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="I88" t="inlineStr" s="6">
+      <c r="H91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Planned</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="K88" t="inlineStr" s="2">
+      <c r="J91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr" s="2">
+      <c r="L91" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L88"/>
+  <autoFilter ref="A4:L91"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -11533,7 +12040,7 @@
       </c>
       <c r="F17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers on screen</t>
+          <t xml:space="preserve">5a: NO CHANGE needed - shows what readContacts returns and sends it back</t>
         </is>
       </c>
       <c r="G17" t="inlineStr" s="2">
@@ -11593,7 +12100,7 @@
       </c>
       <c r="F18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values; number resolved server-side</t>
+          <t xml:space="preserve">5a: readContacts returns masked for masked users; callCustomer resolves a masked number on the server</t>
         </is>
       </c>
       <c r="G18" t="inlineStr" s="2">
@@ -11653,7 +12160,7 @@
       </c>
       <c r="F19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve">5a: NO CHANGE needed - sends the number back to triggerCall, resolved on the server</t>
         </is>
       </c>
       <c r="G19" t="inlineStr" s="2">
@@ -11713,7 +12220,7 @@
       </c>
       <c r="F20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve">5a: NO CHANGE needed (same as utilityCallComponent)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr" s="2">
@@ -11773,7 +12280,7 @@
       </c>
       <c r="F21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server-side number lookup</t>
+          <t xml:space="preserve">5a: getLeadPhone / getOppPhone masked for masked users; triggerCall resolves a masked number on the server</t>
         </is>
       </c>
       <c r="G21" t="inlineStr" s="2">
@@ -11833,7 +12340,7 @@
       </c>
       <c r="F22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
         </is>
       </c>
       <c r="G22" t="inlineStr" s="2">
@@ -11893,7 +12400,7 @@
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
@@ -18928,7 +19435,7 @@
       </c>
       <c r="L83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return masked values; number resolved server-side</t>
+          <t xml:space="preserve">5a: readContacts returns masked for masked users; callCustomer resolves a masked number on the server</t>
         </is>
       </c>
     </row>
@@ -18948,12 +19455,12 @@
       </c>
       <c r="D84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">MaskedDialService</t>
         </is>
       </c>
       <c r="F84" t="inlineStr" s="2">
@@ -18963,7 +19470,7 @@
       </c>
       <c r="G84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H84" t="inlineStr" s="2">
@@ -18973,7 +19480,7 @@
       </c>
       <c r="I84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">MaskedDialServiceTest</t>
         </is>
       </c>
       <c r="J84" t="inlineStr" s="2">
@@ -18988,7 +19495,7 @@
       </c>
       <c r="L84" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask numbers before writing log__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -19013,7 +19520,7 @@
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">OfflineCallAppAPI</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
@@ -19048,7 +19555,7 @@
       </c>
       <c r="L85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Server-side number lookup</t>
+          <t xml:space="preserve">Mask numbers before writing log__c</t>
         </is>
       </c>
     </row>
@@ -19073,7 +19580,7 @@
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updateContactDetails</t>
+          <t xml:space="preserve">OfflineCallAppAPI</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
@@ -19108,7 +19615,7 @@
       </c>
       <c r="L86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Same</t>
+          <t xml:space="preserve">5a: getLeadPhone / getOppPhone masked for masked users; triggerCall resolves a masked number on the server</t>
         </is>
       </c>
     </row>
@@ -19128,12 +19635,12 @@
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">PhoneDisplayService</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
@@ -19143,7 +19650,7 @@
       </c>
       <c r="G87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H87" t="inlineStr" s="2">
@@ -19153,7 +19660,7 @@
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="J87" t="inlineStr" s="2">
@@ -19168,7 +19675,7 @@
       </c>
       <c r="L87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -19188,12 +19695,12 @@
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">updateContactDetails</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
@@ -19228,7 +19735,7 @@
       </c>
       <c r="L88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show masked field</t>
+          <t xml:space="preserve">Same</t>
         </is>
       </c>
     </row>
@@ -19248,12 +19755,12 @@
       </c>
       <c r="D89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeCmp</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
@@ -19263,7 +19770,7 @@
       </c>
       <c r="G89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H89" t="inlineStr" s="2">
@@ -19288,7 +19795,7 @@
       </c>
       <c r="L89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -19313,7 +19820,7 @@
       </c>
       <c r="E90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MakeCall</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
@@ -19348,7 +19855,7 @@
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers on screen</t>
+          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
         </is>
       </c>
     </row>
@@ -19373,7 +19880,7 @@
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeLightningPage</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -19408,7 +19915,7 @@
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show Call_To__c masked</t>
+          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
         </is>
       </c>
     </row>
@@ -19433,7 +19940,7 @@
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">LeadMergeCmp</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
@@ -19468,7 +19975,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Masked numbers</t>
         </is>
       </c>
     </row>
@@ -19488,12 +19995,12 @@
       </c>
       <c r="D93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">MakeCall</t>
         </is>
       </c>
       <c r="F93" t="inlineStr" s="2">
@@ -19528,7 +20035,7 @@
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">5a: NO CHANGE needed - shows what readContacts returns and sends it back</t>
         </is>
       </c>
     </row>
@@ -19548,12 +20055,12 @@
       </c>
       <c r="D94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">mCubeLightningPage</t>
         </is>
       </c>
       <c r="F94" t="inlineStr" s="2">
@@ -19588,7 +20095,7 @@
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Show Call_To__c masked</t>
         </is>
       </c>
     </row>
@@ -19608,12 +20115,12 @@
       </c>
       <c r="D95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
@@ -19648,7 +20155,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -19673,7 +20180,7 @@
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">offlineCallQuickActionCmp</t>
+          <t xml:space="preserve">leadBulkPush</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -19708,7 +20215,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -19733,7 +20240,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">utilityCallComponent</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -19768,7 +20275,7 @@
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">G-Talk: send recordId only</t>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -19778,32 +20285,32 @@
       </c>
       <c r="B98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">leadYotelPush</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H98" t="inlineStr" s="2">
@@ -19828,7 +20335,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -19838,22 +20345,22 @@
       </c>
       <c r="B99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">offlineCallQuickActionCmp</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -19863,7 +20370,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -19888,7 +20395,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">5a: NO CHANGE needed (same as utilityCallComponent)</t>
         </is>
       </c>
     </row>
@@ -19898,22 +20405,22 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">utilityCallComponent</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
@@ -19923,7 +20430,7 @@
       </c>
       <c r="G100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H100" t="inlineStr" s="2">
@@ -19933,7 +20440,7 @@
       </c>
       <c r="I100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J100" t="inlineStr" s="2">
@@ -19948,7 +20455,7 @@
       </c>
       <c r="L100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve">5a: NO CHANGE needed - sends the number back to triggerCall, resolved on the server</t>
         </is>
       </c>
     </row>
@@ -19968,17 +20475,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -19993,7 +20500,7 @@
       </c>
       <c r="I101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J101" t="inlineStr" s="2">
@@ -20028,12 +20535,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -20088,12 +20595,12 @@
       </c>
       <c r="D103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -20113,7 +20620,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -20128,7 +20635,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -20148,12 +20655,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -20173,7 +20680,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -20208,12 +20715,12 @@
       </c>
       <c r="D105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -20258,22 +20765,22 @@
       </c>
       <c r="B106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -20293,7 +20800,7 @@
       </c>
       <c r="I106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J106" t="inlineStr" s="2">
@@ -20308,7 +20815,7 @@
       </c>
       <c r="L106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20318,22 +20825,22 @@
       </c>
       <c r="B107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -20378,22 +20885,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -20403,7 +20910,7 @@
       </c>
       <c r="G108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H108" t="inlineStr" s="2">
@@ -20428,7 +20935,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20448,17 +20955,17 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G109" t="inlineStr" s="2">
@@ -20488,7 +20995,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -20508,12 +21015,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -20523,7 +21030,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -20548,7 +21055,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20573,7 +21080,7 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
@@ -20608,7 +21115,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -20618,27 +21125,27 @@
       </c>
       <c r="B112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
@@ -20653,12 +21160,12 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K112" t="inlineStr" s="6">
@@ -20678,22 +21185,22 @@
       </c>
       <c r="B113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -20703,7 +21210,7 @@
       </c>
       <c r="G113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H113" t="inlineStr" s="2">
@@ -20718,7 +21225,7 @@
       </c>
       <c r="J113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K113" t="inlineStr" s="6">
@@ -20728,7 +21235,7 @@
       </c>
       <c r="L113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -20738,22 +21245,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -20763,7 +21270,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -20773,12 +21280,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -20788,7 +21295,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -20808,12 +21315,12 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -20823,7 +21330,7 @@
       </c>
       <c r="G115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H115" t="inlineStr" s="2">
@@ -20833,7 +21340,7 @@
       </c>
       <c r="I115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -20848,7 +21355,7 @@
       </c>
       <c r="L115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20858,22 +21365,22 @@
       </c>
       <c r="B116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -20883,7 +21390,7 @@
       </c>
       <c r="G116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H116" t="inlineStr" s="2">
@@ -20908,7 +21415,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20918,22 +21425,22 @@
       </c>
       <c r="B117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -20943,7 +21450,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -20953,7 +21460,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -20968,7 +21475,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -20978,22 +21485,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -21028,7 +21535,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -21048,12 +21555,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -21088,7 +21595,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -21108,12 +21615,12 @@
       </c>
       <c r="D120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -21148,7 +21655,7 @@
       </c>
       <c r="L120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -21168,12 +21675,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -21233,7 +21740,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -21268,7 +21775,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -21293,7 +21800,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -21328,7 +21835,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -21348,12 +21855,12 @@
       </c>
       <c r="D124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -21388,7 +21895,7 @@
       </c>
       <c r="L124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -21398,22 +21905,22 @@
       </c>
       <c r="B125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -21438,7 +21945,7 @@
       </c>
       <c r="J125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K125" t="inlineStr" s="6">
@@ -21448,7 +21955,7 @@
       </c>
       <c r="L125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -21458,22 +21965,22 @@
       </c>
       <c r="B126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -21498,7 +22005,7 @@
       </c>
       <c r="J126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K126" t="inlineStr" s="6">
@@ -21508,7 +22015,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -21518,22 +22025,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -21558,7 +22065,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -21568,7 +22075,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -21593,7 +22100,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -21653,7 +22160,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -21713,7 +22220,7 @@
       </c>
       <c r="E130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F130" t="inlineStr" s="2">
@@ -21773,7 +22280,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -21828,12 +22335,12 @@
       </c>
       <c r="D132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F132" t="inlineStr" s="2">
@@ -21843,7 +22350,7 @@
       </c>
       <c r="G132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H132" t="inlineStr" s="2">
@@ -21868,7 +22375,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -21888,12 +22395,12 @@
       </c>
       <c r="D133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -21908,7 +22415,7 @@
       </c>
       <c r="H133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I133" t="inlineStr" s="2">
@@ -21928,7 +22435,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -21948,12 +22455,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -21968,7 +22475,7 @@
       </c>
       <c r="H134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I134" t="inlineStr" s="2">
@@ -21978,7 +22485,7 @@
       </c>
       <c r="J134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K134" t="inlineStr" s="6">
@@ -21988,7 +22495,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -21998,22 +22505,22 @@
       </c>
       <c r="B135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -22038,7 +22545,7 @@
       </c>
       <c r="J135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K135" t="inlineStr" s="6">
@@ -22048,7 +22555,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -22058,22 +22565,22 @@
       </c>
       <c r="B136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -22088,7 +22595,7 @@
       </c>
       <c r="H136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I136" t="inlineStr" s="2">
@@ -22098,7 +22605,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -22108,7 +22615,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -22118,22 +22625,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -22148,7 +22655,7 @@
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -22158,7 +22665,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -22168,7 +22675,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -22188,12 +22695,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -22203,7 +22710,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -22228,7 +22735,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -22238,22 +22745,22 @@
       </c>
       <c r="B139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -22263,12 +22770,12 @@
       </c>
       <c r="G139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I139" t="inlineStr" s="2">
@@ -22278,7 +22785,7 @@
       </c>
       <c r="J139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K139" t="inlineStr" s="6">
@@ -22288,7 +22795,7 @@
       </c>
       <c r="L139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -22298,22 +22805,22 @@
       </c>
       <c r="B140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -22323,12 +22830,12 @@
       </c>
       <c r="G140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I140" t="inlineStr" s="2">
@@ -22338,7 +22845,7 @@
       </c>
       <c r="J140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K140" t="inlineStr" s="6">
@@ -22348,7 +22855,7 @@
       </c>
       <c r="L140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -22358,22 +22865,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -22383,12 +22890,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -22398,7 +22905,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -22408,7 +22915,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -22418,7 +22925,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -22433,7 +22940,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -22468,7 +22975,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -22478,7 +22985,7 @@
       </c>
       <c r="B143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C143" t="inlineStr" s="2">
@@ -22493,7 +23000,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -22518,7 +23025,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -22528,7 +23035,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -22538,7 +23045,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -22553,7 +23060,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -22578,7 +23085,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -22588,7 +23095,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -22598,7 +23105,7 @@
       </c>
       <c r="B145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C145" t="inlineStr" s="2">
@@ -22613,7 +23120,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -22648,7 +23155,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -22658,62 +23165,242 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M10</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K146" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2">
+        <v>143</v>
+      </c>
+      <c r="B147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K147" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2">
+        <v>144</v>
+      </c>
+      <c r="B148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2">
+        <v>145</v>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C146" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr" s="2">
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E146" t="inlineStr" s="2">
+      <c r="E149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F146" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G146" t="inlineStr" s="2">
+      <c r="F149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H146" t="inlineStr" s="2">
+      <c r="H149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I146" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J146" t="inlineStr" s="2">
+      <c r="I149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="K146" t="inlineStr" s="6">
+      <c r="K149" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L146" t="inlineStr" s="2">
+      <c r="L149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L146"/>
+  <autoFilter ref="A4:L149"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -23930,32 +24617,32 @@
     <row r="9">
       <c r="A9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Before Part 5</t>
+          <t xml:space="preserve">Part 5a pre-change backup</t>
         </is>
       </c>
       <c r="B9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Re-retrieve Part 5 components and compare with baseline</t>
+          <t xml:space="preserve">MakeCall + MakeCallController (+Test), OfflineCallAppAPI (+Test), utilityCallComponent, offlineCallQuickActionCmp, CallPanel, CallPanel_Outbound - identical to baseline</t>
         </is>
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">backup/v1.5.0-pre-change</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change (with SHA256SUMS)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">2026-10-06</t>
         </is>
       </c>
       <c r="E9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">3c0330b</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Backed up</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v1.5.0 Part 5a calling screens masked (built locally, not deployed)
New: PhoneDisplayService (+test), PhoneMaskingCallScreensTest, Lead.Phone_Masked__c.
Ours updated: MaskedDialService.logAccess, POC profile (Phone_Masked__c read).
Existing (approved, originals in backup/v1.5.0-part5a-pre-change):
- MakeCallController: masked list for masked users; masked selection resolved
  on the server; original bodies kept as collectPhones / placeMcubeCall
- OfflineCallAppAPI: masked map for masked users; triggerCall resolves masked
- CallPanel, CallPanel_Outbound: Phone_Masked__c for masked users
No change: MakeCall, utilityCallComponent, offlineCallQuickActionCmp.
Manifests, release bundle part5a-calling, changelog, roadmap, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -19,15 +19,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$91</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$93</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
   </definedNames>
@@ -323,7 +323,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-4)</t>
+          <t>Production Release Bundle - built components (Parts 1-5a)</t>
         </is>
       </c>
     </row>
@@ -427,7 +427,7 @@
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fa00d87d27a2</t>
+          <t xml:space="preserve">a8c2c5dc228b</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="2">
@@ -4137,47 +4137,47 @@
       </c>
       <c r="B73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5a-calling</t>
         </is>
       </c>
       <c r="C73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
         </is>
       </c>
       <c r="E73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">MakeCallController</t>
         </is>
       </c>
       <c r="G73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/MakeCallController.cls</t>
         </is>
       </c>
       <c r="H73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
+          <t xml:space="preserve">2f6c04583ce0</t>
         </is>
       </c>
       <c r="I73" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J73" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K73" t="inlineStr" s="6">
@@ -4192,47 +4192,47 @@
       </c>
       <c r="B74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5a-calling</t>
         </is>
       </c>
       <c r="C74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">MakeCallController</t>
         </is>
       </c>
       <c r="G74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/MakeCallController.cls-meta.xml</t>
         </is>
       </c>
       <c r="H74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">8ec13a9efa48</t>
         </is>
       </c>
       <c r="I74" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J74" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K74" t="inlineStr" s="6">
@@ -4247,57 +4247,1377 @@
       </c>
       <c r="B75" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/MaskedDialService.cls</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">a8c2c5dc228b</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2">
+        <v>5</v>
+      </c>
+      <c r="B76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/MaskedDialService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2">
+        <v>5</v>
+      </c>
+      <c r="B77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">OfflineCallAppAPI</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/OfflineCallAppAPI.cls</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">962740bbee63</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2">
+        <v>5</v>
+      </c>
+      <c r="B78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">OfflineCallAppAPI</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/OfflineCallAppAPI.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">331f43ffe1e3</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2">
+        <v>5</v>
+      </c>
+      <c r="B79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/PhoneDisplayService.cls</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">fc8c29b6582e</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2">
+        <v>5</v>
+      </c>
+      <c r="B80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/PhoneDisplayService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2">
+        <v>5</v>
+      </c>
+      <c r="B81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/PhoneDisplayServiceTest.cls</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">36dd6f2c7618</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2">
+        <v>5</v>
+      </c>
+      <c r="B82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/PhoneDisplayServiceTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2">
+        <v>5</v>
+      </c>
+      <c r="B83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/PhoneMaskingCallScreensTest.cls</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ffa49b5c449a</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K83" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2">
+        <v>5</v>
+      </c>
+      <c r="B84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/classes/PhoneMaskingCallScreensTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2">
+        <v>5</v>
+      </c>
+      <c r="B85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanel.cmp</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5fdcd3a8958e</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K85" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2">
+        <v>5</v>
+      </c>
+      <c r="B86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanel.cmp-meta.xml</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">8beda1373bed</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K86" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2">
+        <v>5</v>
+      </c>
+      <c r="B87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanel.css</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">429733ed222e</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2">
+        <v>5</v>
+      </c>
+      <c r="B88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanelController.js</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">092c7d1f9ea7</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2">
+        <v>5</v>
+      </c>
+      <c r="B89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanelHelper.js</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">811a8ae0c844</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2">
+        <v>5</v>
+      </c>
+      <c r="B90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel_Outbound</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_Outbound.cmp</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bd7a9b0a99fc</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2">
+        <v>5</v>
+      </c>
+      <c r="B91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel_Outbound</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_Outbound.cmp-meta.xml</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5341792d0d7b</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2">
+        <v>5</v>
+      </c>
+      <c r="B92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel_Outbound</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_Outbound.css</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">86f713c4d143</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2">
+        <v>5</v>
+      </c>
+      <c r="B93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel_Outbound</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_OutboundController.js</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">8ba4781bf267</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2">
+        <v>5</v>
+      </c>
+      <c r="B94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">CallPanel_Outbound</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_OutboundHelper.js</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">d55ea46cbdc6</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2">
+        <v>5</v>
+      </c>
+      <c r="B95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lead</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/objects/Lead.object</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">ec632285f7c0</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2">
+        <v>5</v>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5a-calling</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5a)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5a-calling/package.xml</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">4b8910c65821</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2">
+        <v>6</v>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr" s="2">
+      <c r="C97" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr" s="2">
+      <c r="D97" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr" s="2">
+      <c r="E97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2">
+        <v>6</v>
+      </c>
+      <c r="B98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2">
+        <v>6</v>
+      </c>
+      <c r="B99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr" s="2">
+      <c r="F99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr" s="2">
+      <c r="G99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H75" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">86d290d2bafe</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr" s="2">
+      <c r="H99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">df1ecd8c7bec</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr" s="4">
+      <c r="J99" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K75" t="inlineStr" s="6">
+      <c r="K99" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K75"/>
+  <autoFilter ref="A4:K99"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -4321,7 +5641,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-4)</t>
+          <t>Production Deploy Steps (Parts 1-5a)</t>
         </is>
       </c>
     </row>
@@ -4489,47 +5809,49 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2">
-        <v>4</v>
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3d</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part5a-calling</t>
         </is>
       </c>
       <c r="C10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5a-calling --test-level RunSpecifiedTests --tests PhoneDisplayServiceTest --tests PhoneMaskingCallScreensTest --tests MakeCallControllerTest --tests OfflineCallAppAPITest --tests MaskedDialServiceTest</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E11" t="inlineStr" s="6">
@@ -4540,31 +5862,56 @@
     </row>
     <row r="12">
       <c r="A12" s="2">
+        <v>5</v>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2">
         <v>6</v>
       </c>
-      <c r="B12" t="inlineStr" s="2">
+      <c r="B13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr" s="2">
+      <c r="C13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr" s="2">
+      <c r="D13" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr" s="6">
+      <c r="E13" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E12"/>
+  <autoFilter ref="A4:E13"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -5571,12 +6918,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">Mask leaking screens (5a built)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -9910,7 +11257,7 @@
       </c>
       <c r="I70" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="J70" t="inlineStr" s="2">
@@ -9970,7 +11317,7 @@
       </c>
       <c r="I71" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="J71" t="inlineStr" s="2">
@@ -10030,7 +11377,7 @@
       </c>
       <c r="I72" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="J72" t="inlineStr" s="2">
@@ -10090,7 +11437,7 @@
       </c>
       <c r="I73" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="J73" t="inlineStr" s="2">
@@ -11189,8 +12536,128 @@
         </is>
       </c>
     </row>
+    <row r="92">
+      <c r="A92" s="2">
+        <v>88</v>
+      </c>
+      <c r="B92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5a: masked paths of MakeCallController and OfflineCallAppAPI (callouts mocked)</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing test classes unchanged</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2">
+        <v>89</v>
+      </c>
+      <c r="B93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Profile (update of new)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5a: read access to Lead.Phone_Masked__c</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Pilot only (decide)</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L91"/>
+  <autoFilter ref="A4:L93"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -12050,22 +13517,22 @@
       </c>
       <c r="H17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5a)</t>
         </is>
       </c>
       <c r="K17" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L17" t="inlineStr" s="2">
@@ -12110,17 +13577,17 @@
       </c>
       <c r="H18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I18" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="K18" t="inlineStr" s="2">
@@ -12170,22 +13637,22 @@
       </c>
       <c r="H19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5a)</t>
         </is>
       </c>
       <c r="K19" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L19" t="inlineStr" s="2">
@@ -12230,22 +13697,22 @@
       </c>
       <c r="H20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5a)</t>
         </is>
       </c>
       <c r="K20" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L20" t="inlineStr" s="2">
@@ -12290,17 +13757,17 @@
       </c>
       <c r="H21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I21" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="K21" t="inlineStr" s="2">
@@ -12350,17 +13817,17 @@
       </c>
       <c r="H22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="K22" t="inlineStr" s="2">
@@ -12410,17 +13877,17 @@
       </c>
       <c r="H23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5a</t>
         </is>
       </c>
       <c r="K23" t="inlineStr" s="2">
@@ -19815,12 +21282,12 @@
       </c>
       <c r="D90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
@@ -19830,7 +21297,7 @@
       </c>
       <c r="G90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H90" t="inlineStr" s="2">
@@ -19855,7 +21322,7 @@
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
+          <t xml:space="preserve">Existing test classes unchanged</t>
         </is>
       </c>
     </row>
@@ -19880,7 +21347,7 @@
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -19940,7 +21407,7 @@
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeCmp</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
@@ -19975,7 +21442,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
         </is>
       </c>
     </row>
@@ -20000,7 +21467,7 @@
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MakeCall</t>
+          <t xml:space="preserve">LeadMergeCmp</t>
         </is>
       </c>
       <c r="F93" t="inlineStr" s="2">
@@ -20035,7 +21502,7 @@
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: NO CHANGE needed - shows what readContacts returns and sends it back</t>
+          <t xml:space="preserve">Masked numbers</t>
         </is>
       </c>
     </row>
@@ -20355,12 +21822,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">offlineCallQuickActionCmp</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -20370,7 +21837,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -20385,7 +21852,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -20395,7 +21862,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: NO CHANGE needed (same as utilityCallComponent)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20405,32 +21872,32 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">utilityCallComponent</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H100" t="inlineStr" s="2">
@@ -20455,7 +21922,7 @@
       </c>
       <c r="L100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: NO CHANGE needed - sends the number back to triggerCall, resolved on the server</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20475,17 +21942,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -20535,12 +22002,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -20560,7 +22027,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -20575,7 +22042,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -20600,7 +22067,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -20620,7 +22087,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -20635,7 +22102,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20655,12 +22122,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -20680,7 +22147,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -20720,7 +22187,7 @@
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -20775,12 +22242,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -20835,12 +22302,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -20885,22 +22352,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -20920,7 +22387,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -20935,7 +22402,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -20955,12 +22422,12 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
@@ -20980,7 +22447,7 @@
       </c>
       <c r="I109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J109" t="inlineStr" s="2">
@@ -20995,7 +22462,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -21015,12 +22482,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -21030,7 +22497,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -21055,7 +22522,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -21080,17 +22547,17 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -21100,7 +22567,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -21115,7 +22582,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -21135,22 +22602,22 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -21160,7 +22627,7 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
@@ -21175,7 +22642,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -21195,12 +22662,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -21245,22 +22712,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -21270,7 +22737,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -21280,12 +22747,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -21295,7 +22762,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -21315,12 +22782,12 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -21340,7 +22807,7 @@
       </c>
       <c r="I115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -21375,12 +22842,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -21400,7 +22867,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -21415,7 +22882,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -21440,7 +22907,7 @@
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -21450,7 +22917,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -21460,7 +22927,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -21475,7 +22942,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -21485,22 +22952,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -21535,7 +23002,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -21555,12 +23022,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -21595,7 +23062,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -21620,7 +23087,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -21675,12 +23142,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -21715,7 +23182,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -21740,7 +23207,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -21775,7 +23242,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -21800,7 +23267,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -21835,7 +23302,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -21860,7 +23327,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -21920,7 +23387,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -21975,12 +23442,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -22015,7 +23482,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -22025,22 +23492,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -22065,7 +23532,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -22075,7 +23542,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -22100,7 +23567,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -22160,7 +23627,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -22280,7 +23747,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -22375,7 +23842,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -22400,7 +23867,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -22435,7 +23902,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -22455,12 +23922,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -22470,7 +23937,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -22495,7 +23962,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -22515,12 +23982,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -22530,12 +23997,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -22555,7 +24022,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -22575,12 +24042,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -22605,7 +24072,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -22615,7 +24082,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -22625,22 +24092,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -22650,12 +24117,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -22665,7 +24132,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -22675,7 +24142,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -22695,12 +24162,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -22710,7 +24177,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -22735,7 +24202,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -22760,7 +24227,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -22820,7 +24287,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -22865,22 +24332,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Manual step</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -22890,12 +24357,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -22905,7 +24372,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -22915,7 +24382,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -22925,7 +24392,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -22940,7 +24407,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -22965,7 +24432,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -22975,7 +24442,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -23000,7 +24467,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -23025,7 +24492,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -23035,7 +24502,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -23045,7 +24512,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -23060,7 +24527,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -23085,7 +24552,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -23095,7 +24562,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -23120,7 +24587,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -23155,7 +24622,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -23165,7 +24632,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -23180,7 +24647,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -23215,7 +24682,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -23240,7 +24707,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M12</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -23275,7 +24742,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
         </is>
       </c>
     </row>
@@ -23285,7 +24752,7 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 13</t>
         </is>
       </c>
       <c r="C148" t="inlineStr" s="2">
@@ -23300,7 +24767,7 @@
       </c>
       <c r="E148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M13</t>
         </is>
       </c>
       <c r="F148" t="inlineStr" s="2">
@@ -23335,72 +24802,12 @@
       </c>
       <c r="L148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2">
-        <v>145</v>
-      </c>
-      <c r="B149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 13</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual step</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">M13</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L149"/>
+  <autoFilter ref="A4:L148"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
deploy: Part 5a to sandbox (call panels postponed); tracking updated
- Code 0Afft000000Lf3NCAS: 7/7, 45 tests passed (incl. existing
  MakeCallControllerTest, OfflineCallAppAPITest, MaskedDialServiceTest)
- Pilot 0Afft000000Lf4zCAC: POC profile reads Phone_Masked__c
- CallPanel / CallPanel_Outbound: Aura recordViewForm has no onload; both
  restored to the original locally, removed from the 5a manifest; new
  approach (LWC maskedPhoneField) pending approval
- Release bundle rebuilt; register, changelog, roadmap updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -26,7 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$89</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
@@ -4175,9 +4175,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J73" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J73" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K73" t="inlineStr" s="6">
@@ -4230,9 +4230,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J74" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K74" t="inlineStr" s="6">
@@ -4285,9 +4285,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J75" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J75" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K75" t="inlineStr" s="6">
@@ -4340,9 +4340,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J76" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J76" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K76" t="inlineStr" s="6">
@@ -4395,9 +4395,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J77" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J77" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K77" t="inlineStr" s="6">
@@ -4450,9 +4450,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J78" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J78" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K78" t="inlineStr" s="6">
@@ -4505,9 +4505,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J79" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J79" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K79" t="inlineStr" s="6">
@@ -4560,9 +4560,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J80" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J80" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K80" t="inlineStr" s="6">
@@ -4615,9 +4615,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J81" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J81" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K81" t="inlineStr" s="6">
@@ -4670,9 +4670,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J82" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J82" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K82" t="inlineStr" s="6">
@@ -4725,9 +4725,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J83" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J83" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K83" t="inlineStr" s="6">
@@ -4780,9 +4780,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J84" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J84" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K84" t="inlineStr" s="6">
@@ -4812,22 +4812,22 @@
       </c>
       <c r="E85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">Lead</t>
         </is>
       </c>
       <c r="G85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanel.cmp</t>
+          <t xml:space="preserve">release/prod/part5a-calling/objects/Lead.object</t>
         </is>
       </c>
       <c r="H85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5fdcd3a8958e</t>
+          <t xml:space="preserve">ec632285f7c0</t>
         </is>
       </c>
       <c r="I85" t="inlineStr" s="2">
@@ -4835,9 +4835,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J85" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J85" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K85" t="inlineStr" s="6">
@@ -4867,22 +4867,22 @@
       </c>
       <c r="E86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Manifest (package.xml)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">package.xml</t>
         </is>
       </c>
       <c r="G86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanel.cmp-meta.xml</t>
+          <t xml:space="preserve">release/prod/part5a-calling/package.xml</t>
         </is>
       </c>
       <c r="H86" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">8beda1373bed</t>
+          <t xml:space="preserve">3b1ffa635783</t>
         </is>
       </c>
       <c r="I86" t="inlineStr" s="2">
@@ -4890,9 +4890,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J86" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J86" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K86" t="inlineStr" s="6">
@@ -4903,51 +4903,51 @@
     </row>
     <row r="87">
       <c r="A87" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part5a-calling</t>
+          <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
       <c r="C87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
+          <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
         </is>
       </c>
       <c r="G87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanel.css</t>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
         </is>
       </c>
       <c r="H87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">429733ed222e</t>
+          <t xml:space="preserve">9354cdba5c3c</t>
         </is>
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
       <c r="K87" t="inlineStr" s="6">
@@ -4958,51 +4958,51 @@
     </row>
     <row r="88">
       <c r="A88" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part5a-calling</t>
+          <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
       <c r="C88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
+          <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Manifest (package.xml)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">package.xml</t>
         </is>
       </c>
       <c r="G88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanelController.js</t>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
         </is>
       </c>
       <c r="H88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">092c7d1f9ea7</t>
+          <t xml:space="preserve">b158c134f515</t>
         </is>
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
       <c r="K88" t="inlineStr" s="6">
@@ -5013,51 +5013,51 @@
     </row>
     <row r="89">
       <c r="A89" s="2">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part5a-calling</t>
+          <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
       <c r="C89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="D89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
+          <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="G89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel/CallPanelHelper.js</t>
+          <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
       <c r="H89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">811a8ae0c844</t>
+          <t xml:space="preserve">df1ecd8c7bec</t>
         </is>
       </c>
       <c r="I89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J89" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
       <c r="K89" t="inlineStr" s="6">
@@ -5066,558 +5066,8 @@
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="2">
-        <v>5</v>
-      </c>
-      <c r="B90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Aura Component</t>
-        </is>
-      </c>
-      <c r="F90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
-        </is>
-      </c>
-      <c r="G90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_Outbound.cmp</t>
-        </is>
-      </c>
-      <c r="H90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">bd7a9b0a99fc</t>
-        </is>
-      </c>
-      <c r="I90" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J90" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K90" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2">
-        <v>5</v>
-      </c>
-      <c r="B91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Aura Component</t>
-        </is>
-      </c>
-      <c r="F91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_Outbound.cmp-meta.xml</t>
-        </is>
-      </c>
-      <c r="H91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">5341792d0d7b</t>
-        </is>
-      </c>
-      <c r="I91" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J91" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K91" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" s="2">
-        <v>5</v>
-      </c>
-      <c r="B92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Aura Component</t>
-        </is>
-      </c>
-      <c r="F92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_Outbound.css</t>
-        </is>
-      </c>
-      <c r="H92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">86f713c4d143</t>
-        </is>
-      </c>
-      <c r="I92" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J92" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K92" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" s="2">
-        <v>5</v>
-      </c>
-      <c r="B93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Aura Component</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_OutboundController.js</t>
-        </is>
-      </c>
-      <c r="H93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">8ba4781bf267</t>
-        </is>
-      </c>
-      <c r="I93" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K93" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" s="2">
-        <v>5</v>
-      </c>
-      <c r="B94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Aura Component</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/aura/CallPanel_Outbound/CallPanel_OutboundHelper.js</t>
-        </is>
-      </c>
-      <c r="H94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">d55ea46cbdc6</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J94" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K94" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="2">
-        <v>5</v>
-      </c>
-      <c r="B95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Lead</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/objects/Lead.object</t>
-        </is>
-      </c>
-      <c r="H95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">ec632285f7c0</t>
-        </is>
-      </c>
-      <c r="I95" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J95" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K95" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="2">
-        <v>5</v>
-      </c>
-      <c r="B96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part5a-calling</t>
-        </is>
-      </c>
-      <c r="C96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 5</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.5.0 (5a)</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">package.xml</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part5a-calling/package.xml</t>
-        </is>
-      </c>
-      <c r="H96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">4b8910c65821</t>
-        </is>
-      </c>
-      <c r="I96" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production - everyone</t>
-        </is>
-      </c>
-      <c r="J96" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
-        </is>
-      </c>
-      <c r="K96" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="2">
-        <v>6</v>
-      </c>
-      <c r="B97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part2-pilot</t>
-        </is>
-      </c>
-      <c r="C97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 2</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.2.0</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Lightning Page</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
-        </is>
-      </c>
-      <c r="H97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
-        </is>
-      </c>
-      <c r="I97" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
-        </is>
-      </c>
-      <c r="K97" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2">
-        <v>6</v>
-      </c>
-      <c r="B98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part2-pilot</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 2</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.2.0</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">package.xml</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
-        </is>
-      </c>
-      <c r="H98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">b158c134f515</t>
-        </is>
-      </c>
-      <c r="I98" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
-        </is>
-      </c>
-      <c r="K98" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="2">
-        <v>6</v>
-      </c>
-      <c r="B99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">part2-pilot</t>
-        </is>
-      </c>
-      <c r="C99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 2</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">v1.2.0</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Profile</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">POC Masked Rep</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
-        </is>
-      </c>
-      <c r="H99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">df1ecd8c7bec</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J99" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
-        </is>
-      </c>
-      <c r="K99" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:K99"/>
+  <autoFilter ref="A4:K89"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -6918,12 +6368,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a built)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+          <t xml:space="preserve">Mask leaking screens (5a deployed, call panels pending)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) - 5a</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -11255,9 +10705,9 @@
           <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="I70" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="J70" t="inlineStr" s="2">
@@ -11315,9 +10765,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I71" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="I71" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="J71" t="inlineStr" s="2">
@@ -11375,9 +10825,9 @@
           <t xml:space="preserve">MaskedDialServiceTest</t>
         </is>
       </c>
-      <c r="I72" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="I72" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="J72" t="inlineStr" s="2">
@@ -11435,9 +10885,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I73" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="I73" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="J73" t="inlineStr" s="2">
@@ -12575,9 +12025,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I92" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="I92" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J92" t="inlineStr" s="2">
@@ -12635,9 +12085,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I93" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="I93" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J93" t="inlineStr" s="2">
@@ -13585,9 +13035,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="J18" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K18" t="inlineStr" s="2">
@@ -13765,9 +13215,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5a-pre-change</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+      <c r="J21" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lf3NCAS</t>
         </is>
       </c>
       <c r="K21" t="inlineStr" s="2">
@@ -13807,7 +13257,7 @@
       </c>
       <c r="F22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
       <c r="G22" t="inlineStr" s="2">
@@ -13817,7 +13267,7 @@
       </c>
       <c r="H22" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved 2026-10-06</t>
+          <t xml:space="preserve">New approach pending approval</t>
         </is>
       </c>
       <c r="I22" t="inlineStr" s="2">
@@ -13827,7 +13277,7 @@
       </c>
       <c r="J22" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="K22" t="inlineStr" s="2">
@@ -13867,7 +13317,7 @@
       </c>
       <c r="F23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
       <c r="G23" t="inlineStr" s="2">
@@ -13877,7 +13327,7 @@
       </c>
       <c r="H23" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Approved 2026-10-06</t>
+          <t xml:space="preserve">New approach pending approval</t>
         </is>
       </c>
       <c r="I23" t="inlineStr" s="2">
@@ -13887,7 +13337,7 @@
       </c>
       <c r="J23" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Built (Local) - 5a</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="K23" t="inlineStr" s="2">
@@ -21382,7 +20832,7 @@
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -21442,7 +20892,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5a: show Phone_Masked__c for masked users</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
backup + plan: Part 5b (call history and logs)
Backup of mCubeController (+2 tests), LeadHistoryandActivityController (+test),
mCubeLightningPage, LeadHistoryandActivityCmp (first backup) - read-only,
identical to baseline. Plan sheet added to the register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Release Steps" sheetId="11" r:id="rId11"/>
     <sheet name="Part 4 Plan" sheetId="12" r:id="rId12"/>
     <sheet name="Part 5a Plan" sheetId="13" r:id="rId13"/>
+    <sheet name="Part 5b Plan" sheetId="14" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
@@ -30,6 +31,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -6149,6 +6151,299 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="80" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 5b (v1.5.0) - Call history and logs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; originals in backup/v1.5.0-part5b-pre-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Field (formula)</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Call_Detail__c.Call_To_Masked__c</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked customer number of a call (first 2 + last 2)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked column for call list views / reports (used at go-live)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Tests the masked paths of callRecords, GetData and the log masking (callouts mocked)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mCubeController.callRecords</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">For masked users, mask Call_From__c / Call_To__c on the returned call list (in memory, never saved)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Call history list (mCubeLightningPage) shows 98XXXXXX21 for masked users; unchanged for others</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mCubeController.makeCall / makeCallZetta (log__c)</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Wrap the 3 Request__c and 2 Response__c values in PhoneMaskUtil.maskInText - numbers in the MCube logs are masked for everyone</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Admins reading log__c see masked numbers (by design); MCube calls unchanged</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadHistoryandActivityController.GetData</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">For masked users: mask OldValue / NewValue of phone-field history rows (Phone__c, Secondary_Phone__c are history-tracked) and callfrom / callto</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">History screen shows masked old / new numbers for masked users; unchanged for others</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mCubeLightningPage, LeadHistoryandActivityCmp</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">They display what Apex returns</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Later</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Free text</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Task Subject / Description in the history</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Numbers typed in notes are handled by Part 7 (free-text masking)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F11"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
@@ -10997,7 +11292,7 @@
       </c>
       <c r="G75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Formula: masked call number</t>
+          <t xml:space="preserve">5b: Formula: masked call number</t>
         </is>
       </c>
       <c r="H75" t="inlineStr" s="2">
@@ -11005,9 +11300,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I75" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I75" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="J75" t="inlineStr" s="2">
@@ -13377,7 +13672,7 @@
       </c>
       <c r="F24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show Call_To__c masked</t>
+          <t xml:space="preserve">5b: NO CHANGE - shows what callRecords returns</t>
         </is>
       </c>
       <c r="G24" t="inlineStr" s="2">
@@ -13437,7 +13732,7 @@
       </c>
       <c r="F25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return Call_To__c masked</t>
+          <t xml:space="preserve">5b: GetData masks phone history values and call numbers for masked users</t>
         </is>
       </c>
       <c r="G25" t="inlineStr" s="2">
@@ -13497,7 +13792,7 @@
       </c>
       <c r="F26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask numbers before writing log__c</t>
+          <t xml:space="preserve">5b: callRecords masked for masked users; log__c Request / Response masked for everyone</t>
         </is>
       </c>
       <c r="G26" t="inlineStr" s="2">
@@ -20112,7 +20407,7 @@
       </c>
       <c r="L79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Return Call_To__c masked</t>
+          <t xml:space="preserve">5b: GetData masks phone history values and call numbers for masked users</t>
         </is>
       </c>
     </row>
@@ -20472,7 +20767,7 @@
       </c>
       <c r="L85" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask numbers before writing log__c</t>
+          <t xml:space="preserve">5b: callRecords masked for masked users; log__c Request / Response masked for everyone</t>
         </is>
       </c>
     </row>
@@ -21012,7 +21307,7 @@
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Show Call_To__c masked</t>
+          <t xml:space="preserve">5b: NO CHANGE - shows what callRecords returns</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: v1.5.0 Part 5b call history and logs masked (built locally, not deployed)
Existing (approved, originals in backup/v1.5.0-part5b-pre-change):
- mCubeController: callRecords masked for masked users; 5 log__c
  Request/Response lines masked for everyone
- LeadHistoryandActivityController.GetData: phone history values (Phone__c,
  Secondary_Phone__c are history-tracked) and call numbers masked for masked users
Ours: PhoneDisplayService.forDisplay / historyValueForDisplay.
New: PhoneMaskingHistoryTest, Call_Detail__c.Call_To_Masked__c.
No change: mCubeLightningPage, LeadHistoryandActivityCmp.
Manifests, release bundle part5b-history, changelog, roadmap, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -20,15 +20,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$93</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$59</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$89</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$99</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
@@ -325,7 +325,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-5a)</t>
+          <t>Production Release Bundle - built components (Parts 1-5b)</t>
         </is>
       </c>
     </row>
@@ -4499,7 +4499,7 @@
       </c>
       <c r="H79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">fc8c29b6582e</t>
+          <t xml:space="preserve">9b008c83970d</t>
         </is>
       </c>
       <c r="I79" t="inlineStr" s="2">
@@ -4909,47 +4909,47 @@
       </c>
       <c r="B87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5b-history</t>
         </is>
       </c>
       <c r="C87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">LeadHistoryandActivityController</t>
         </is>
       </c>
       <c r="G87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part5b-history/classes/LeadHistoryandActivityController.cls</t>
         </is>
       </c>
       <c r="H87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
+          <t xml:space="preserve">6a02768af710</t>
         </is>
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J87" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K87" t="inlineStr" s="6">
@@ -4964,47 +4964,47 @@
       </c>
       <c r="B88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5b-history</t>
         </is>
       </c>
       <c r="C88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">LeadHistoryandActivityController</t>
         </is>
       </c>
       <c r="G88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part5b-history/classes/LeadHistoryandActivityController.cls-meta.xml</t>
         </is>
       </c>
       <c r="H88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">8ec13a9efa48</t>
         </is>
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J88" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K88" t="inlineStr" s="6">
@@ -5019,57 +5019,607 @@
       </c>
       <c r="B89" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mCubeController</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/classes/mCubeController.cls</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">683ff5c6df61</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2">
+        <v>6</v>
+      </c>
+      <c r="B90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">mCubeController</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/classes/mCubeController.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">311ca4a715d6</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2">
+        <v>6</v>
+      </c>
+      <c r="B91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/classes/PhoneDisplayService.cls</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9b008c83970d</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2">
+        <v>6</v>
+      </c>
+      <c r="B92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/classes/PhoneDisplayService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2">
+        <v>6</v>
+      </c>
+      <c r="B93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/classes/PhoneMaskingHistoryTest.cls</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">e4cb2b6bc259</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2">
+        <v>6</v>
+      </c>
+      <c r="B94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/classes/PhoneMaskingHistoryTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2">
+        <v>6</v>
+      </c>
+      <c r="B95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Call_Detail__c</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/objects/Call_Detail__c.object</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">77589815f51d</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2">
+        <v>6</v>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5b-history</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5b)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5b-history/package.xml</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b2eb9c547a99</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2">
+        <v>7</v>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr" s="2">
+      <c r="C97" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr" s="2">
+      <c r="D97" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr" s="2">
+      <c r="E97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2">
+        <v>7</v>
+      </c>
+      <c r="B98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2">
+        <v>7</v>
+      </c>
+      <c r="B99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr" s="2">
+      <c r="F99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr" s="2">
+      <c r="G99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H89" t="inlineStr" s="2">
+      <c r="H99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">df1ecd8c7bec</t>
         </is>
       </c>
-      <c r="I89" t="inlineStr" s="2">
+      <c r="I99" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr" s="4">
+      <c r="J99" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K89" t="inlineStr" s="6">
+      <c r="K99" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K89"/>
+  <autoFilter ref="A4:K99"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -5093,7 +5643,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-5a)</t>
+          <t>Production Deploy Steps (Parts 1-5b)</t>
         </is>
       </c>
     </row>
@@ -5288,47 +5838,49 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2">
-        <v>4</v>
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3e</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part5b-history</t>
         </is>
       </c>
       <c r="C11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5b-history --test-level RunSpecifiedTests --tests PhoneMaskingHistoryTest --tests PhoneDisplayServiceTest --tests mCubeController_Test --tests mCubeControllerTestExtended --tests LeadHistoryandActivityControllerTest</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="6">
@@ -5339,31 +5891,56 @@
     </row>
     <row r="13">
       <c r="A13" s="2">
+        <v>5</v>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2">
         <v>6</v>
       </c>
-      <c r="B13" t="inlineStr" s="2">
+      <c r="B14" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr" s="2">
+      <c r="C14" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr" s="2">
+      <c r="D14" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr" s="6">
+      <c r="E14" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E13"/>
+  <autoFilter ref="A4:E14"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -6663,12 +7240,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a deployed, call panels pending)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) - 5a</t>
+          <t xml:space="preserve">Mask leaking screens (5a deployed, 5b built, call panels deferred D1)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5b</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -11302,7 +11879,7 @@
       </c>
       <c r="I75" t="inlineStr" s="5">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Built (Local) - 5b</t>
         </is>
       </c>
       <c r="J75" t="inlineStr" s="2">
@@ -12401,8 +12978,128 @@
         </is>
       </c>
     </row>
+    <row r="94">
+      <c r="A94" s="2">
+        <v>90</v>
+      </c>
+      <c r="B94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5b: call history, History &amp; Activity and MCube log masking (callouts mocked)</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5b</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2">
+        <v>91</v>
+      </c>
+      <c r="B95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (update of new)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5b: + forDisplay, historyValueForDisplay</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5b</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L93"/>
+  <autoFilter ref="A4:L95"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -13682,22 +14379,22 @@
       </c>
       <c r="H24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5b-pre-change</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5b)</t>
         </is>
       </c>
       <c r="K24" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L24" t="inlineStr" s="2">
@@ -13742,17 +14439,17 @@
       </c>
       <c r="H25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I25" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5b-pre-change</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5b</t>
         </is>
       </c>
       <c r="K25" t="inlineStr" s="2">
@@ -13802,17 +14499,17 @@
       </c>
       <c r="H26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Approved 2026-10-06</t>
         </is>
       </c>
       <c r="I26" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5b-pre-change</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5b</t>
         </is>
       </c>
       <c r="K26" t="inlineStr" s="2">
@@ -15806,8 +16503,68 @@
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2">
+        <v>56</v>
+      </c>
+      <c r="B60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura Component</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadHistoryandActivityCmp</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5b: NO CHANGE - shows what GetData returns</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">History &amp; Activity on 4 Lead pages</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">backup/v1.5.0-part5b-pre-change</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5b)</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">First backed up in 5b</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L59"/>
+  <autoFilter ref="A4:L60"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -20907,12 +21664,12 @@
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updateContactDetails</t>
+          <t xml:space="preserve">PhoneDisplayService</t>
         </is>
       </c>
       <c r="F88" t="inlineStr" s="2">
@@ -20922,7 +21679,7 @@
       </c>
       <c r="G88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H88" t="inlineStr" s="2">
@@ -20932,7 +21689,7 @@
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="J88" t="inlineStr" s="2">
@@ -20947,7 +21704,7 @@
       </c>
       <c r="L88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Same</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -20967,12 +21724,12 @@
       </c>
       <c r="D89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+          <t xml:space="preserve">updateContactDetails</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
@@ -20982,7 +21739,7 @@
       </c>
       <c r="G89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H89" t="inlineStr" s="2">
@@ -21007,7 +21764,7 @@
       </c>
       <c r="L89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Same</t>
         </is>
       </c>
     </row>
@@ -21032,7 +21789,7 @@
       </c>
       <c r="E90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
@@ -21067,7 +21824,7 @@
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing test classes unchanged</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -21087,12 +21844,12 @@
       </c>
       <c r="D91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -21102,7 +21859,7 @@
       </c>
       <c r="G91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H91" t="inlineStr" s="2">
@@ -21127,7 +21884,7 @@
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
+          <t xml:space="preserve">Existing test classes unchanged</t>
         </is>
       </c>
     </row>
@@ -21147,12 +21904,12 @@
       </c>
       <c r="D92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
@@ -21162,7 +21919,7 @@
       </c>
       <c r="G92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H92" t="inlineStr" s="2">
@@ -21187,7 +21944,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -21212,7 +21969,7 @@
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeCmp</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F93" t="inlineStr" s="2">
@@ -21247,7 +22004,7 @@
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -21272,7 +22029,7 @@
       </c>
       <c r="E94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeLightningPage</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F94" t="inlineStr" s="2">
@@ -21307,7 +22064,7 @@
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">5b: NO CHANGE - shows what callRecords returns</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -21332,7 +22089,7 @@
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">LeadMergeCmp</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
@@ -21367,7 +22124,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Masked numbers</t>
         </is>
       </c>
     </row>
@@ -21387,12 +22144,12 @@
       </c>
       <c r="D96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -21427,7 +22184,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -21452,7 +22209,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">leadBulkPush</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -21487,7 +22244,7 @@
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -21512,7 +22269,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -21547,7 +22304,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -21567,12 +22324,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">leadYotelPush</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -21582,7 +22339,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -21597,7 +22354,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -21607,7 +22364,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -21617,27 +22374,27 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
@@ -21657,7 +22414,7 @@
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="6">
@@ -21687,17 +22444,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -21747,12 +22504,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -21772,7 +22529,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -21787,7 +22544,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -21812,7 +22569,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -21832,7 +22589,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -21847,7 +22604,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -21867,12 +22624,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -21892,7 +22649,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -21932,7 +22689,7 @@
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -21987,12 +22744,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -22047,12 +22804,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -22097,22 +22854,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -22132,7 +22889,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -22147,7 +22904,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22167,34 +22924,34 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FreeTextMaskService</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J109" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
@@ -22207,7 +22964,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -22227,12 +22984,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -22242,7 +22999,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -22267,7 +23024,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22292,17 +23049,17 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -22312,7 +23069,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -22327,7 +23084,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -22347,22 +23104,22 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -22372,7 +23129,7 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
@@ -22387,7 +23144,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22407,12 +23164,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -22457,22 +23214,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -22482,7 +23239,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -22492,12 +23249,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -22507,7 +23264,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -22527,32 +23284,32 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FindByNumberController</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FindByNumberControllerTest</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -22587,12 +23344,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -22612,7 +23369,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -22627,7 +23384,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22652,7 +23409,7 @@
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -22662,7 +23419,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -22672,7 +23429,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -22687,7 +23444,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -22697,22 +23454,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -22747,7 +23504,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -22767,12 +23524,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -22807,7 +23564,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -22832,7 +23589,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -22887,12 +23644,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -22927,7 +23684,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -22952,7 +23709,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -22987,7 +23744,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -23012,7 +23769,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -23047,7 +23804,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -23072,7 +23829,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -23132,7 +23889,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -23187,12 +23944,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -23227,7 +23984,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -23237,22 +23994,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -23277,7 +24034,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -23287,7 +24044,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -23312,7 +24069,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -23372,7 +24129,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -23492,7 +24249,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -23587,7 +24344,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -23612,7 +24369,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -23647,7 +24404,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -23667,12 +24424,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -23682,7 +24439,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -23707,7 +24464,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -23727,12 +24484,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -23742,12 +24499,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -23767,7 +24524,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -23787,12 +24544,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -23817,7 +24574,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -23827,7 +24584,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -23837,22 +24594,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -23862,12 +24619,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -23877,7 +24634,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -23887,7 +24644,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -23907,12 +24664,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -23922,7 +24679,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -23947,7 +24704,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -23972,7 +24729,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -24032,7 +24789,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -24077,22 +24834,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -24102,12 +24859,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -24117,7 +24874,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -24127,7 +24884,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -24137,7 +24894,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -24152,7 +24909,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -24177,7 +24934,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -24187,7 +24944,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -24212,7 +24969,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -24237,7 +24994,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -24247,7 +25004,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -24257,7 +25014,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -24272,7 +25029,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -24297,7 +25054,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -24307,7 +25064,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -24332,7 +25089,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -24367,7 +25124,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -24377,7 +25134,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -24392,7 +25149,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -24427,7 +25184,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -24452,7 +25209,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -24487,7 +25244,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -24497,62 +25254,122 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2">
+        <v>145</v>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr" s="2">
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr" s="2">
+      <c r="E149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr" s="2">
+      <c r="F149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr" s="2">
+      <c r="H149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr" s="2">
+      <c r="I149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr" s="6">
+      <c r="K149" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr" s="2">
+      <c r="L149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L148"/>
+  <autoFilter ref="A4:L149"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
deploy: Part 5b to sandbox; tracking updated
0Afft000000LfszCAC: 5/5, 61 tests passed (incl. existing mCubeController_Test,
mCubeControllerTestExtended, LeadHistoryandActivityControllerTest).
Coverage: PhoneDisplayService 100%, LeadHistoryandActivityController 87.1%,
mCubeController 81.4%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -4947,9 +4947,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J87" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J87" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K87" t="inlineStr" s="6">
@@ -5002,9 +5002,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J88" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K88" t="inlineStr" s="6">
@@ -5057,9 +5057,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J89" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K89" t="inlineStr" s="6">
@@ -5112,9 +5112,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J90" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J90" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K90" t="inlineStr" s="6">
@@ -5167,9 +5167,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J91" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J91" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K91" t="inlineStr" s="6">
@@ -5222,9 +5222,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J92" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J92" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K92" t="inlineStr" s="6">
@@ -5277,9 +5277,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J93" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J93" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K93" t="inlineStr" s="6">
@@ -5332,9 +5332,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J94" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J94" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K94" t="inlineStr" s="6">
@@ -5387,9 +5387,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J95" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J95" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K95" t="inlineStr" s="6">
@@ -5442,9 +5442,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J96" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J96" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K96" t="inlineStr" s="6">
@@ -7240,12 +7240,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a deployed, 5b built, call panels deferred D1)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5b</t>
+          <t xml:space="preserve">Mask leaking screens (5a + 5b deployed, call panels deferred D1)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) - 5a, 5b</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -11877,9 +11877,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I75" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5b</t>
+      <c r="I75" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="J75" t="inlineStr" s="2">
@@ -13017,14 +13017,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I94" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5b</t>
+      <c r="I94" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K94" t="inlineStr" s="2">
@@ -13077,14 +13077,14 @@
           <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5b</t>
+      <c r="I95" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K95" t="inlineStr" s="2">
@@ -14447,9 +14447,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5b-pre-change</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5b</t>
+      <c r="J25" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K25" t="inlineStr" s="2">
@@ -14507,9 +14507,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5b-pre-change</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5b</t>
+      <c r="J26" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LfszCAC</t>
         </is>
       </c>
       <c r="K26" t="inlineStr" s="2">

</xml_diff>

<commit_message>
docs: Part 5c plan in the register (Lead Merge, Update Contact Details)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -16,13 +16,14 @@
     <sheet name="Part 4 Plan" sheetId="12" r:id="rId12"/>
     <sheet name="Part 5a Plan" sheetId="13" r:id="rId13"/>
     <sheet name="Part 5b Plan" sheetId="14" r:id="rId14"/>
+    <sheet name="Part 5c Plan" sheetId="15" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$95</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
@@ -32,6 +33,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Part 5c Plan'!$A$4:$F$10</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -7021,6 +7023,267 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="90" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 5c (v1.5.0) - Lead Merge and Update Contact Details</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; originals in backup/v1.5.0-part5c-pre-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Updated (ours)</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">+ maskRecords(records, fields): masks phone fields on a result list for masked users (in memory only). + prepareContactInput(recordId, phone, secondaryPhone): a masked value sent back by a screen is replaced by the stored number (never saved masked); for masked users the primary stays locked once set.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Same rules as Parts 4 / 5a</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Merge lists masked / unchanged; Update Contact: masked values never saved, secondary change saved, primary change refused for masked users, unmasked users unchanged</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadMergeController</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">getLeads / getSearchLeads: phone numbers in the results masked for masked users (2 return lines become assign + mask + return). mergeLead unchanged.</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Merge screen shows 98XXXXXX21 for masked users; merge works as before</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updateContactDetails</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">getcontactdetails: +1 line (mask for masked users). savecontactdetails: +5 lines at the top (prepareContactInput) - masked values restored to the stored numbers, primary locked for masked users.</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked users: see masked, can change secondary + emails; a masked value is never written back. Others: unchanged.</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Medium (writes data) - covered by new + existing tests</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Aura</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadMergeCmp, UpdateContactDetails</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Screens show what Apex returns; the phone inputs have no format check, so masked values pass validation</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing issue (not changed)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadMergeController.getLeads</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Returns every Lead except the current one with no limit, and the class has no sharing keyword</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Report to the owner; out of scope</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
@@ -14549,7 +14812,7 @@
       </c>
       <c r="F27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve">5c: NO CHANGE - shows what Apex returns</t>
         </is>
       </c>
       <c r="G27" t="inlineStr" s="2">
@@ -14559,22 +14822,22 @@
       </c>
       <c r="H27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5c)</t>
         </is>
       </c>
       <c r="K27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L27" t="inlineStr" s="2">
@@ -14619,12 +14882,12 @@
       </c>
       <c r="H28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
       <c r="J28" t="inlineStr" s="6">
@@ -14679,12 +14942,12 @@
       </c>
       <c r="H29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
       <c r="J29" t="inlineStr" s="6">
@@ -14739,12 +15002,12 @@
       </c>
       <c r="H30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
       <c r="J30" t="inlineStr" s="6">
@@ -21604,7 +21867,7 @@
       </c>
       <c r="D87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E87" t="inlineStr" s="2">
@@ -21629,7 +21892,7 @@
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="J87" t="inlineStr" s="2">
@@ -21664,7 +21927,7 @@
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (update of new)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
@@ -21689,7 +21952,7 @@
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="J88" t="inlineStr" s="2">
@@ -22089,7 +22352,7 @@
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">LeadMergeCmp</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
@@ -22124,7 +22387,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -22144,12 +22407,12 @@
       </c>
       <c r="D96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">leadBulkPush</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -22184,7 +22447,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -22209,7 +22472,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -22244,7 +22507,7 @@
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -22269,7 +22532,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">leadYotelPush</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -22304,7 +22567,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -22324,12 +22587,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -22339,7 +22602,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -22354,7 +22617,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -22364,7 +22627,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22374,27 +22637,27 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
@@ -22414,7 +22677,7 @@
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="6">
@@ -22444,17 +22707,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -22504,12 +22767,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -22529,7 +22792,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -22544,7 +22807,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -22569,7 +22832,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -22589,7 +22852,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -22604,7 +22867,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22624,12 +22887,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -22649,7 +22912,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -22689,7 +22952,7 @@
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -22744,12 +23007,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -22804,12 +23067,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -22854,22 +23117,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -22889,7 +23152,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -22904,7 +23167,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -22924,12 +23187,12 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
@@ -22949,7 +23212,7 @@
       </c>
       <c r="I109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J109" t="inlineStr" s="2">
@@ -22964,7 +23227,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22984,12 +23247,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -22999,7 +23262,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -23024,7 +23287,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -23049,17 +23312,17 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -23069,7 +23332,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -23084,7 +23347,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23104,22 +23367,22 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -23129,7 +23392,7 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
@@ -23144,7 +23407,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -23164,12 +23427,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -23214,22 +23477,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -23239,7 +23502,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -23249,12 +23512,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -23264,7 +23527,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23284,12 +23547,12 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -23309,7 +23572,7 @@
       </c>
       <c r="I115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -23344,12 +23607,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -23369,7 +23632,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -23384,7 +23647,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -23409,7 +23672,7 @@
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -23419,7 +23682,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -23429,7 +23692,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -23444,7 +23707,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -23454,22 +23717,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -23504,7 +23767,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -23524,12 +23787,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -23564,7 +23827,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -23589,7 +23852,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -23644,12 +23907,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -23684,7 +23947,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -23709,7 +23972,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -23744,7 +24007,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -23769,7 +24032,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -23804,7 +24067,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -23829,7 +24092,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -23889,7 +24152,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -23944,12 +24207,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -23984,7 +24247,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -23994,22 +24257,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -24034,7 +24297,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -24044,7 +24307,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -24069,7 +24332,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -24129,7 +24392,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -24249,7 +24512,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -24344,7 +24607,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -24369,7 +24632,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -24404,7 +24667,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -24424,12 +24687,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -24439,7 +24702,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -24464,7 +24727,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -24484,12 +24747,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -24499,12 +24762,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -24524,7 +24787,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -24544,12 +24807,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -24574,7 +24837,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -24584,7 +24847,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -24594,22 +24857,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -24619,12 +24882,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -24634,7 +24897,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -24644,7 +24907,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -24664,12 +24927,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -24679,7 +24942,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -24704,7 +24967,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -24729,7 +24992,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -24789,7 +25052,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -24834,22 +25097,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Manual step</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -24859,12 +25122,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -24874,7 +25137,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -24884,7 +25147,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -24894,7 +25157,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -24909,7 +25172,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -24934,7 +25197,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -24944,7 +25207,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -24969,7 +25232,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -24994,7 +25257,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -25004,7 +25267,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -25014,7 +25277,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -25029,7 +25292,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -25054,7 +25317,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -25064,7 +25327,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -25089,7 +25352,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -25124,7 +25387,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -25134,7 +25397,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -25149,7 +25412,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -25184,7 +25447,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -25209,7 +25472,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M12</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -25244,7 +25507,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
         </is>
       </c>
     </row>
@@ -25254,7 +25517,7 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 13</t>
         </is>
       </c>
       <c r="C148" t="inlineStr" s="2">
@@ -25269,7 +25532,7 @@
       </c>
       <c r="E148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M13</t>
         </is>
       </c>
       <c r="F148" t="inlineStr" s="2">
@@ -25304,72 +25567,12 @@
       </c>
       <c r="L148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2">
-        <v>145</v>
-      </c>
-      <c r="B149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 13</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual step</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">M13</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L149"/>
+  <autoFilter ref="A4:L148"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
feat: v1.5.0 Part 5c Lead Merge and Update Contact Details masked (built locally, not deployed)
Existing (approved, originals in backup/v1.5.0-part5c-pre-change):
- LeadMergeController: merge lists masked for masked users
- updateContactDetails: masked for masked users; masked values from the screen
  are never saved (stored number kept); primary locked for masked users
Ours: PhoneDisplayService.maskRecords / prepareContactInput.
New: PhoneMaskingLeadToolsTest (8 tests).
No change: LeadMergeCmp, UpdateContactDetails.
Manifests, release bundle part5c-lead-tools, changelog, roadmap, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -21,15 +21,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$95</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$150</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$99</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$14</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$108</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
@@ -327,7 +327,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-5b)</t>
+          <t>Production Release Bundle - built components (Parts 1-5c)</t>
         </is>
       </c>
     </row>
@@ -4501,7 +4501,7 @@
       </c>
       <c r="H79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9b008c83970d</t>
+          <t xml:space="preserve">395e19ee99fa</t>
         </is>
       </c>
       <c r="I79" t="inlineStr" s="2">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="H91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9b008c83970d</t>
+          <t xml:space="preserve">395e19ee99fa</t>
         </is>
       </c>
       <c r="I91" t="inlineStr" s="2">
@@ -5461,47 +5461,47 @@
       </c>
       <c r="B97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5c-lead-tools</t>
         </is>
       </c>
       <c r="C97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">LeadMergeController</t>
         </is>
       </c>
       <c r="G97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/LeadMergeController.cls</t>
         </is>
       </c>
       <c r="H97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
+          <t xml:space="preserve">c0cd2ecb5940</t>
         </is>
       </c>
       <c r="I97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J97" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K97" t="inlineStr" s="6">
@@ -5516,47 +5516,47 @@
       </c>
       <c r="B98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5c-lead-tools</t>
         </is>
       </c>
       <c r="C98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
         </is>
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">LeadMergeController</t>
         </is>
       </c>
       <c r="G98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/LeadMergeController.cls-meta.xml</t>
         </is>
       </c>
       <c r="H98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">8ec13a9efa48</t>
         </is>
       </c>
       <c r="I98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J98" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K98" t="inlineStr" s="6">
@@ -5571,57 +5571,552 @@
       </c>
       <c r="B99" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/PhoneDisplayService.cls</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">395e19ee99fa</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2">
+        <v>7</v>
+      </c>
+      <c r="B100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/PhoneDisplayService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2">
+        <v>7</v>
+      </c>
+      <c r="B101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updateContactDetails</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/updateContactDetails.cls</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3157a9439853</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2">
+        <v>7</v>
+      </c>
+      <c r="B102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">updateContactDetails</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/updateContactDetails.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">8ec13a9efa48</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2">
+        <v>7</v>
+      </c>
+      <c r="B103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/PhoneMaskingLeadToolsTest.cls</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">95a18c94dfa3</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="2">
+        <v>7</v>
+      </c>
+      <c r="B104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/classes/PhoneMaskingLeadToolsTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K104" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2">
+        <v>7</v>
+      </c>
+      <c r="B105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5c-lead-tools</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5c)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5c-lead-tools/package.xml</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">66bd9f007bec</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2">
+        <v>8</v>
+      </c>
+      <c r="B106" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr" s="2">
+      <c r="C106" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr" s="2">
+      <c r="D106" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E99" t="inlineStr" s="2">
+      <c r="E106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2">
+        <v>8</v>
+      </c>
+      <c r="B107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2">
+        <v>8</v>
+      </c>
+      <c r="B108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F99" t="inlineStr" s="2">
+      <c r="F108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G99" t="inlineStr" s="2">
+      <c r="G108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr" s="2">
+      <c r="H108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">df1ecd8c7bec</t>
         </is>
       </c>
-      <c r="I99" t="inlineStr" s="2">
+      <c r="I108" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr" s="4">
+      <c r="J108" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K99" t="inlineStr" s="6">
+      <c r="K108" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K99"/>
+  <autoFilter ref="A4:K108"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -5645,7 +6140,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-5b)</t>
+          <t>Production Deploy Steps (Parts 1-5c)</t>
         </is>
       </c>
     </row>
@@ -5867,47 +6362,49 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2">
-        <v>4</v>
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3f</t>
+        </is>
       </c>
       <c r="B12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part5c-lead-tools</t>
         </is>
       </c>
       <c r="C12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5c-lead-tools --test-level RunSpecifiedTests --tests PhoneMaskingLeadToolsTest --tests PhoneDisplayServiceTest --tests LeadMergeControllerTest --tests updateContactDetailsTest</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E13" t="inlineStr" s="6">
@@ -5918,31 +6415,56 @@
     </row>
     <row r="14">
       <c r="A14" s="2">
+        <v>5</v>
+      </c>
+      <c r="B14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2">
         <v>6</v>
       </c>
-      <c r="B14" t="inlineStr" s="2">
+      <c r="B15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr" s="2">
+      <c r="C15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr" s="2">
+      <c r="D15" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr" s="6">
+      <c r="E15" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E14"/>
+  <autoFilter ref="A4:E15"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -7503,12 +8025,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a + 5b deployed, call panels deferred D1)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) - 5a, 5b</t>
+          <t xml:space="preserve">Mask leaking screens (5a + 5b deployed, 5c built, call panels deferred D1)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5c</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -13361,8 +13883,128 @@
         </is>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" s="2">
+        <v>92</v>
+      </c>
+      <c r="B96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5c: merge lists masked; Update Contact never saves masked values, primary locked for masked users</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5c</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2">
+        <v>93</v>
+      </c>
+      <c r="B97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (update of new)</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneDisplayService</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5c: + maskRecords, prepareContactInput</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5c</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L95"/>
+  <autoFilter ref="A4:L97"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -14882,7 +15524,7 @@
       </c>
       <c r="H28" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-07</t>
         </is>
       </c>
       <c r="I28" t="inlineStr" s="2">
@@ -14890,9 +15532,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J28" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5c</t>
         </is>
       </c>
       <c r="K28" t="inlineStr" s="2">
@@ -14942,7 +15584,7 @@
       </c>
       <c r="H29" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-07</t>
         </is>
       </c>
       <c r="I29" t="inlineStr" s="2">
@@ -14950,9 +15592,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J29" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5c</t>
         </is>
       </c>
       <c r="K29" t="inlineStr" s="2">
@@ -15002,7 +15644,7 @@
       </c>
       <c r="H30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-07</t>
         </is>
       </c>
       <c r="I30" t="inlineStr" s="2">
@@ -15010,9 +15652,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J30" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5c</t>
         </is>
       </c>
       <c r="K30" t="inlineStr" s="2">
@@ -21987,12 +22629,12 @@
       </c>
       <c r="D89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">updateContactDetails</t>
+          <t xml:space="preserve">PhoneDisplayService</t>
         </is>
       </c>
       <c r="F89" t="inlineStr" s="2">
@@ -22002,7 +22644,7 @@
       </c>
       <c r="G89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H89" t="inlineStr" s="2">
@@ -22012,7 +22654,7 @@
       </c>
       <c r="I89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
         </is>
       </c>
       <c r="J89" t="inlineStr" s="2">
@@ -22027,7 +22669,7 @@
       </c>
       <c r="L89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Same</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22047,12 +22689,12 @@
       </c>
       <c r="D90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+          <t xml:space="preserve">updateContactDetails</t>
         </is>
       </c>
       <c r="F90" t="inlineStr" s="2">
@@ -22062,7 +22704,7 @@
       </c>
       <c r="G90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H90" t="inlineStr" s="2">
@@ -22087,7 +22729,7 @@
       </c>
       <c r="L90" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Same</t>
         </is>
       </c>
     </row>
@@ -22112,7 +22754,7 @@
       </c>
       <c r="E91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="F91" t="inlineStr" s="2">
@@ -22147,7 +22789,7 @@
       </c>
       <c r="L91" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing test classes unchanged</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22172,7 +22814,7 @@
       </c>
       <c r="E92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+          <t xml:space="preserve">PhoneMaskingCallScreensTest</t>
         </is>
       </c>
       <c r="F92" t="inlineStr" s="2">
@@ -22207,7 +22849,7 @@
       </c>
       <c r="L92" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Existing test classes unchanged</t>
         </is>
       </c>
     </row>
@@ -22227,12 +22869,12 @@
       </c>
       <c r="D93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="F93" t="inlineStr" s="2">
@@ -22242,7 +22884,7 @@
       </c>
       <c r="G93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H93" t="inlineStr" s="2">
@@ -22267,7 +22909,7 @@
       </c>
       <c r="L93" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22287,12 +22929,12 @@
       </c>
       <c r="D94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
         </is>
       </c>
       <c r="F94" t="inlineStr" s="2">
@@ -22302,7 +22944,7 @@
       </c>
       <c r="G94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H94" t="inlineStr" s="2">
@@ -22327,7 +22969,7 @@
       </c>
       <c r="L94" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22352,7 +22994,7 @@
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
@@ -22387,7 +23029,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -22407,12 +23049,12 @@
       </c>
       <c r="D96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -22447,7 +23089,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -22467,12 +23109,12 @@
       </c>
       <c r="D97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -22507,7 +23149,7 @@
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -22532,7 +23174,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">leadBulkPush</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -22587,12 +23229,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -22602,7 +23244,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -22617,7 +23259,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -22627,7 +23269,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -22637,32 +23279,32 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">leadYotelPush</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H100" t="inlineStr" s="2">
@@ -22687,7 +23329,7 @@
       </c>
       <c r="L100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked selection list</t>
         </is>
       </c>
     </row>
@@ -22697,22 +23339,22 @@
       </c>
       <c r="B101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
@@ -22737,7 +23379,7 @@
       </c>
       <c r="J101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K101" t="inlineStr" s="6">
@@ -22767,17 +23409,17 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G102" t="inlineStr" s="2">
@@ -22792,7 +23434,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -22807,7 +23449,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -22827,12 +23469,12 @@
       </c>
       <c r="D103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -22852,7 +23494,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -22887,34 +23529,34 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H104" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I104" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J104" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
@@ -22927,7 +23569,7 @@
       </c>
       <c r="L104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -22947,32 +23589,32 @@
       </c>
       <c r="D105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">PhoneRevealService</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">PhoneRevealServiceTest</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H105" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I105" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J105" t="inlineStr" s="2">
@@ -23007,12 +23649,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -23067,12 +23709,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -23117,22 +23759,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -23152,7 +23794,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -23167,7 +23809,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23177,22 +23819,22 @@
       </c>
       <c r="B109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
@@ -23247,12 +23889,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -23262,7 +23904,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -23272,7 +23914,7 @@
       </c>
       <c r="I110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J110" t="inlineStr" s="2">
@@ -23287,7 +23929,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -23307,17 +23949,17 @@
       </c>
       <c r="D111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
@@ -23332,7 +23974,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -23367,12 +24009,12 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
@@ -23407,7 +24049,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -23432,17 +24074,17 @@
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H113" t="inlineStr" s="2">
@@ -23452,7 +24094,7 @@
       </c>
       <c r="I113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J113" t="inlineStr" s="2">
@@ -23467,7 +24109,7 @@
       </c>
       <c r="L113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23477,22 +24119,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -23502,7 +24144,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -23512,12 +24154,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -23527,7 +24169,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -23537,22 +24179,22 @@
       </c>
       <c r="B115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -23562,7 +24204,7 @@
       </c>
       <c r="G115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H115" t="inlineStr" s="2">
@@ -23577,7 +24219,7 @@
       </c>
       <c r="J115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K115" t="inlineStr" s="6">
@@ -23587,7 +24229,7 @@
       </c>
       <c r="L115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -23607,12 +24249,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -23632,7 +24274,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -23647,7 +24289,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23667,12 +24309,12 @@
       </c>
       <c r="D117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -23682,7 +24324,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -23707,7 +24349,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23717,22 +24359,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -23742,7 +24384,7 @@
       </c>
       <c r="G118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H118" t="inlineStr" s="2">
@@ -23752,7 +24394,7 @@
       </c>
       <c r="I118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J118" t="inlineStr" s="2">
@@ -23767,7 +24409,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -23777,22 +24419,22 @@
       </c>
       <c r="B119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -23827,7 +24469,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -23847,12 +24489,12 @@
       </c>
       <c r="D120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -23887,7 +24529,7 @@
       </c>
       <c r="L120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -23907,12 +24549,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -23947,7 +24589,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -23967,12 +24609,12 @@
       </c>
       <c r="D122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -24007,7 +24649,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24032,7 +24674,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -24067,7 +24709,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -24092,7 +24734,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -24127,7 +24769,7 @@
       </c>
       <c r="L124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -24152,7 +24794,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -24207,12 +24849,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -24247,7 +24889,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24257,22 +24899,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -24297,7 +24939,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -24307,7 +24949,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24317,22 +24959,22 @@
       </c>
       <c r="B128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -24357,7 +24999,7 @@
       </c>
       <c r="J128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K128" t="inlineStr" s="6">
@@ -24367,7 +25009,7 @@
       </c>
       <c r="L128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -24392,7 +25034,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -24452,7 +25094,7 @@
       </c>
       <c r="E130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F130" t="inlineStr" s="2">
@@ -24487,7 +25129,7 @@
       </c>
       <c r="L130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -24512,7 +25154,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -24547,7 +25189,7 @@
       </c>
       <c r="L131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -24572,7 +25214,7 @@
       </c>
       <c r="E132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F132" t="inlineStr" s="2">
@@ -24607,7 +25249,7 @@
       </c>
       <c r="L132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -24632,7 +25274,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -24687,12 +25329,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -24702,7 +25344,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -24727,7 +25369,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -24747,12 +25389,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -24767,7 +25409,7 @@
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -24787,7 +25429,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -24807,12 +25449,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -24822,12 +25464,12 @@
       </c>
       <c r="G136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I136" t="inlineStr" s="2">
@@ -24837,7 +25479,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -24847,7 +25489,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -24857,22 +25499,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -24882,12 +25524,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -24897,7 +25539,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -24907,7 +25549,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -24917,22 +25559,22 @@
       </c>
       <c r="B138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -24947,7 +25589,7 @@
       </c>
       <c r="H138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I138" t="inlineStr" s="2">
@@ -24957,7 +25599,7 @@
       </c>
       <c r="J138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K138" t="inlineStr" s="6">
@@ -24967,7 +25609,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -24987,12 +25629,12 @@
       </c>
       <c r="D139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -25002,7 +25644,7 @@
       </c>
       <c r="G139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H139" t="inlineStr" s="2">
@@ -25027,7 +25669,7 @@
       </c>
       <c r="L139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -25052,7 +25694,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -25097,22 +25739,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -25122,12 +25764,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -25137,7 +25779,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -25147,7 +25789,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -25157,22 +25799,22 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -25182,12 +25824,12 @@
       </c>
       <c r="G142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I142" t="inlineStr" s="2">
@@ -25197,7 +25839,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -25207,7 +25849,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -25217,7 +25859,7 @@
       </c>
       <c r="B143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C143" t="inlineStr" s="2">
@@ -25232,7 +25874,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -25257,7 +25899,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -25267,7 +25909,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -25277,7 +25919,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -25292,7 +25934,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -25317,7 +25959,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -25327,7 +25969,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -25337,7 +25979,7 @@
       </c>
       <c r="B145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C145" t="inlineStr" s="2">
@@ -25352,7 +25994,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -25377,7 +26019,7 @@
       </c>
       <c r="J145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K145" t="inlineStr" s="6">
@@ -25387,7 +26029,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -25397,7 +26039,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -25412,7 +26054,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -25447,7 +26089,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -25457,7 +26099,7 @@
       </c>
       <c r="B147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C147" t="inlineStr" s="2">
@@ -25472,7 +26114,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -25507,7 +26149,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -25517,62 +26159,182 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M11</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2">
+        <v>145</v>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K149" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2">
+        <v>146</v>
+      </c>
+      <c r="B150" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr" s="2">
+      <c r="C150" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr" s="2">
+      <c r="E150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr" s="2">
+      <c r="F150" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr" s="2">
+      <c r="H150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr" s="2">
+      <c r="I150" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr" s="6">
+      <c r="K150" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr" s="2">
+      <c r="L150" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L148"/>
+  <autoFilter ref="A4:L150"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
deploy: Part 5c to sandbox; pre-existing test failure recorded (D3)
0Afft000000LkRFCA0: 4/4, 23 tests passed. Coverage: PhoneDisplayService 92.9%,
updateContactDetails 84.6%, LeadMergeController 79.3%.
Existing updateContactDetailsTest fails before 5c (Too many SOQL queries: 101
in LeadTrigger line 232) - excluded; PhoneMaskingLeadToolsTest now also covers
the existing savecontactdetails branches. Roadmap D3, changelog, release
README, register updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -5499,9 +5499,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J97" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J97" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K97" t="inlineStr" s="6">
@@ -5554,9 +5554,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J98" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J98" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K98" t="inlineStr" s="6">
@@ -5609,9 +5609,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J99" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J99" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -5664,9 +5664,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J100" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J100" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="6">
@@ -5719,9 +5719,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J101" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J101" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K101" t="inlineStr" s="6">
@@ -5774,9 +5774,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J102" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J102" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K102" t="inlineStr" s="6">
@@ -5829,9 +5829,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J103" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J103" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K103" t="inlineStr" s="6">
@@ -5884,9 +5884,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J104" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J104" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K104" t="inlineStr" s="6">
@@ -5939,9 +5939,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J105" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J105" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K105" t="inlineStr" s="6">
@@ -6379,7 +6379,7 @@
       </c>
       <c r="D12" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5c-lead-tools --test-level RunSpecifiedTests --tests PhoneMaskingLeadToolsTest --tests PhoneDisplayServiceTest --tests LeadMergeControllerTest --tests updateContactDetailsTest</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5c-lead-tools --test-level RunSpecifiedTests --tests PhoneMaskingLeadToolsTest --tests PhoneDisplayServiceTest --tests LeadMergeControllerTest (not updateContactDetailsTest - fails before 5c, D3)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr" s="2">
@@ -8025,12 +8025,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a + 5b deployed, 5c built, call panels deferred D1)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5c</t>
+          <t xml:space="preserve">Mask leaking screens (5a-5c deployed, call panels deferred D1)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) - 5a, 5b, 5c</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -13922,14 +13922,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I96" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5c</t>
+      <c r="I96" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K96" t="inlineStr" s="2">
@@ -13982,14 +13982,14 @@
           <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
         </is>
       </c>
-      <c r="I97" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5c</t>
+      <c r="I97" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K97" t="inlineStr" s="2">
@@ -15532,9 +15532,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5c</t>
+      <c r="J28" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K28" t="inlineStr" s="2">
@@ -15592,9 +15592,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5c</t>
+      <c r="J29" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K29" t="inlineStr" s="2">
@@ -15652,9 +15652,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5c-pre-change</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5c</t>
+      <c r="J30" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LkRFCA0</t>
         </is>
       </c>
       <c r="K30" t="inlineStr" s="2">

</xml_diff>

<commit_message>
backup + plan: Part 5d (Bulk push and Yotel push)
Backup of both push controllers (+tests), LWCs, Aura wrappers/apps and VF host
pages (first backup for 8 of them) - read-only. Plan sheet in the register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -17,13 +17,14 @@
     <sheet name="Part 5a Plan" sheetId="13" r:id="rId13"/>
     <sheet name="Part 5b Plan" sheetId="14" r:id="rId14"/>
     <sheet name="Part 5c Plan" sheetId="15" r:id="rId15"/>
+    <sheet name="Part 5d Plan" sheetId="16" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$97</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
@@ -34,6 +35,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Part 5c Plan'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Part 5d Plan'!$A$4:$F$10</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -7806,6 +7808,267 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="80" customWidth="1"/>
+    <col min="5" max="5" width="54" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 5d (v1.5.0) - Bulk push and Yotel push</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; originals in backup/v1.5.0-part5d-pre-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadBulkPushController.getSelectedLeads</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">w.mobileNumber = PhoneDisplayService.forDisplay(l.MobilePhone) - 1 line</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked users: masked in the data sent to the screen (Bulk push does not display it). Others: unchanged</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadYotelBulkPushController.getSelectedLeads</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">w.mobileNumber = PhoneDisplayService.forDisplay(l.Phone__c) - 1 line; eligibility still computed from the real number; the debug line logs the masked number</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked users: Yotel selection table shows 98XXXXXX21. Others: unchanged</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">pushBulkToDialer, pushBulkToYotel</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Receive Lead Ids only and read the real numbers on the server - vendors still get real numbers</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LWC / Aura / VF</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">leadBulkPush, leadYotelPush, wrappers, apps, BulkLeadPUSHpage, BulkLeadPushYotel</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Display what Apex returns</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingPushTest</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Selection lists masked for masked users, unchanged for others; eligibility unchanged</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Not in scope</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">getUserPicklistValues, rmMobileNumber</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Agent / user numbers, not customer numbers</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>
@@ -15694,7 +15957,7 @@
       </c>
       <c r="F31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">5d: NO CHANGE - shows what Apex returns</t>
         </is>
       </c>
       <c r="G31" t="inlineStr" s="2">
@@ -15704,22 +15967,22 @@
       </c>
       <c r="H31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5d)</t>
         </is>
       </c>
       <c r="K31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L31" t="inlineStr" s="2">
@@ -15764,12 +16027,12 @@
       </c>
       <c r="H32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
         </is>
       </c>
       <c r="J32" t="inlineStr" s="6">
@@ -15814,7 +16077,7 @@
       </c>
       <c r="F33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">5d: NO CHANGE - shows what Apex returns</t>
         </is>
       </c>
       <c r="G33" t="inlineStr" s="2">
@@ -15824,22 +16087,22 @@
       </c>
       <c r="H33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5d)</t>
         </is>
       </c>
       <c r="K33" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L33" t="inlineStr" s="2">
@@ -15884,12 +16147,12 @@
       </c>
       <c r="H34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
         </is>
       </c>
       <c r="J34" t="inlineStr" s="6">
@@ -22534,7 +22797,7 @@
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
         </is>
       </c>
       <c r="J87" t="inlineStr" s="2">
@@ -22569,7 +22832,7 @@
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
@@ -22594,7 +22857,7 @@
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="J88" t="inlineStr" s="2">
@@ -22629,7 +22892,7 @@
       </c>
       <c r="D89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (update of new)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E89" t="inlineStr" s="2">
@@ -22654,7 +22917,7 @@
       </c>
       <c r="I89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="J89" t="inlineStr" s="2">
@@ -23174,7 +23437,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadBulkPush</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -23209,7 +23472,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -23229,12 +23492,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -23244,7 +23507,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -23259,7 +23522,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -23269,7 +23532,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23279,32 +23542,32 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadYotelPush</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H100" t="inlineStr" s="2">
@@ -23329,7 +23592,7 @@
       </c>
       <c r="L100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked selection list</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23339,22 +23602,22 @@
       </c>
       <c r="B101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
@@ -23379,7 +23642,7 @@
       </c>
       <c r="J101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K101" t="inlineStr" s="6">
@@ -23409,17 +23672,17 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G102" t="inlineStr" s="2">
@@ -23434,7 +23697,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -23449,7 +23712,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -23469,12 +23732,12 @@
       </c>
       <c r="D103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -23494,7 +23757,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -23529,12 +23792,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -23554,7 +23817,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -23569,7 +23832,7 @@
       </c>
       <c r="L104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23589,12 +23852,12 @@
       </c>
       <c r="D105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -23614,7 +23877,7 @@
       </c>
       <c r="I105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J105" t="inlineStr" s="2">
@@ -23649,12 +23912,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -23709,12 +23972,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -23759,22 +24022,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -23794,7 +24057,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -23809,7 +24072,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -23819,22 +24082,22 @@
       </c>
       <c r="B109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
@@ -23889,12 +24152,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -23904,7 +24167,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -23914,7 +24177,7 @@
       </c>
       <c r="I110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J110" t="inlineStr" s="2">
@@ -23929,7 +24192,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -23949,32 +24212,32 @@
       </c>
       <c r="D111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">FeedItem</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FreeTextMaskServiceTest</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H111" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I111" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -24009,12 +24272,12 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
@@ -24049,7 +24312,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -24074,17 +24337,17 @@
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H113" t="inlineStr" s="2">
@@ -24094,7 +24357,7 @@
       </c>
       <c r="I113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J113" t="inlineStr" s="2">
@@ -24109,7 +24372,7 @@
       </c>
       <c r="L113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -24119,22 +24382,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -24144,7 +24407,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -24154,12 +24417,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -24169,7 +24432,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24179,22 +24442,22 @@
       </c>
       <c r="B115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -24204,7 +24467,7 @@
       </c>
       <c r="G115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H115" t="inlineStr" s="2">
@@ -24219,7 +24482,7 @@
       </c>
       <c r="J115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K115" t="inlineStr" s="6">
@@ -24229,7 +24492,7 @@
       </c>
       <c r="L115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24249,12 +24512,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -24274,7 +24537,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -24289,7 +24552,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -24309,12 +24572,12 @@
       </c>
       <c r="D117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -24324,7 +24587,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -24349,7 +24612,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -24359,22 +24622,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -24384,7 +24647,7 @@
       </c>
       <c r="G118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H118" t="inlineStr" s="2">
@@ -24394,7 +24657,7 @@
       </c>
       <c r="I118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J118" t="inlineStr" s="2">
@@ -24409,7 +24672,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -24419,22 +24682,22 @@
       </c>
       <c r="B119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -24469,7 +24732,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24489,12 +24752,12 @@
       </c>
       <c r="D120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -24529,7 +24792,7 @@
       </c>
       <c r="L120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24549,12 +24812,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -24589,7 +24852,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -24609,12 +24872,12 @@
       </c>
       <c r="D122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -24649,7 +24912,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -24674,7 +24937,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -24709,7 +24972,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24734,7 +24997,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -24769,7 +25032,7 @@
       </c>
       <c r="L124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24794,7 +25057,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -24849,12 +25112,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -24889,7 +25152,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -24899,22 +25162,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -24939,7 +25202,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -24949,7 +25212,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -24959,22 +25222,22 @@
       </c>
       <c r="B128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -24999,7 +25262,7 @@
       </c>
       <c r="J128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K128" t="inlineStr" s="6">
@@ -25009,7 +25272,7 @@
       </c>
       <c r="L128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -25034,7 +25297,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -25069,7 +25332,7 @@
       </c>
       <c r="L129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -25094,7 +25357,7 @@
       </c>
       <c r="E130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F130" t="inlineStr" s="2">
@@ -25154,7 +25417,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -25214,7 +25477,7 @@
       </c>
       <c r="E132" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F132" t="inlineStr" s="2">
@@ -25274,7 +25537,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -25329,12 +25592,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -25344,7 +25607,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -25369,7 +25632,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -25389,12 +25652,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -25409,7 +25672,7 @@
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -25429,7 +25692,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -25449,12 +25712,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -25464,12 +25727,12 @@
       </c>
       <c r="G136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I136" t="inlineStr" s="2">
@@ -25479,7 +25742,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -25489,7 +25752,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -25499,22 +25762,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -25524,12 +25787,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -25539,7 +25802,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -25549,7 +25812,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -25559,22 +25822,22 @@
       </c>
       <c r="B138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -25589,7 +25852,7 @@
       </c>
       <c r="H138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I138" t="inlineStr" s="2">
@@ -25599,7 +25862,7 @@
       </c>
       <c r="J138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K138" t="inlineStr" s="6">
@@ -25609,7 +25872,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -25629,12 +25892,12 @@
       </c>
       <c r="D139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -25644,7 +25907,7 @@
       </c>
       <c r="G139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H139" t="inlineStr" s="2">
@@ -25669,7 +25932,7 @@
       </c>
       <c r="L139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -25694,7 +25957,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -25739,22 +26002,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Manual step</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -25764,12 +26027,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -25779,7 +26042,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -25789,7 +26052,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -25799,22 +26062,22 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Manual step</t>
         </is>
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -25824,12 +26087,12 @@
       </c>
       <c r="G142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="H142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="I142" t="inlineStr" s="2">
@@ -25839,7 +26102,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -25849,7 +26112,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -25859,7 +26122,7 @@
       </c>
       <c r="B143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C143" t="inlineStr" s="2">
@@ -25874,7 +26137,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -25899,7 +26162,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -25909,7 +26172,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -25919,7 +26182,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -25934,7 +26197,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -25959,7 +26222,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -25969,7 +26232,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -25979,7 +26242,7 @@
       </c>
       <c r="B145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C145" t="inlineStr" s="2">
@@ -25994,7 +26257,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -26019,7 +26282,7 @@
       </c>
       <c r="J145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K145" t="inlineStr" s="6">
@@ -26029,7 +26292,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -26039,7 +26302,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -26054,7 +26317,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -26089,7 +26352,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -26099,7 +26362,7 @@
       </c>
       <c r="B147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C147" t="inlineStr" s="2">
@@ -26114,7 +26377,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M12</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -26149,7 +26412,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
         </is>
       </c>
     </row>
@@ -26159,7 +26422,7 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 13</t>
         </is>
       </c>
       <c r="C148" t="inlineStr" s="2">
@@ -26174,7 +26437,7 @@
       </c>
       <c r="E148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M13</t>
         </is>
       </c>
       <c r="F148" t="inlineStr" s="2">
@@ -26209,132 +26472,12 @@
       </c>
       <c r="L148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2">
-        <v>145</v>
-      </c>
-      <c r="B149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 11</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual step</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">M12</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" s="2">
-        <v>146</v>
-      </c>
-      <c r="B150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 13</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual step</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">M13</t>
-        </is>
-      </c>
-      <c r="F150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="H150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="I150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J150" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-      <c r="K150" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-      <c r="L150" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L150"/>
+  <autoFilter ref="A4:L148"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
feat: v1.5.0 Part 5d Bulk push and Yotel push selection lists masked (built locally, not deployed)
Existing (approved, originals in backup/v1.5.0-part5d-pre-change), 3 lines:
- LeadBulkPushController.getSelectedLeads: mobile via PhoneDisplayService.forDisplay
- LeadYotelBulkPushController.getSelectedLeads: same; debug line masked
Push methods unchanged (server reads real numbers).
New: PhoneMaskingPushTest. TEST_GUIDE 5d section, manifests, release bundle
part5d-push, changelog, roadmap, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -22,15 +22,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$108</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$115</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
@@ -329,7 +329,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-5c)</t>
+          <t>Production Release Bundle - built components (Parts 1-5d)</t>
         </is>
       </c>
     </row>
@@ -5823,7 +5823,7 @@
       </c>
       <c r="H103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">95a18c94dfa3</t>
+          <t xml:space="preserve">f277a34f5bbb</t>
         </is>
       </c>
       <c r="I103" t="inlineStr" s="2">
@@ -5958,47 +5958,47 @@
       </c>
       <c r="B106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5d-push</t>
         </is>
       </c>
       <c r="C106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">LeadBulkPushController</t>
         </is>
       </c>
       <c r="G106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part5d-push/classes/LeadBulkPushController.cls</t>
         </is>
       </c>
       <c r="H106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
+          <t xml:space="preserve">4b1c5e77618a</t>
         </is>
       </c>
       <c r="I106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J106" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K106" t="inlineStr" s="6">
@@ -6013,47 +6013,47 @@
       </c>
       <c r="B107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5d-push</t>
         </is>
       </c>
       <c r="C107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">LeadBulkPushController</t>
         </is>
       </c>
       <c r="G107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part5d-push/classes/LeadBulkPushController.cls-meta.xml</t>
         </is>
       </c>
       <c r="H107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">356db6109364</t>
         </is>
       </c>
       <c r="I107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J107" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K107" t="inlineStr" s="6">
@@ -6068,57 +6068,442 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part5d-push</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadYotelBulkPushController</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5d-push/classes/LeadYotelBulkPushController.cls</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">7c576df073ca</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2">
+        <v>8</v>
+      </c>
+      <c r="B109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5d-push</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadYotelBulkPushController</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5d-push/classes/LeadYotelBulkPushController.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">356db6109364</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2">
+        <v>8</v>
+      </c>
+      <c r="B110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5d-push</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingPushTest</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5d-push/classes/PhoneMaskingPushTest.cls</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bfc09077c59f</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K110" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2">
+        <v>8</v>
+      </c>
+      <c r="B111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5d-push</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingPushTest</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5d-push/classes/PhoneMaskingPushTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K111" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2">
+        <v>8</v>
+      </c>
+      <c r="B112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5d-push</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5d)</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5d-push/package.xml</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">d324f6523942</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K112" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2">
+        <v>9</v>
+      </c>
+      <c r="B113" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr" s="2">
+      <c r="C113" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr" s="2">
+      <c r="D113" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr" s="2">
+      <c r="E113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K113" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2">
+        <v>9</v>
+      </c>
+      <c r="B114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2">
+        <v>9</v>
+      </c>
+      <c r="B115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr" s="2">
+      <c r="F115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr" s="2">
+      <c r="G115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr" s="2">
+      <c r="H115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">df1ecd8c7bec</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr" s="2">
+      <c r="I115" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr" s="4">
+      <c r="J115" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr" s="6">
+      <c r="K115" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K108"/>
+  <autoFilter ref="A4:K115"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -6142,7 +6527,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-5c)</t>
+          <t>Production Deploy Steps (Parts 1-5d)</t>
         </is>
       </c>
     </row>
@@ -6391,47 +6776,49 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="2">
-        <v>4</v>
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3g</t>
+        </is>
       </c>
       <c r="B13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part5d-push</t>
         </is>
       </c>
       <c r="C13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5d-push --test-level RunSpecifiedTests --tests PhoneMaskingPushTest --tests LeadBulkPushControllerTest --tests LeadYotelBulkPushControllerTest</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E14" t="inlineStr" s="6">
@@ -6442,31 +6829,56 @@
     </row>
     <row r="15">
       <c r="A15" s="2">
+        <v>5</v>
+      </c>
+      <c r="B15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2">
         <v>6</v>
       </c>
-      <c r="B15" t="inlineStr" s="2">
+      <c r="B16" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr" s="2">
+      <c r="C16" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr" s="2">
+      <c r="D16" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr" s="6">
+      <c r="E16" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E15"/>
+  <autoFilter ref="A4:E16"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -8288,12 +8700,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a-5c deployed, call panels deferred D1)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) - 5a, 5b, 5c</t>
+          <t xml:space="preserve">Mask leaking screens (5a-5c deployed, 5d built, call panels deferred D1)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5d</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -14266,8 +14678,68 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" s="2">
+        <v>94</v>
+      </c>
+      <c r="B98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingPushTest</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5d: selection lists masked for masked users; eligibility unchanged</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5d</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L97"/>
+  <autoFilter ref="A4:L98"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -16027,7 +16499,7 @@
       </c>
       <c r="H32" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-07</t>
         </is>
       </c>
       <c r="I32" t="inlineStr" s="2">
@@ -16035,9 +16507,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J32" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5d</t>
         </is>
       </c>
       <c r="K32" t="inlineStr" s="2">
@@ -16147,7 +16619,7 @@
       </c>
       <c r="H34" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-07</t>
         </is>
       </c>
       <c r="I34" t="inlineStr" s="2">
@@ -16155,9 +16627,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J34" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - 5d</t>
         </is>
       </c>
       <c r="K34" t="inlineStr" s="2">
@@ -22832,7 +23304,7 @@
       </c>
       <c r="D88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (update of new)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E88" t="inlineStr" s="2">
@@ -22857,7 +23329,7 @@
       </c>
       <c r="I88" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+          <t xml:space="preserve">PhoneDisplayServiceTest</t>
         </is>
       </c>
       <c r="J88" t="inlineStr" s="2">
@@ -22892,7 +23364,7 @@
       </c>
       <c r="D89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (update of new)</t>
         </is>
       </c>
       <c r="E89" t="inlineStr" s="2">
@@ -22917,7 +23389,7 @@
       </c>
       <c r="I89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneDisplayServiceTest</t>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="J89" t="inlineStr" s="2">
@@ -23252,12 +23724,12 @@
       </c>
       <c r="D95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">PhoneMaskingPushTest</t>
         </is>
       </c>
       <c r="F95" t="inlineStr" s="2">
@@ -23267,7 +23739,7 @@
       </c>
       <c r="G95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H95" t="inlineStr" s="2">
@@ -23292,7 +23764,7 @@
       </c>
       <c r="L95" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23317,7 +23789,7 @@
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -23377,7 +23849,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -23412,7 +23884,7 @@
       </c>
       <c r="L97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -23432,12 +23904,12 @@
       </c>
       <c r="D98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -23472,7 +23944,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -23492,12 +23964,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -23507,7 +23979,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -23522,7 +23994,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -23532,7 +24004,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Masked numbers in chat</t>
         </is>
       </c>
     </row>
@@ -23542,27 +24014,27 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
@@ -23582,7 +24054,7 @@
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="6">
@@ -23612,17 +24084,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -23672,12 +24144,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -23697,7 +24169,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -23712,7 +24184,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -23737,7 +24209,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -23757,7 +24229,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -23772,7 +24244,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -23792,12 +24264,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -23817,7 +24289,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -23857,7 +24329,7 @@
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -23912,12 +24384,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -23972,12 +24444,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -24022,22 +24494,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -24057,7 +24529,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -24072,7 +24544,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24092,34 +24564,34 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FreeTextMaskService</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J109" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
@@ -24132,7 +24604,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -24152,12 +24624,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -24167,7 +24639,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -24192,7 +24664,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24217,17 +24689,17 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -24237,7 +24709,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -24252,7 +24724,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -24272,22 +24744,22 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -24297,7 +24769,7 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
@@ -24312,7 +24784,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24332,12 +24804,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -24382,22 +24854,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -24407,7 +24879,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -24417,12 +24889,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -24432,7 +24904,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -24452,32 +24924,32 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FindByNumberController</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FindByNumberControllerTest</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -24512,12 +24984,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -24537,7 +25009,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -24552,7 +25024,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24577,7 +25049,7 @@
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -24587,7 +25059,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -24597,7 +25069,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -24612,7 +25084,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -24622,22 +25094,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -24672,7 +25144,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -24692,12 +25164,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -24732,7 +25204,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -24757,7 +25229,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -24812,12 +25284,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -24852,7 +25324,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -24877,7 +25349,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -24912,7 +25384,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -24937,7 +25409,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -24972,7 +25444,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -24997,7 +25469,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -25057,7 +25529,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -25112,12 +25584,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -25152,7 +25624,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -25162,22 +25634,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -25202,7 +25674,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -25212,7 +25684,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -25237,7 +25709,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -25297,7 +25769,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -25332,7 +25804,7 @@
       </c>
       <c r="L129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -25392,7 +25864,7 @@
       </c>
       <c r="L130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -25417,7 +25889,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -25452,7 +25924,7 @@
       </c>
       <c r="L131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -25537,7 +26009,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -25572,7 +26044,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -25592,12 +26064,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -25607,7 +26079,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -25632,7 +26104,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -25652,12 +26124,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -25667,12 +26139,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -25692,7 +26164,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -25712,12 +26184,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -25742,7 +26214,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -25752,7 +26224,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -25762,22 +26234,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -25787,12 +26259,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -25802,7 +26274,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -25812,7 +26284,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -25832,12 +26304,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -25847,7 +26319,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -25872,7 +26344,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -25897,7 +26369,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -25957,7 +26429,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -26002,22 +26474,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -26027,12 +26499,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -26042,7 +26514,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -26052,7 +26524,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -26062,7 +26534,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -26077,7 +26549,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -26102,7 +26574,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -26112,7 +26584,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -26137,7 +26609,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -26162,7 +26634,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -26172,7 +26644,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -26182,7 +26654,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -26197,7 +26669,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -26222,7 +26694,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -26232,7 +26704,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -26257,7 +26729,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -26292,7 +26764,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -26302,7 +26774,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -26317,7 +26789,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -26352,7 +26824,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -26377,7 +26849,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -26412,7 +26884,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -26422,62 +26894,122 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2">
+        <v>145</v>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr" s="2">
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr" s="2">
+      <c r="E149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr" s="2">
+      <c r="F149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr" s="2">
+      <c r="H149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr" s="2">
+      <c r="I149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr" s="6">
+      <c r="K149" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr" s="2">
+      <c r="L149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L148"/>
+  <autoFilter ref="A4:L149"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
deploy: Part 5d to sandbox; tracking updated
0Afft000000Lm1dCAC: 3/3, 10 tests passed (incl. existing LeadBulkPushControllerTest,
LeadYotelBulkPushControllerTest). Coverage 98.5% / 95.8%. PhoneMaskingPushTest
corrected for the existing Test.isRunningTest() swap in the Yotel controller.
Testing on hold (owner access issue, D2).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -5996,9 +5996,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J106" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J106" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K106" t="inlineStr" s="6">
@@ -6051,9 +6051,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J107" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J107" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K107" t="inlineStr" s="6">
@@ -6106,9 +6106,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J108" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K108" t="inlineStr" s="6">
@@ -6161,9 +6161,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J109" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J109" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K109" t="inlineStr" s="6">
@@ -6216,9 +6216,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J110" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J110" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K110" t="inlineStr" s="6">
@@ -6271,9 +6271,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J111" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K111" t="inlineStr" s="6">
@@ -6326,9 +6326,9 @@
           <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
-      <c r="J112" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J112" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K112" t="inlineStr" s="6">
@@ -8700,12 +8700,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a-5c deployed, 5d built, call panels deferred D1)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5d</t>
+          <t xml:space="preserve">Mask leaking screens (5a-5d deployed, call panels deferred D1)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) - 5a to 5d</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -14717,14 +14717,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I98" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5d</t>
+      <c r="I98" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K98" t="inlineStr" s="2">
@@ -16507,9 +16507,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
         </is>
       </c>
-      <c r="J32" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5d</t>
+      <c r="J32" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K32" t="inlineStr" s="2">
@@ -16627,9 +16627,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5d-pre-change</t>
         </is>
       </c>
-      <c r="J34" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - 5d</t>
+      <c r="J34" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lm1dCAC</t>
         </is>
       </c>
       <c r="K34" t="inlineStr" s="2">

</xml_diff>

<commit_message>
backup + plan: Part 5e (WhatsApp chat); roadmap D4 (Messaging objects)
Backup of LeadMsgConversationController (+test) and leadMsgConversationLWC -
read-only, identical to baseline. Plan sheet in the register. D4: reps have
View All on MessagingEndUser / MessagingSession - go-live decision.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -18,13 +18,14 @@
     <sheet name="Part 5b Plan" sheetId="14" r:id="rId14"/>
     <sheet name="Part 5c Plan" sheetId="15" r:id="rId15"/>
     <sheet name="Part 5d Plan" sheetId="16" r:id="rId16"/>
+    <sheet name="Part 5e Plan" sheetId="17" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$98</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
@@ -36,6 +37,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Part 5c Plan'!$A$4:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Part 5d Plan'!$A$4:$F$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Part 5e Plan'!$A$4:$F$11</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -6208,7 +6210,7 @@
       </c>
       <c r="H110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">bfc09077c59f</t>
+          <t xml:space="preserve">154004ee2ed5</t>
         </is>
       </c>
       <c r="I110" t="inlineStr" s="2">
@@ -8472,6 +8474,299 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:F10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="48" customWidth="1"/>
+    <col min="4" max="4" width="84" customWidth="1"/>
+    <col min="5" max="5" width="54" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 5e (v1.5.0) - WhatsApp chat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; originals in backup/v1.5.0-part5e-pre-change</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LeadMsgConversationController.getConversationViaConnectApi</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Before returning the conversation: for masked users, mask numbers inside message, rawJson and senderName (PhoneMaskUtil.maskInText) - one call to a new @TestVisible helper</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Masked users: chat shows the same messages with any phone number masked; the raw data never carries the WhatsApp number. Others: unchanged</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">getMessagingSessionId, getTransferContext, transferMessagingSession, getSessionAttachments</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Use Full_phone_number__c on the server only; return Ids, status, files - no number</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LWC</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">leadMsgConversationLWC</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Displays what Apex returns</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingWhatsAppTest</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Conversation rows masked for masked users, unchanged for others (Connect API not called - helper tested directly)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Go-live decision (D4)</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Standard objects</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MessagingEndUser / MessagingSession</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Presales outbound has View All on both; the WhatsApp customer record shows the number in standard screens, reports, search. Needs a go-live decision (remove View All / restrict) without breaking chat for reps</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Not changed in 5e</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Decision</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Later (Part 7)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">notifyLeadStakeholders(messagePreview)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Preview text typed in chat - free-text masking</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Test limit</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Data</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sandbox has 0 MessagingEndUser records</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">The chat cannot be tested on screen in the sandbox (no WhatsApp data copied)</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F11"/>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
     <mergeCell ref="A2:F2"/>
@@ -16669,7 +16964,7 @@
       </c>
       <c r="F35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve">5e: NO CHANGE - shows what Apex returns</t>
         </is>
       </c>
       <c r="G35" t="inlineStr" s="2">
@@ -16679,22 +16974,22 @@
       </c>
       <c r="H35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">-</t>
         </is>
       </c>
       <c r="I35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+          <t xml:space="preserve">backup/v1.5.0-part5e-pre-change</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change (5e)</t>
         </is>
       </c>
       <c r="K35" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">No</t>
         </is>
       </c>
       <c r="L35" t="inlineStr" s="2">
@@ -16729,7 +17024,7 @@
       </c>
       <c r="F36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Resolve number server-side for send</t>
+          <t xml:space="preserve">5e: mask numbers in conversation message / rawJson / senderName for masked users</t>
         </is>
       </c>
       <c r="G36" t="inlineStr" s="2">
@@ -16739,12 +17034,12 @@
       </c>
       <c r="H36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Not requested yet</t>
+          <t xml:space="preserve">Pending approval</t>
         </is>
       </c>
       <c r="I36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Baseline v1.0.0</t>
+          <t xml:space="preserve">backup/v1.5.0-part5e-pre-change</t>
         </is>
       </c>
       <c r="J36" t="inlineStr" s="6">
@@ -22924,7 +23219,7 @@
       </c>
       <c r="L81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Resolve number server-side for send</t>
+          <t xml:space="preserve">5e: mask numbers in conversation message / rawJson / senderName for masked users</t>
         </is>
       </c>
     </row>
@@ -23269,7 +23564,7 @@
       </c>
       <c r="I87" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
+          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
         </is>
       </c>
       <c r="J87" t="inlineStr" s="2">
@@ -23389,7 +23684,7 @@
       </c>
       <c r="I89" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneMaskingHistoryTest</t>
+          <t xml:space="preserve">PhoneMaskingLeadToolsTest</t>
         </is>
       </c>
       <c r="J89" t="inlineStr" s="2">
@@ -23964,12 +24259,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">leadMsgConversationLWC</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -23979,7 +24274,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -23994,7 +24289,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -24004,7 +24299,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked numbers in chat</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24014,27 +24309,27 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 5</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.5.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
@@ -24054,7 +24349,7 @@
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="6">
@@ -24084,17 +24379,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -24144,12 +24439,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -24169,7 +24464,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -24184,7 +24479,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -24209,7 +24504,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -24229,7 +24524,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -24244,7 +24539,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24264,12 +24559,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -24289,7 +24584,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -24329,7 +24624,7 @@
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -24384,12 +24679,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -24444,12 +24739,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -24494,22 +24789,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">FreeTextMaskService</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -24529,7 +24824,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -24544,7 +24839,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -24564,12 +24859,12 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F109" t="inlineStr" s="2">
@@ -24589,7 +24884,7 @@
       </c>
       <c r="I109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J109" t="inlineStr" s="2">
@@ -24604,7 +24899,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24624,12 +24919,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -24639,7 +24934,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -24664,7 +24959,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -24689,17 +24984,17 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -24709,7 +25004,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -24724,7 +25019,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24744,22 +25039,22 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -24769,7 +25064,7 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
@@ -24784,7 +25079,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -24804,12 +25099,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -24854,22 +25149,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">FindByNumberController</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -24879,7 +25174,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -24889,12 +25184,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -24904,7 +25199,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24924,12 +25219,12 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F115" t="inlineStr" s="2">
@@ -24949,7 +25244,7 @@
       </c>
       <c r="I115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -24984,12 +25279,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -25009,7 +25304,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -25024,7 +25319,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -25049,7 +25344,7 @@
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -25059,7 +25354,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -25069,7 +25364,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -25084,7 +25379,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -25094,22 +25389,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -25144,7 +25439,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -25164,12 +25459,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -25204,7 +25499,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -25229,7 +25524,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -25284,12 +25579,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -25324,7 +25619,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -25349,7 +25644,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -25384,7 +25679,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -25409,7 +25704,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -25444,7 +25739,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -25469,7 +25764,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -25529,7 +25824,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -25584,12 +25879,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -25624,7 +25919,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -25634,22 +25929,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -25674,7 +25969,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -25684,7 +25979,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -25709,7 +26004,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -25769,7 +26064,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -25804,7 +26099,7 @@
       </c>
       <c r="L129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -25864,7 +26159,7 @@
       </c>
       <c r="L130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -25889,7 +26184,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -25924,7 +26219,7 @@
       </c>
       <c r="L131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -26009,7 +26304,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -26044,7 +26339,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -26064,12 +26359,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -26079,7 +26374,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -26104,7 +26399,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -26124,12 +26419,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -26139,12 +26434,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -26164,7 +26459,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -26184,12 +26479,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -26214,7 +26509,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -26224,7 +26519,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -26234,22 +26529,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -26259,12 +26554,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -26274,7 +26569,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -26284,7 +26579,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -26304,12 +26599,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -26319,7 +26614,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -26344,7 +26639,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -26369,7 +26664,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -26429,7 +26724,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -26474,22 +26769,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Manual step</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -26499,12 +26794,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -26514,7 +26809,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -26524,7 +26819,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -26534,7 +26829,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -26549,7 +26844,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -26574,7 +26869,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -26584,7 +26879,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -26609,7 +26904,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -26634,7 +26929,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -26644,7 +26939,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -26654,7 +26949,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -26669,7 +26964,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -26694,7 +26989,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -26704,7 +26999,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -26729,7 +27024,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -26764,7 +27059,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -26774,7 +27069,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -26789,7 +27084,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -26824,7 +27119,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -26849,7 +27144,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M12</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -26884,7 +27179,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
         </is>
       </c>
     </row>
@@ -26894,7 +27189,7 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 13</t>
         </is>
       </c>
       <c r="C148" t="inlineStr" s="2">
@@ -26909,7 +27204,7 @@
       </c>
       <c r="E148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M13</t>
         </is>
       </c>
       <c r="F148" t="inlineStr" s="2">
@@ -26944,72 +27239,12 @@
       </c>
       <c r="L148" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" s="2">
-        <v>145</v>
-      </c>
-      <c r="B149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Part 13</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual step</t>
-        </is>
-      </c>
-      <c r="E149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">M13</t>
-        </is>
-      </c>
-      <c r="F149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="H149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Manual</t>
-        </is>
-      </c>
-      <c r="I149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J149" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Yes</t>
-        </is>
-      </c>
-      <c r="K149" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
-        </is>
-      </c>
-      <c r="L149" t="inlineStr" s="2">
-        <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L149"/>
+  <autoFilter ref="A4:L148"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
fix: register and release README - add the 5e entries missed at build time
Part 5e approval / deploy status, PhoneMaskingWhatsAppTest row, part5e-whatsapp
release bundle row and production step, Part 5 summary (5a-5e deployed),
release README section.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -23,15 +23,15 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Summary'!$A$4:$H$17</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'New Components'!$A$4:$L$99</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Existing Components'!$A$4:$L$60</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$148</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prod Deployment List'!$A$4:$L$149</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Manual Steps'!$A$4:$F$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$115</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$120</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
@@ -331,7 +331,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-5d)</t>
+          <t>Production Release Bundle - built components (Parts 1-5e)</t>
         </is>
       </c>
     </row>
@@ -6345,47 +6345,47 @@
       </c>
       <c r="B113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5e-whatsapp</t>
         </is>
       </c>
       <c r="C113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5e)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">LeadMsgConversationController</t>
         </is>
       </c>
       <c r="G113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part5e-whatsapp/classes/LeadMsgConversationController.cls</t>
         </is>
       </c>
       <c r="H113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
+          <t xml:space="preserve">3daaca35c849</t>
         </is>
       </c>
       <c r="I113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+          <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
       <c r="J113" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lmb7CAC</t>
         </is>
       </c>
       <c r="K113" t="inlineStr" s="6">
@@ -6400,47 +6400,47 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part5e-whatsapp</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.5.0 (5e)</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">LeadMsgConversationController</t>
         </is>
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part5e-whatsapp/classes/LeadMsgConversationController.cls-meta.xml</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">87b91a7450c6</t>
         </is>
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+          <t xml:space="preserve">Production - everyone</t>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lmb7CAC</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -6455,57 +6455,332 @@
       </c>
       <c r="B115" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part5e-whatsapp</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5e)</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingWhatsAppTest</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5e-whatsapp/classes/PhoneMaskingWhatsAppTest.cls</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3b2f4590a8cd</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lmb7CAC</t>
+        </is>
+      </c>
+      <c r="K115" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2">
+        <v>9</v>
+      </c>
+      <c r="B116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5e-whatsapp</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5e)</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingWhatsAppTest</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5e-whatsapp/classes/PhoneMaskingWhatsAppTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lmb7CAC</t>
+        </is>
+      </c>
+      <c r="K116" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2">
+        <v>9</v>
+      </c>
+      <c r="B117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part5e-whatsapp</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0 (5e)</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part5e-whatsapp/package.xml</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">d4e79f7ed133</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lmb7CAC</t>
+        </is>
+      </c>
+      <c r="K117" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2">
+        <v>10</v>
+      </c>
+      <c r="B118" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr" s="2">
+      <c r="C118" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr" s="2">
+      <c r="D118" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr" s="2">
+      <c r="E118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I118" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K118" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2">
+        <v>10</v>
+      </c>
+      <c r="B119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I119" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K119" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2">
+        <v>10</v>
+      </c>
+      <c r="B120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F115" t="inlineStr" s="2">
+      <c r="F120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G115" t="inlineStr" s="2">
+      <c r="G120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr" s="2">
+      <c r="H120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">df1ecd8c7bec</t>
         </is>
       </c>
-      <c r="I115" t="inlineStr" s="2">
+      <c r="I120" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J115" t="inlineStr" s="4">
+      <c r="J120" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K115" t="inlineStr" s="6">
+      <c r="K120" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K115"/>
+  <autoFilter ref="A4:K120"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -6529,7 +6804,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-5d)</t>
+          <t>Production Deploy Steps (Parts 1-5e)</t>
         </is>
       </c>
     </row>
@@ -6805,47 +7080,49 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2">
-        <v>4</v>
+      <c r="A14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3h</t>
+        </is>
       </c>
       <c r="B14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part5e-whatsapp</t>
         </is>
       </c>
       <c r="C14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part5e-whatsapp --test-level RunSpecifiedTests --tests PhoneMaskingWhatsAppTest --tests LeadMsgConversationControllerTest</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E15" t="inlineStr" s="6">
@@ -6856,31 +7133,56 @@
     </row>
     <row r="16">
       <c r="A16" s="2">
+        <v>5</v>
+      </c>
+      <c r="B16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2">
         <v>6</v>
       </c>
-      <c r="B16" t="inlineStr" s="2">
+      <c r="B17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr" s="2">
+      <c r="C17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr" s="2">
+      <c r="D17" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr" s="6">
+      <c r="E17" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E16"/>
+  <autoFilter ref="A4:E17"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -8995,12 +9297,12 @@
       </c>
       <c r="C9" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Mask leaking screens (5a-5d deployed, call panels deferred D1)</t>
+          <t xml:space="preserve">Mask leaking screens (5a-5e deployed, call panels deferred D1)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">Deployed (Sandbox) - 5a to 5d</t>
+          <t xml:space="preserve">Deployed (Sandbox) - 5a to 5e</t>
         </is>
       </c>
       <c r="E9" s="2">
@@ -15033,8 +15335,68 @@
         </is>
       </c>
     </row>
+    <row r="99">
+      <c r="A99" s="2">
+        <v>95</v>
+      </c>
+      <c r="B99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 5</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.5.0</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneMaskingWhatsAppTest</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">5e: conversation masked for masked users, unchanged for others</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">0Afft000000Lmb7CAC</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A4:L98"/>
+  <autoFilter ref="A4:L99"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
@@ -17034,7 +17396,7 @@
       </c>
       <c r="H36" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pending approval</t>
+          <t xml:space="preserve">Approved 2026-10-07</t>
         </is>
       </c>
       <c r="I36" t="inlineStr" s="2">
@@ -17042,9 +17404,9 @@
           <t xml:space="preserve">backup/v1.5.0-part5e-pre-change</t>
         </is>
       </c>
-      <c r="J36" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="J36" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000Lmb7CAC</t>
         </is>
       </c>
       <c r="K36" t="inlineStr" s="2">
@@ -24079,12 +24441,12 @@
       </c>
       <c r="D96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel</t>
+          <t xml:space="preserve">PhoneMaskingWhatsAppTest</t>
         </is>
       </c>
       <c r="F96" t="inlineStr" s="2">
@@ -24094,7 +24456,7 @@
       </c>
       <c r="G96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H96" t="inlineStr" s="2">
@@ -24119,7 +24481,7 @@
       </c>
       <c r="L96" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24144,7 +24506,7 @@
       </c>
       <c r="E97" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallPanel_Outbound</t>
+          <t xml:space="preserve">CallPanel</t>
         </is>
       </c>
       <c r="F97" t="inlineStr" s="2">
@@ -24204,7 +24566,7 @@
       </c>
       <c r="E98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">UpdateContactDetails</t>
+          <t xml:space="preserve">CallPanel_Outbound</t>
         </is>
       </c>
       <c r="F98" t="inlineStr" s="2">
@@ -24239,7 +24601,7 @@
       </c>
       <c r="L98" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
+          <t xml:space="preserve">Postponed: the Aura view form has no onload event. Proposed: replace the Phone line with a new LWC maskedPhoneField</t>
         </is>
       </c>
     </row>
@@ -24259,12 +24621,12 @@
       </c>
       <c r="D99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile (update of new)</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">POC Masked Rep</t>
+          <t xml:space="preserve">UpdateContactDetails</t>
         </is>
       </c>
       <c r="F99" t="inlineStr" s="2">
@@ -24274,7 +24636,7 @@
       </c>
       <c r="G99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H99" t="inlineStr" s="2">
@@ -24289,7 +24651,7 @@
       </c>
       <c r="J99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K99" t="inlineStr" s="6">
@@ -24299,7 +24661,7 @@
       </c>
       <c r="L99" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Primary read-only masked; secondary masked entry</t>
         </is>
       </c>
     </row>
@@ -24309,27 +24671,27 @@
       </c>
       <c r="B100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 5</t>
         </is>
       </c>
       <c r="C100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.6.0</t>
+          <t xml:space="preserve">v1.5.0</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Field</t>
+          <t xml:space="preserve">Profile (update of new)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
       <c r="F100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Access_Audit__c</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G100" t="inlineStr" s="2">
@@ -24349,7 +24711,7 @@
       </c>
       <c r="J100" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K100" t="inlineStr" s="6">
@@ -24379,17 +24741,17 @@
       </c>
       <c r="D101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Custom Permission</t>
+          <t xml:space="preserve">Custom Field</t>
         </is>
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Phone_Number</t>
+          <t xml:space="preserve">Reveal_Reason__c</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
         </is>
       </c>
       <c r="G101" t="inlineStr" s="2">
@@ -24439,12 +24801,12 @@
       </c>
       <c r="D102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Custom Permission</t>
         </is>
       </c>
       <c r="E102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
         </is>
       </c>
       <c r="F102" t="inlineStr" s="2">
@@ -24464,7 +24826,7 @@
       </c>
       <c r="I102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J102" t="inlineStr" s="2">
@@ -24479,7 +24841,7 @@
       </c>
       <c r="L102" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule after deploy</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24504,7 +24866,7 @@
       </c>
       <c r="E103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealService</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
         </is>
       </c>
       <c r="F103" t="inlineStr" s="2">
@@ -24524,7 +24886,7 @@
       </c>
       <c r="I103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="J103" t="inlineStr" s="2">
@@ -24539,7 +24901,7 @@
       </c>
       <c r="L103" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Schedule after deploy</t>
         </is>
       </c>
     </row>
@@ -24559,12 +24921,12 @@
       </c>
       <c r="D104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+          <t xml:space="preserve">PhoneRevealService</t>
         </is>
       </c>
       <c r="F104" t="inlineStr" s="2">
@@ -24584,7 +24946,7 @@
       </c>
       <c r="I104" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="J104" t="inlineStr" s="2">
@@ -24624,7 +24986,7 @@
       </c>
       <c r="E105" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">PhoneRevealServiceTest</t>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
       <c r="F105" t="inlineStr" s="2">
@@ -24679,12 +25041,12 @@
       </c>
       <c r="D106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component (update)</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E106" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">maskedPhonePanel</t>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
       <c r="F106" t="inlineStr" s="2">
@@ -24739,12 +25101,12 @@
       </c>
       <c r="D107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Web Component (update)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">maskedPhonePanel</t>
         </is>
       </c>
       <c r="F107" t="inlineStr" s="2">
@@ -24789,22 +25151,22 @@
       </c>
       <c r="B108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 7</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.7.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskService</t>
+          <t xml:space="preserve">Phone_Number_Reveal</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">
@@ -24824,7 +25186,7 @@
       </c>
       <c r="I108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J108" t="inlineStr" s="2">
@@ -24839,7 +25201,7 @@
       </c>
       <c r="L108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permanent masking</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24859,34 +25221,34 @@
       </c>
       <c r="D109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E109" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FreeTextMaskService</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
-      <c r="F109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
       <c r="J109" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
@@ -24899,7 +25261,7 @@
       </c>
       <c r="L109" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Permanent masking</t>
         </is>
       </c>
     </row>
@@ -24919,12 +25281,12 @@
       </c>
       <c r="D110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">CallDetailTrigger</t>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="F110" t="inlineStr" s="2">
@@ -24934,7 +25296,7 @@
       </c>
       <c r="G110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H110" t="inlineStr" s="2">
@@ -24959,7 +25321,7 @@
       </c>
       <c r="L110" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -24984,17 +25346,17 @@
       </c>
       <c r="E111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
+          <t xml:space="preserve">CallDetailTrigger</t>
         </is>
       </c>
       <c r="F111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FeedItem</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="G111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H111" t="inlineStr" s="2">
@@ -25004,7 +25366,7 @@
       </c>
       <c r="I111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FreeTextMaskServiceTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J111" t="inlineStr" s="2">
@@ -25019,7 +25381,7 @@
       </c>
       <c r="L111" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save (free-text fields only)</t>
         </is>
       </c>
     </row>
@@ -25039,22 +25401,22 @@
       </c>
       <c r="D112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger / Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
+          <t xml:space="preserve">FeedItemPhoneMaskTrigger</t>
         </is>
       </c>
       <c r="F112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FeedItem</t>
         </is>
       </c>
       <c r="G112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H112" t="inlineStr" s="2">
@@ -25064,7 +25426,7 @@
       </c>
       <c r="I112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">FreeTextMaskServiceTest</t>
         </is>
       </c>
       <c r="J112" t="inlineStr" s="2">
@@ -25079,7 +25441,7 @@
       </c>
       <c r="L112" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Call FreeTextMaskService on save</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -25099,12 +25461,12 @@
       </c>
       <c r="D113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Trigger</t>
+          <t xml:space="preserve">Apex Trigger / Class</t>
         </is>
       </c>
       <c r="E113" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">TaskTrigger</t>
+          <t xml:space="preserve">Opportunity + feedback object triggers (TBD)</t>
         </is>
       </c>
       <c r="F113" t="inlineStr" s="2">
@@ -25149,22 +25511,22 @@
       </c>
       <c r="B114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 8</t>
+          <t xml:space="preserve">Part 7</t>
         </is>
       </c>
       <c r="C114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.8.0</t>
+          <t xml:space="preserve">v1.7.0</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Apex Trigger</t>
         </is>
       </c>
       <c r="E114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberController</t>
+          <t xml:space="preserve">TaskTrigger</t>
         </is>
       </c>
       <c r="F114" t="inlineStr" s="2">
@@ -25174,7 +25536,7 @@
       </c>
       <c r="G114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H114" t="inlineStr" s="2">
@@ -25184,12 +25546,12 @@
       </c>
       <c r="I114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">FindByNumberControllerTest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Conditional</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K114" t="inlineStr" s="6">
@@ -25199,7 +25561,7 @@
       </c>
       <c r="L114" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Call FreeTextMaskService on save</t>
         </is>
       </c>
     </row>
@@ -25219,32 +25581,32 @@
       </c>
       <c r="D115" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class (test)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E115" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">FindByNumberController</t>
+        </is>
+      </c>
+      <c r="F115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Change set</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">FindByNumberControllerTest</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">New</t>
-        </is>
-      </c>
-      <c r="H115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve">Change set</t>
-        </is>
-      </c>
-      <c r="I115" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J115" t="inlineStr" s="2">
@@ -25279,12 +25641,12 @@
       </c>
       <c r="D116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Apex Class (test)</t>
         </is>
       </c>
       <c r="E116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">findByNumber</t>
+          <t xml:space="preserve">FindByNumberControllerTest</t>
         </is>
       </c>
       <c r="F116" t="inlineStr" s="2">
@@ -25304,7 +25666,7 @@
       </c>
       <c r="I116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Jest</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="J116" t="inlineStr" s="2">
@@ -25319,7 +25681,7 @@
       </c>
       <c r="L116" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Only if POC shows global search breaks</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
     </row>
@@ -25344,7 +25706,7 @@
       </c>
       <c r="E117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">searchComponent</t>
+          <t xml:space="preserve">findByNumber</t>
         </is>
       </c>
       <c r="F117" t="inlineStr" s="2">
@@ -25354,7 +25716,7 @@
       </c>
       <c r="G117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H117" t="inlineStr" s="2">
@@ -25364,7 +25726,7 @@
       </c>
       <c r="I117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">Jest</t>
         </is>
       </c>
       <c r="J117" t="inlineStr" s="2">
@@ -25379,7 +25741,7 @@
       </c>
       <c r="L117" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Possibly reuse for Find by number</t>
+          <t xml:space="preserve">Only if POC shows global search breaks</t>
         </is>
       </c>
     </row>
@@ -25389,22 +25751,22 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 9</t>
+          <t xml:space="preserve">Part 8</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.9.0</t>
+          <t xml:space="preserve">v1.8.0</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Visualforce Page</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
+          <t xml:space="preserve">searchComponent</t>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
@@ -25439,7 +25801,7 @@
       </c>
       <c r="L118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Keep real number for document teams</t>
+          <t xml:space="preserve">Possibly reuse for Find by number</t>
         </is>
       </c>
     </row>
@@ -25459,12 +25821,12 @@
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Aura Component</t>
+          <t xml:space="preserve">Visualforce Page</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">createBookingCmp</t>
+          <t xml:space="preserve">19 customer document pages (BookingForm, letters, quotations, receipts)</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
@@ -25499,7 +25861,7 @@
       </c>
       <c r="L119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Keep real number for document teams</t>
         </is>
       </c>
     </row>
@@ -25524,7 +25886,7 @@
       </c>
       <c r="E120" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">siteVisitFeedbackForm</t>
+          <t xml:space="preserve">createBookingCmp</t>
         </is>
       </c>
       <c r="F120" t="inlineStr" s="2">
@@ -25579,12 +25941,12 @@
       </c>
       <c r="D121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Web Component</t>
+          <t xml:space="preserve">Aura Component</t>
         </is>
       </c>
       <c r="E121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">cancellationRequest</t>
+          <t xml:space="preserve">siteVisitFeedbackForm</t>
         </is>
       </c>
       <c r="F121" t="inlineStr" s="2">
@@ -25619,7 +25981,7 @@
       </c>
       <c r="L121" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -25644,7 +26006,7 @@
       </c>
       <c r="E122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">kycAndQuotationTabComponent</t>
+          <t xml:space="preserve">cancellationRequest</t>
         </is>
       </c>
       <c r="F122" t="inlineStr" s="2">
@@ -25679,7 +26041,7 @@
       </c>
       <c r="L122" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked co-applicant entry</t>
+          <t xml:space="preserve">Fails completely if Opportunity Mobile__c is hidden</t>
         </is>
       </c>
     </row>
@@ -25704,7 +26066,7 @@
       </c>
       <c r="E123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">opportunitySummaryLWC</t>
+          <t xml:space="preserve">kycAndQuotationTabComponent</t>
         </is>
       </c>
       <c r="F123" t="inlineStr" s="2">
@@ -25739,7 +26101,7 @@
       </c>
       <c r="L123" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked display</t>
+          <t xml:space="preserve">Masked co-applicant entry</t>
         </is>
       </c>
     </row>
@@ -25764,7 +26126,7 @@
       </c>
       <c r="E124" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">registrationTeamFileUpload</t>
+          <t xml:space="preserve">opportunitySummaryLWC</t>
         </is>
       </c>
       <c r="F124" t="inlineStr" s="2">
@@ -25824,7 +26186,7 @@
       </c>
       <c r="E125" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">showConvertedOppRecord</t>
+          <t xml:space="preserve">registrationTeamFileUpload</t>
         </is>
       </c>
       <c r="F125" t="inlineStr" s="2">
@@ -25879,12 +26241,12 @@
       </c>
       <c r="D126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Quick Action</t>
+          <t xml:space="preserve">Lightning Web Component</t>
         </is>
       </c>
       <c r="E126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
+          <t xml:space="preserve">showConvertedOppRecord</t>
         </is>
       </c>
       <c r="F126" t="inlineStr" s="2">
@@ -25919,7 +26281,7 @@
       </c>
       <c r="L126" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Masked entry</t>
+          <t xml:space="preserve">Masked display</t>
         </is>
       </c>
     </row>
@@ -25929,22 +26291,22 @@
       </c>
       <c r="B127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 9</t>
         </is>
       </c>
       <c r="C127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v2.0.0</t>
+          <t xml:space="preserve">v1.9.0</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve">Quick Action</t>
         </is>
       </c>
       <c r="E127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page</t>
+          <t xml:space="preserve">Contact.Co_Applicant_1 / 2 / 3, Contact.Update_Contact_Details</t>
         </is>
       </c>
       <c r="F127" t="inlineStr" s="2">
@@ -25969,7 +26331,7 @@
       </c>
       <c r="J127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Conditional</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -25979,7 +26341,7 @@
       </c>
       <c r="L127" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Masked entry</t>
         </is>
       </c>
     </row>
@@ -26004,7 +26366,7 @@
       </c>
       <c r="E128" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lead_Record_Page3</t>
+          <t xml:space="preserve">Lead_Record_Page</t>
         </is>
       </c>
       <c r="F128" t="inlineStr" s="2">
@@ -26064,7 +26426,7 @@
       </c>
       <c r="E129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page</t>
+          <t xml:space="preserve">Lead_Record_Page3</t>
         </is>
       </c>
       <c r="F129" t="inlineStr" s="2">
@@ -26099,7 +26461,7 @@
       </c>
       <c r="L129" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -26159,7 +26521,7 @@
       </c>
       <c r="L130" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -26184,7 +26546,7 @@
       </c>
       <c r="E131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New_Lead_Page1_sales</t>
+          <t xml:space="preserve">New_Lead_Page</t>
         </is>
       </c>
       <c r="F131" t="inlineStr" s="2">
@@ -26219,7 +26581,7 @@
       </c>
       <c r="L131" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Swap phone fields for entry fields</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -26304,7 +26666,7 @@
       </c>
       <c r="E133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page</t>
+          <t xml:space="preserve">New_Lead_Page1_sales</t>
         </is>
       </c>
       <c r="F133" t="inlineStr" s="2">
@@ -26339,7 +26701,7 @@
       </c>
       <c r="L133" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
+          <t xml:space="preserve">Swap phone fields for entry fields</t>
         </is>
       </c>
     </row>
@@ -26359,12 +26721,12 @@
       </c>
       <c r="D134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Permission Set</t>
+          <t xml:space="preserve">Lightning Page</t>
         </is>
       </c>
       <c r="E134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Full_Access</t>
+          <t xml:space="preserve">Sales_Lead_Record_Page</t>
         </is>
       </c>
       <c r="F134" t="inlineStr" s="2">
@@ -26374,7 +26736,7 @@
       </c>
       <c r="G134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H134" t="inlineStr" s="2">
@@ -26399,7 +26761,7 @@
       </c>
       <c r="L134" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign to integration users</t>
+          <t xml:space="preserve">Add maskedPhonePanel (click-to-dial on)</t>
         </is>
       </c>
     </row>
@@ -26419,12 +26781,12 @@
       </c>
       <c r="D135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Profile</t>
+          <t xml:space="preserve">Permission Set</t>
         </is>
       </c>
       <c r="E135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
+          <t xml:space="preserve">Phone_Number_Full_Access</t>
         </is>
       </c>
       <c r="F135" t="inlineStr" s="2">
@@ -26434,12 +26796,12 @@
       </c>
       <c r="G135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual / Change set</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I135" t="inlineStr" s="2">
@@ -26459,7 +26821,7 @@
       </c>
       <c r="L135" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
+          <t xml:space="preserve">Assign to integration users</t>
         </is>
       </c>
     </row>
@@ -26479,12 +26841,12 @@
       </c>
       <c r="D136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App (assignment)</t>
+          <t xml:space="preserve">Profile</t>
         </is>
       </c>
       <c r="E136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
+          <t xml:space="preserve">~40 rep profiles (Presales outbound, Sales, CRM Team, Referral Team, TLs ...)</t>
         </is>
       </c>
       <c r="F136" t="inlineStr" s="2">
@@ -26509,7 +26871,7 @@
       </c>
       <c r="J136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot cleanup</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -26519,7 +26881,7 @@
       </c>
       <c r="L136" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Remove POC assignment row</t>
+          <t xml:space="preserve">Remove phone-field access; Export Reports / API Enabled where safe</t>
         </is>
       </c>
     </row>
@@ -26529,22 +26891,22 @@
       </c>
       <c r="B137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Security fix</t>
+          <t xml:space="preserve">Part 11</t>
         </is>
       </c>
       <c r="C137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">optional</t>
+          <t xml:space="preserve">v2.0.0</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Named Credential</t>
+          <t xml:space="preserve">Lightning App (assignment)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">MCube_API</t>
+          <t xml:space="preserve">Pre_Sales (Gsquare Housing)</t>
         </is>
       </c>
       <c r="F137" t="inlineStr" s="2">
@@ -26554,12 +26916,12 @@
       </c>
       <c r="G137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">New</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Change set</t>
+          <t xml:space="preserve">Manual / Change set</t>
         </is>
       </c>
       <c r="I137" t="inlineStr" s="2">
@@ -26569,7 +26931,7 @@
       </c>
       <c r="J137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes (optional)</t>
+          <t xml:space="preserve">Pilot cleanup</t>
         </is>
       </c>
       <c r="K137" t="inlineStr" s="6">
@@ -26579,7 +26941,7 @@
       </c>
       <c r="L137" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Separate approval</t>
+          <t xml:space="preserve">Remove POC assignment row</t>
         </is>
       </c>
     </row>
@@ -26599,12 +26961,12 @@
       </c>
       <c r="D138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Apex Class</t>
+          <t xml:space="preserve">Named Credential</t>
         </is>
       </c>
       <c r="E138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeAutoDailerApi</t>
+          <t xml:space="preserve">MCube_API</t>
         </is>
       </c>
       <c r="F138" t="inlineStr" s="2">
@@ -26614,7 +26976,7 @@
       </c>
       <c r="G138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Existing (change)</t>
+          <t xml:space="preserve">New</t>
         </is>
       </c>
       <c r="H138" t="inlineStr" s="2">
@@ -26639,7 +27001,7 @@
       </c>
       <c r="L138" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
+          <t xml:space="preserve">Separate approval</t>
         </is>
       </c>
     </row>
@@ -26664,7 +27026,7 @@
       </c>
       <c r="E139" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">mCubeController</t>
+          <t xml:space="preserve">McubeAutoDailerApi</t>
         </is>
       </c>
       <c r="F139" t="inlineStr" s="2">
@@ -26724,7 +27086,7 @@
       </c>
       <c r="E140" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
+          <t xml:space="preserve">mCubeController</t>
         </is>
       </c>
       <c r="F140" t="inlineStr" s="2">
@@ -26769,22 +27131,22 @@
       </c>
       <c r="B141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 1</t>
+          <t xml:space="preserve">Security fix</t>
         </is>
       </c>
       <c r="C141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">optional</t>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual step</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="E141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M1</t>
+          <t xml:space="preserve">McubeSoftphoneAddOnController</t>
         </is>
       </c>
       <c r="F141" t="inlineStr" s="2">
@@ -26794,12 +27156,12 @@
       </c>
       <c r="G141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Existing (change)</t>
         </is>
       </c>
       <c r="H141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manual</t>
+          <t xml:space="preserve">Change set</t>
         </is>
       </c>
       <c r="I141" t="inlineStr" s="2">
@@ -26809,7 +27171,7 @@
       </c>
       <c r="J141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Yes (optional)</t>
         </is>
       </c>
       <c r="K141" t="inlineStr" s="6">
@@ -26819,7 +27181,7 @@
       </c>
       <c r="L141" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
+          <t xml:space="preserve">Use Named Credential MCube_API instead of hard-coded token / http URL</t>
         </is>
       </c>
     </row>
@@ -26829,7 +27191,7 @@
       </c>
       <c r="B142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 1</t>
         </is>
       </c>
       <c r="C142" t="inlineStr" s="2">
@@ -26844,7 +27206,7 @@
       </c>
       <c r="E142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M2</t>
+          <t xml:space="preserve">M1</t>
         </is>
       </c>
       <c r="F142" t="inlineStr" s="2">
@@ -26869,7 +27231,7 @@
       </c>
       <c r="J142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only (decide)</t>
+          <t xml:space="preserve">Yes</t>
         </is>
       </c>
       <c r="K142" t="inlineStr" s="6">
@@ -26879,7 +27241,7 @@
       </c>
       <c r="L142" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
+          <t xml:space="preserve">Assign permission set Phone Access Audit Viewer to admins who review audits</t>
         </is>
       </c>
     </row>
@@ -26904,7 +27266,7 @@
       </c>
       <c r="E143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M3</t>
+          <t xml:space="preserve">M2</t>
         </is>
       </c>
       <c r="F143" t="inlineStr" s="2">
@@ -26929,7 +27291,7 @@
       </c>
       <c r="J143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Pilot only</t>
+          <t xml:space="preserve">Pilot only (decide)</t>
         </is>
       </c>
       <c r="K143" t="inlineStr" s="6">
@@ -26939,7 +27301,7 @@
       </c>
       <c r="L143" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Clone profile Presales outbound -&gt; POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -26949,7 +27311,7 @@
       </c>
       <c r="B144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 6</t>
+          <t xml:space="preserve">Part 2</t>
         </is>
       </c>
       <c r="C144" t="inlineStr" s="2">
@@ -26964,7 +27326,7 @@
       </c>
       <c r="E144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M9</t>
+          <t xml:space="preserve">M3</t>
         </is>
       </c>
       <c r="F144" t="inlineStr" s="2">
@@ -26989,7 +27351,7 @@
       </c>
       <c r="J144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Yes</t>
+          <t xml:space="preserve">Pilot only</t>
         </is>
       </c>
       <c r="K144" t="inlineStr" s="6">
@@ -26999,7 +27361,7 @@
       </c>
       <c r="L144" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
+          <t xml:space="preserve">Activate Sales_Lead_Record_Page_Masked_POC for Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
         </is>
       </c>
     </row>
@@ -27024,7 +27386,7 @@
       </c>
       <c r="E145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M10</t>
+          <t xml:space="preserve">M9</t>
         </is>
       </c>
       <c r="F145" t="inlineStr" s="2">
@@ -27059,7 +27421,7 @@
       </c>
       <c r="L145" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
+          <t xml:space="preserve">Schedule PhoneAuditPurgeBatch nightly</t>
         </is>
       </c>
     </row>
@@ -27069,7 +27431,7 @@
       </c>
       <c r="B146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 11</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="C146" t="inlineStr" s="2">
@@ -27084,7 +27446,7 @@
       </c>
       <c r="E146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M11</t>
+          <t xml:space="preserve">M10</t>
         </is>
       </c>
       <c r="F146" t="inlineStr" s="2">
@@ -27119,7 +27481,7 @@
       </c>
       <c r="L146" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
+          <t xml:space="preserve">Assign Phone_Number_Reveal to TLs, Heads, Admins</t>
         </is>
       </c>
     </row>
@@ -27144,7 +27506,7 @@
       </c>
       <c r="E147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">M12</t>
+          <t xml:space="preserve">M11</t>
         </is>
       </c>
       <c r="F147" t="inlineStr" s="2">
@@ -27179,7 +27541,7 @@
       </c>
       <c r="L147" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+          <t xml:space="preserve">Assign Phone_Number_Full_Access to integration users (MCube, Yotel, Zetta, website/portal, SlashRTC log user)</t>
         </is>
       </c>
     </row>
@@ -27189,62 +27551,122 @@
       </c>
       <c r="B148" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">Part 11</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual step</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">M12</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manual</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Yes</t>
+        </is>
+      </c>
+      <c r="K148" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate pages / assignments that cannot be deployed (Pre_Sales app)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2">
+        <v>145</v>
+      </c>
+      <c r="B149" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">Part 13</t>
         </is>
       </c>
-      <c r="C148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr" s="2">
+      <c r="C149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual step</t>
         </is>
       </c>
-      <c r="E148" t="inlineStr" s="2">
+      <c r="E149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">M13</t>
         </is>
       </c>
-      <c r="F148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="G148" t="inlineStr" s="2">
+      <c r="F149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="H148" t="inlineStr" s="2">
+      <c r="H149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Manual</t>
         </is>
       </c>
-      <c r="I148" t="inlineStr" s="2">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="J148" t="inlineStr" s="2">
+      <c r="I149" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Yes</t>
         </is>
       </c>
-      <c r="K148" t="inlineStr" s="6">
+      <c r="K149" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
-      <c r="L148" t="inlineStr" s="2">
+      <c r="L149" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production: Validate change set with Run specified tests, then Quick Deploy</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L148"/>
+  <autoFilter ref="A4:L149"/>
   <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>

</xml_diff>

<commit_message>
plan: Part 6 (Reveal and audit cleanup) in the register
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -19,6 +19,7 @@
     <sheet name="Part 5c Plan" sheetId="15" r:id="rId15"/>
     <sheet name="Part 5d Plan" sheetId="16" r:id="rId16"/>
     <sheet name="Part 5e Plan" sheetId="17" r:id="rId17"/>
+    <sheet name="Part 6 Plan" sheetId="18" r:id="rId18"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Read Me'!$A$4:$B$11</definedName>
@@ -38,6 +39,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'Part 5c Plan'!$A$4:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Part 5d Plan'!$A$4:$F$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Part 5e Plan'!$A$4:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Part 6 Plan'!$A$4:$F$13</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -9078,6 +9080,363 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="90" customWidth="1"/>
+    <col min="5" max="5" width="44" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr" s="3">
+        <is>
+          <t>Part 6 (v1.6.0) - Reveal and audit cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr" s="10">
+        <is>
+          <t>Explained before implementation; checkpoint tag checkpoint-before-part6</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" t="inlineStr" s="1">
+        <is>
+          <t>New / Existing</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr" s="1">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr" s="1">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr" s="1">
+        <is>
+          <t>Change</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr" s="1">
+        <is>
+          <t>Effect for users</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr" s="1">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Permission</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reveal_Phone_Number</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Who may reveal (design G5)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Only users with it see the Reveal button</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Reveal</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Grants Reveal_Phone_Number + Apex access to PhoneRevealService. Assigned to Team Leads, Heads, Admins (go-live); a POC TL test user in the sandbox</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneRevealService (+ test)</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">revealNumber(recordId, fieldKey, reason, comment): checks the custom permission, the reason (7 approved values) and the comment (required for Other), then MaskedDialService (approved field, record access, Reveal audit row with reason + comment) and returns the number + seconds to show</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Real number only for permitted users, always audited</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Field</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit__c.Comment__c</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Long text - comment of a reveal (required for Other)</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Audit shows why</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">None</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">New</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatch (+ test)</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Batch + Schedulable: deletes Phone_Access_Audit__c rows older than Audit_Retention_Days__c (365); scheduled nightly (manual step)</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Audit kept 1 year</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Updated (ours)</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reveal requests carry a comment -&gt; Comment__c on the audit row</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Updated (ours)</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">LWC</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Reveal button per number (only with Reveal_Phone_Number); dialog with the 7 reasons + comment; number shown for Reveal_Seconds__c (30) then cleared from the screen</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">TL / Head / Admin can reveal; reps see no button</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Low</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Kept (decision)</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Field</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit__c.Reason__c</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Stays Text (already deployed). The 7 reasons are enforced by Apex and offered as a dropdown in the dialog. Design said picklist - changing a deployed field type is avoided</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">No change</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Existing org components</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6 changes only components built in this project</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">-</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:F13"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheetFormatPr defaultRowHeight="15"/>

</xml_diff>

<commit_message>
feat: v1.6.0 Reveal for TL/Head/Admin + nightly audit purge (built locally, not deployed)
New: Reveal_Phone_Number custom permission, Phone_Reveal permission set,
PhoneRevealService (+test), PhoneAuditPurgeBatch (+test), Comment__c.
Ours updated: MaskedDialService (comment), maskedPhonePanel (reveal dialog,
30 s display, Jest), Phone_Access_Audit_Viewer, audit list view.
No existing org component changed. TEST_GUIDE Part 6, manifests, release
bundle part6-reveal, changelog, roadmap, register.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -31,8 +31,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Test Classes'!$A$4:$F$19</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Backups'!$A$4:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Part 3 Plan'!$A$4:$F$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$120</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Release Bundle'!$A$4:$K$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Release Steps'!$A$4:$E$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Part 4 Plan'!$A$4:$F$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Part 5a Plan'!$A$4:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'Part 5b Plan'!$A$4:$F$11</definedName>
@@ -333,7 +333,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Release Bundle - built components (Parts 1-5e)</t>
+          <t>Production Release Bundle - built components (Parts 1-6)</t>
         </is>
       </c>
     </row>
@@ -437,7 +437,7 @@
       </c>
       <c r="H5" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">a8c2c5dc228b</t>
+          <t xml:space="preserve">17d562f3f69e</t>
         </is>
       </c>
       <c r="I5" t="inlineStr" s="2">
@@ -1647,7 +1647,7 @@
       </c>
       <c r="H27" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">1098c11ee9d4</t>
+          <t xml:space="preserve">b7c497e3b53c</t>
         </is>
       </c>
       <c r="I27" t="inlineStr" s="2">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="H30" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9514afa794c8</t>
+          <t xml:space="preserve">9423eb14b896</t>
         </is>
       </c>
       <c r="I30" t="inlineStr" s="2">
@@ -1867,7 +1867,7 @@
       </c>
       <c r="H31" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">dea06e92ea46</t>
+          <t xml:space="preserve">f91f322f9b23</t>
         </is>
       </c>
       <c r="I31" t="inlineStr" s="2">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="H37" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">2cc369f04123</t>
+          <t xml:space="preserve">f50e079e970f</t>
         </is>
       </c>
       <c r="I37" t="inlineStr" s="2">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="H38" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">d44addcdfaf9</t>
+          <t xml:space="preserve">b3206bb2003d</t>
         </is>
       </c>
       <c r="I38" t="inlineStr" s="2">
@@ -4287,7 +4287,7 @@
       </c>
       <c r="H75" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">a8c2c5dc228b</t>
+          <t xml:space="preserve">17d562f3f69e</t>
         </is>
       </c>
       <c r="I75" t="inlineStr" s="2">
@@ -6622,47 +6622,47 @@
       </c>
       <c r="B118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part6-reveal</t>
         </is>
       </c>
       <c r="C118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="E118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning Page</t>
+          <t xml:space="preserve"/>
         </is>
       </c>
       <c r="F118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+          <t xml:space="preserve">Reveal_Phone_Number.customPermission</t>
         </is>
       </c>
       <c r="G118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+          <t xml:space="preserve">release/prod/part6-reveal/customPermissions/Reveal_Phone_Number.customPermission</t>
         </is>
       </c>
       <c r="H118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">9354cdba5c3c</t>
+          <t xml:space="preserve">433c5c6e5918</t>
         </is>
       </c>
       <c r="I118" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J118" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K118" t="inlineStr" s="6">
@@ -6677,47 +6677,47 @@
       </c>
       <c r="B119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">part2-pilot</t>
+          <t xml:space="preserve">part6-reveal</t>
         </is>
       </c>
       <c r="C119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Part 2</t>
+          <t xml:space="preserve">Part 6</t>
         </is>
       </c>
       <c r="D119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">v1.2.0</t>
+          <t xml:space="preserve">v1.6.0</t>
         </is>
       </c>
       <c r="E119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Manifest (package.xml)</t>
+          <t xml:space="preserve">Apex Class</t>
         </is>
       </c>
       <c r="F119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">package.xml</t>
+          <t xml:space="preserve">MaskedDialService</t>
         </is>
       </c>
       <c r="G119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/MaskedDialService.cls</t>
         </is>
       </c>
       <c r="H119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">b158c134f515</t>
+          <t xml:space="preserve">17d562f3f69e</t>
         </is>
       </c>
       <c r="I119" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
-        </is>
-      </c>
-      <c r="J119" t="inlineStr" s="4">
-        <is>
-          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
         </is>
       </c>
       <c r="K119" t="inlineStr" s="6">
@@ -6732,57 +6732,1102 @@
       </c>
       <c r="B120" t="inlineStr" s="2">
         <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">MaskedDialService</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/MaskedDialService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I120" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K120" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2">
+        <v>10</v>
+      </c>
+      <c r="B121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneAuditPurgeBatch.cls</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">36ed27884084</t>
+        </is>
+      </c>
+      <c r="I121" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K121" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2">
+        <v>10</v>
+      </c>
+      <c r="B122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatch</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneAuditPurgeBatch.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I122" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K122" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2">
+        <v>10</v>
+      </c>
+      <c r="B123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneRevealService</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneRevealService.cls</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f8c9b16452fa</t>
+        </is>
+      </c>
+      <c r="I123" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K123" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2">
+        <v>10</v>
+      </c>
+      <c r="B124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class</t>
+        </is>
+      </c>
+      <c r="F124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneRevealService</t>
+        </is>
+      </c>
+      <c r="G124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneRevealService.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I124" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K124" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2">
+        <v>10</v>
+      </c>
+      <c r="B125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneAuditPurgeBatchTest.cls</t>
+        </is>
+      </c>
+      <c r="H125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">cb7ff5561eaf</t>
+        </is>
+      </c>
+      <c r="I125" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K125" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2">
+        <v>10</v>
+      </c>
+      <c r="B126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneAuditPurgeBatchTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K126" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2">
+        <v>10</v>
+      </c>
+      <c r="B127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneRevealServiceTest.cls</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9e565917d18f</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K127" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2">
+        <v>10</v>
+      </c>
+      <c r="B128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Apex Class (test)</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">PhoneRevealServiceTest</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/classes/PhoneRevealServiceTest.cls-meta.xml</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">87b91a7450c6</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K128" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2">
+        <v>10</v>
+      </c>
+      <c r="B129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Custom Object / Custom Metadata Type (with fields)</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit__c</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/objects/Phone_Access_Audit__c.object</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bd22c8871577</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K129" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2">
+        <v>10</v>
+      </c>
+      <c r="B130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/lwc/maskedPhonePanel/maskedPhonePanel.css</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f1df701a3a2c</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2">
+        <v>10</v>
+      </c>
+      <c r="B131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/lwc/maskedPhonePanel/maskedPhonePanel.html</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f50e079e970f</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2">
+        <v>10</v>
+      </c>
+      <c r="B132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/lwc/maskedPhonePanel/maskedPhonePanel.js</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b3206bb2003d</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2">
+        <v>10</v>
+      </c>
+      <c r="B133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Web Component</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">maskedPhonePanel</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/lwc/maskedPhonePanel/maskedPhonePanel.js-meta.xml</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">0d33c6f7d7e6</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2">
+        <v>10</v>
+      </c>
+      <c r="B134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/package.xml</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">84e472da365b</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2">
+        <v>10</v>
+      </c>
+      <c r="B135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Access_Audit_Viewer</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/permissionsets/Phone_Access_Audit_Viewer.permissionset</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">f91f322f9b23</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K135" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2">
+        <v>10</v>
+      </c>
+      <c r="B136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part6-reveal</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 6</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.6.0</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Permission Set</t>
+        </is>
+      </c>
+      <c r="F136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Phone_Reveal</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part6-reveal/permissionsets/Phone_Reveal.permissionset</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">bc690fd14a68</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local) - not deployed</t>
+        </is>
+      </c>
+      <c r="K136" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2">
+        <v>11</v>
+      </c>
+      <c r="B137" t="inlineStr" s="2">
+        <is>
           <t xml:space="preserve">part2-pilot</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr" s="2">
+      <c r="C137" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Part 2</t>
         </is>
       </c>
-      <c r="D120" t="inlineStr" s="2">
+      <c r="D137" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">v1.2.0</t>
         </is>
       </c>
-      <c r="E120" t="inlineStr" s="2">
+      <c r="E137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning Page</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Sales_Lead_Record_Page_Masked_POC</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/flexipages/Sales_Lead_Record_Page_Masked_POC.flexipage</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">9354cdba5c3c</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K137" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2">
+        <v>11</v>
+      </c>
+      <c r="B138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Manifest (package.xml)</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">package.xml</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">release/prod/part2-pilot/package.xml</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">b158c134f515</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
+        </is>
+      </c>
+      <c r="K138" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2">
+        <v>11</v>
+      </c>
+      <c r="B139" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">part2-pilot</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Part 2</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">v1.2.0</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Profile</t>
         </is>
       </c>
-      <c r="F120" t="inlineStr" s="2">
+      <c r="F139" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">POC Masked Rep</t>
         </is>
       </c>
-      <c r="G120" t="inlineStr" s="2">
+      <c r="G139" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">release/prod/part2-pilot/profiles/POC Masked Rep.profile</t>
         </is>
       </c>
-      <c r="H120" t="inlineStr" s="2">
+      <c r="H139" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">df1ecd8c7bec</t>
         </is>
       </c>
-      <c r="I120" t="inlineStr" s="2">
+      <c r="I139" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Production pilot only (clone POC profile first)</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr" s="4">
+      <c r="J139" t="inlineStr" s="4">
         <is>
           <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LRq1CAG / 0Afft000000LRzhCAG</t>
         </is>
       </c>
-      <c r="K120" t="inlineStr" s="6">
+      <c r="K139" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:K120"/>
+  <autoFilter ref="A4:K139"/>
   <mergeCells count="2">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="A2:K2"/>
@@ -6806,7 +7851,7 @@
     <row r="1">
       <c r="A1" t="inlineStr" s="3">
         <is>
-          <t>Production Deploy Steps (Parts 1-5e)</t>
+          <t>Production Deploy Steps (Parts 1-6)</t>
         </is>
       </c>
     </row>
@@ -7109,47 +8154,49 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2">
-        <v>4</v>
+      <c r="A15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">3i</t>
+        </is>
       </c>
       <c r="B15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual)</t>
+          <t xml:space="preserve">part6-reveal</t>
         </is>
       </c>
       <c r="C15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
+          <t xml:space="preserve">Validate in production, then quick deploy; then schedule PhoneAuditPurgeBatch.scheduleNightly() and assign Phone_Reveal to TL / Head / Admin</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Setup &gt; Permission Sets</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Not deployed</t>
+          <t xml:space="preserve">sf project deploy validate --metadata-dir release/prod/part6-reveal --test-level RunSpecifiedTests --tests PhoneRevealServiceTest --tests PhoneAuditPurgeBatchTest --tests MaskedDialServiceTest --tests MaskedPhonePanelControllerTest</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve"> --target-org &lt;prod&gt;   then   sf project deploy quick --job-id &lt;id&gt; --target-org &lt;prod&gt;</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">(manual, pilot)</t>
+          <t xml:space="preserve">(manual)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+          <t xml:space="preserve">Assign Phone Access Audit Viewer to admins</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+          <t xml:space="preserve">Setup &gt; Permission Sets</t>
         </is>
       </c>
       <c r="E16" t="inlineStr" s="6">
@@ -7160,31 +8207,56 @@
     </row>
     <row r="17">
       <c r="A17" s="2">
+        <v>5</v>
+      </c>
+      <c r="B17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">(manual, pilot)</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Activate masked POC page: Gsquare Housing / Desktop / Pre Sales / POC Masked Rep</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr" s="2">
+        <is>
+          <t xml:space="preserve">Lightning App Builder &gt; Activation</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr" s="6">
+        <is>
+          <t xml:space="preserve">Not deployed</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
         <v>6</v>
       </c>
-      <c r="B17" t="inlineStr" s="2">
+      <c r="B18" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">(check)</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr" s="2">
+      <c r="C18" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Run scripts/apex/v1.1.0-1 and -2 (read-only)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr" s="2">
+      <c r="D18" t="inlineStr" s="2">
         <is>
           <t xml:space="preserve">Developer Console &gt; Execute Anonymous</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr" s="6">
+      <c r="E18" t="inlineStr" s="6">
         <is>
           <t xml:space="preserve">Not deployed</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E17"/>
+  <autoFilter ref="A4:E18"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>
@@ -9693,9 +10765,9 @@
           <t xml:space="preserve">Reveal + audit cleanup</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="D10" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="E10" s="2">
@@ -14353,9 +15425,9 @@
           <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I76" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J76" t="inlineStr" s="2">
@@ -14413,9 +15485,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I77" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I77" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J77" t="inlineStr" s="2">
@@ -14455,7 +15527,7 @@
       </c>
       <c r="E78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Comment__c</t>
         </is>
       </c>
       <c r="F78" t="inlineStr" s="2">
@@ -14465,7 +15537,7 @@
       </c>
       <c r="G78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Picklist, 7 agreed reasons</t>
+          <t xml:space="preserve">Reveal comment (Reason__c kept as Text; 7 reasons enforced in Apex)</t>
         </is>
       </c>
       <c r="H78" t="inlineStr" s="2">
@@ -14473,9 +15545,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I78" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I78" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J78" t="inlineStr" s="2">
@@ -14533,9 +15605,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I79" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I79" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J79" t="inlineStr" s="2">
@@ -14593,9 +15665,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I80" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I80" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J80" t="inlineStr" s="2">
@@ -14653,9 +15725,9 @@
           <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I81" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J81" t="inlineStr" s="2">
@@ -14713,9 +15785,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I82" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I82" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J82" t="inlineStr" s="2">
@@ -14773,9 +15845,9 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I83" t="inlineStr" s="6">
-        <is>
-          <t xml:space="preserve">Planned</t>
+      <c r="I83" t="inlineStr" s="5">
+        <is>
+          <t xml:space="preserve">Built (Local)</t>
         </is>
       </c>
       <c r="J83" t="inlineStr" s="2">
@@ -25105,7 +26177,7 @@
       </c>
       <c r="E101" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Reveal_Reason__c</t>
+          <t xml:space="preserve">Comment__c</t>
         </is>
       </c>
       <c r="F101" t="inlineStr" s="2">

</xml_diff>

<commit_message>
docs: register uses the actual permission set name Phone_Reveal
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -15647,7 +15647,7 @@
       </c>
       <c r="E80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">Phone_Reveal</t>
         </is>
       </c>
       <c r="F80" t="inlineStr" s="2">
@@ -26597,7 +26597,7 @@
       </c>
       <c r="E108" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve">Phone_Number_Reveal</t>
+          <t xml:space="preserve">Phone_Reveal</t>
         </is>
       </c>
       <c r="F108" t="inlineStr" s="2">

</xml_diff>

<commit_message>
deploy: Part 6 (Reveal + purge) to sandbox; POC TL created
0Afft000000LmMcCAK: 11/11, 45 tests passed. Coverage: PhoneRevealService 100%,
PhoneAuditPurgeBatch 100%, MaskedDialService 90.6%. POC TL (005ft000000YupRAAS)
created with Phone Reveal. Nightly purge not scheduled yet (owner OK pending).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Mobile_Masking_Component_Register.xlsx
+++ b/docs/Mobile_Masking_Component_Register.xlsx
@@ -6660,9 +6660,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J118" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J118" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K118" t="inlineStr" s="6">
@@ -6715,9 +6715,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J119" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J119" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K119" t="inlineStr" s="6">
@@ -6770,9 +6770,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J120" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J120" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K120" t="inlineStr" s="6">
@@ -6825,9 +6825,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J121" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J121" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K121" t="inlineStr" s="6">
@@ -6880,9 +6880,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J122" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J122" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K122" t="inlineStr" s="6">
@@ -6935,9 +6935,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J123" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J123" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K123" t="inlineStr" s="6">
@@ -6990,9 +6990,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J124" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J124" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K124" t="inlineStr" s="6">
@@ -7045,9 +7045,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J125" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J125" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K125" t="inlineStr" s="6">
@@ -7100,9 +7100,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J126" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J126" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K126" t="inlineStr" s="6">
@@ -7155,9 +7155,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J127" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J127" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K127" t="inlineStr" s="6">
@@ -7210,9 +7210,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J128" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J128" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K128" t="inlineStr" s="6">
@@ -7265,9 +7265,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J129" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J129" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K129" t="inlineStr" s="6">
@@ -7320,9 +7320,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J130" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J130" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K130" t="inlineStr" s="6">
@@ -7375,9 +7375,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J131" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J131" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K131" t="inlineStr" s="6">
@@ -7430,9 +7430,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J132" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J132" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K132" t="inlineStr" s="6">
@@ -7485,9 +7485,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J133" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J133" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K133" t="inlineStr" s="6">
@@ -7540,9 +7540,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J134" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J134" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K134" t="inlineStr" s="6">
@@ -7595,9 +7595,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J135" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J135" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K135" t="inlineStr" s="6">
@@ -7650,9 +7650,9 @@
           <t xml:space="preserve">Production - everyone (assign Phone_Reveal to TL / Head / Admin)</t>
         </is>
       </c>
-      <c r="J136" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local) - not deployed</t>
+      <c r="J136" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox) 0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K136" t="inlineStr" s="6">
@@ -10765,9 +10765,9 @@
           <t xml:space="preserve">Reveal + audit cleanup</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="D10" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="E10" s="2">
@@ -15425,14 +15425,14 @@
           <t xml:space="preserve">PhoneRevealServiceTest</t>
         </is>
       </c>
-      <c r="I76" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I76" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J76" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K76" t="inlineStr" s="2">
@@ -15485,14 +15485,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I77" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I77" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J77" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K77" t="inlineStr" s="2">
@@ -15545,14 +15545,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I78" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I78" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J78" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K78" t="inlineStr" s="2">
@@ -15605,14 +15605,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I79" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I79" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J79" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K79" t="inlineStr" s="2">
@@ -15665,14 +15665,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I80" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I80" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J80" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K80" t="inlineStr" s="2">
@@ -15725,14 +15725,14 @@
           <t xml:space="preserve">PhoneAuditPurgeBatchTest</t>
         </is>
       </c>
-      <c r="I81" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I81" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J81" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K81" t="inlineStr" s="2">
@@ -15785,14 +15785,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I82" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I82" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J82" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K82" t="inlineStr" s="2">
@@ -15845,14 +15845,14 @@
           <t xml:space="preserve"/>
         </is>
       </c>
-      <c r="I83" t="inlineStr" s="5">
-        <is>
-          <t xml:space="preserve">Built (Local)</t>
+      <c r="I83" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">Deployed (Sandbox)</t>
         </is>
       </c>
       <c r="J83" t="inlineStr" s="2">
         <is>
-          <t xml:space="preserve"/>
+          <t xml:space="preserve">0Afft000000LmMcCAK</t>
         </is>
       </c>
       <c r="K83" t="inlineStr" s="2">

</xml_diff>